<commit_message>
fix(query): remove hard-coded benchmark answers; report measured results
- delete try_plan_branching / try_cross_version_overview / try_elective_credits
  (canned text with fixed numbers and page refs, not read from the database)
- graduation audit: keep only DSBA 2565 thresholds verified against the book (p.15),
  require the student's own numbers, drop the unverified GPAX 2.00 line
- document relation: label files by detected degree_level instead of from/to order,
  drop the static readme.txt sentence
- re-run the 28-question benchmark and re-review: 25 correct / 1 partial / 2 wrong
  (C1 wrong, C3 mismatch); update manual_review.json, reviewed_run.json, tester.xlsx, README
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +76,14 @@
       <color rgb="00B45309"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -122,20 +128,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF7ED"/>
+        <bgColor rgb="00FFF7ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
         <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7ED"/>
-        <bgColor rgb="00FFF7ED"/>
+        <fgColor rgb="00FAF5FF"/>
+        <bgColor rgb="00FAF5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAF5FF"/>
-        <bgColor rgb="00FAF5FF"/>
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -220,16 +232,16 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -600,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -695,7 +707,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>28/28 ข้อ — เกณฑ์หลวม (บางข้อตรวจแค่มีตัวเลข) ไม่ใช่การยืนยันว่าถูก</t>
+          <t>27/28 ข้อ — เกณฑ์หลวม (บางข้อตรวจแค่มีตัวเลข) ไม่ใช่การยืนยันว่าถูก</t>
         </is>
       </c>
     </row>
@@ -707,7 +719,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ถูกครบ 23 · ถูกบางส่วน 5 · ผิด 0 · ยังไม่ได้ตรวจ 0</t>
+          <t>ถูกครบ 25 · ถูกบางส่วน 1 · ผิด/ไม่ตรงเฉลย 2 · ยังไม่ได้ตรวจ 0</t>
         </is>
       </c>
     </row>
@@ -719,7 +731,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>เฉลี่ย 0.47s · เร็วสุด 0.05s · ช้าสุด 3.98s · ต่ำกว่า 5s 28/28 ข้อ</t>
+          <t>เฉลี่ย 0.65s · เร็วสุด 0.05s · ช้าสุด 4.86s · ต่ำกว่า 5s 28/28 ข้อ</t>
         </is>
       </c>
     </row>
@@ -770,7 +782,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>ผิด</t>
+          <t>ผิด / ไม่ตรงเฉลย</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -807,12 +819,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>0.27</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>0.89</t>
         </is>
       </c>
     </row>
@@ -839,12 +851,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.70</t>
         </is>
       </c>
     </row>
@@ -861,22 +873,22 @@
         <v>7</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>0.86</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>3.98</t>
+          <t>1.58</t>
         </is>
       </c>
     </row>
@@ -890,25 +902,25 @@
         <v>3</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="8" t="n">
-        <v>0</v>
-      </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>2.61</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>0.27</t>
+          <t>4.86</t>
         </is>
       </c>
     </row>
@@ -922,25 +934,25 @@
         <v>28</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.65</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>3.98</t>
+          <t>4.86</t>
         </is>
       </c>
     </row>
@@ -975,30 +987,38 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>4) ข้อ M8, H5, C1, C3 ตอบด้วยข้อความสำเร็จรูปที่เขียนไว้ในโค้ด (structured_query.py) ไม่ได้ดึงจากฐานข้อมูลตอนถาม จึงไม่ควรใช้เป็นหลักฐานว่าระบบสกัดข้อมูลเหล่านั้นได้เอง</t>
+          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้จึงมาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM) ผลของ C1 และ C3 จึงไม่ดี ซึ่งตรงกับที่ระบบทำได้จริง</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ เช่น M8 รันซ้ำ 8 ครั้งพบเลข 12 ในคำตอบ 5 ครั้ง; H5 พบ 8 ครั้งจาก 8</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
+          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
           <t>6) เฉลยข้อ H4 เดิมเขียน 48 วิชา แต่ฐานข้อมูลปัจจุบันให้ 52 (DSBA 2560 71 ชื่อ / 2565 75 ชื่อ) ผลของระบบตรงกับฐานข้อมูล</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="B9:H9"/>
+    <mergeCell ref="A29:H29"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B4:H4"/>
@@ -1202,7 +1222,7 @@
       </c>
       <c r="N2" s="15" t="inlineStr">
         <is>
-          <t>0.07s</t>
+          <t>0.08s</t>
         </is>
       </c>
       <c r="O2" s="18" t="inlineStr">
@@ -1362,7 +1382,7 @@
       </c>
       <c r="N4" s="15" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="O4" s="18" t="inlineStr">
@@ -1457,7 +1477,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="O5" s="18" t="inlineStr">
@@ -1499,7 +1519,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>ชื่อวิชาภาษาอังกฤษของ "ระบบข้อมูลมหัต" คือ **Big Data Systems** [4]</t>
+          <t>ระบบข้อมูลมหัต (Big Data Systems) [4]</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -1533,7 +1553,7 @@
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>1.29s</t>
+          <t>0.89s</t>
         </is>
       </c>
       <c r="O6" s="18" t="inlineStr">
@@ -1625,7 +1645,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="O7" s="18" t="inlineStr">
@@ -1788,7 +1808,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.30s</t>
         </is>
       </c>
       <c r="O9" s="18" t="inlineStr">
@@ -1866,7 +1886,7 @@
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="O10" s="18" t="inlineStr">
@@ -1944,7 +1964,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.08s</t>
         </is>
       </c>
       <c r="O11" s="18" t="inlineStr">
@@ -2029,7 +2049,7 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O12" s="18" t="inlineStr">
@@ -2118,7 +2138,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.41s</t>
         </is>
       </c>
       <c r="O13" s="18" t="inlineStr">
@@ -2209,7 +2229,7 @@
       </c>
       <c r="N14" s="15" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.40s</t>
         </is>
       </c>
       <c r="O14" s="18" t="inlineStr">
@@ -2314,7 +2334,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.27s</t>
         </is>
       </c>
       <c r="O15" s="18" t="inlineStr">
@@ -2409,7 +2429,7 @@
       </c>
       <c r="N16" s="15" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.05s</t>
         </is>
       </c>
       <c r="O16" s="18" t="inlineStr">
@@ -2494,7 +2514,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O17" s="18" t="inlineStr">
@@ -2536,13 +2556,7 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>ตามโครงสร้างหลักสูตร DSBA 2565 (หน้า 15, 19) หมวดวิชาเฉพาะ (รวม 96 หน่วยกิต) มีข้อกำหนดดังนี้:
-1. กลุ่มวิชาชีพเฉพาะด้าน (หรือวิชาเฉพาะเลือก): กำหนดให้เก็บ **ไม่น้อยกว่า 12 หน่วยกิต** โดยนักศึกษาต้องเลือกลงทะเบียนเรียนในกลุ่มวิชาชีพเฉพาะด้านกลุ่มใดกลุ่มหนึ่งจาก 3 แขนง ได้แก่:
-   - แขนงวิทยาการข้อมูล (Data Science)
-   - แขนงการวิเคราะห์เชิงสถิติ (Statistical Analysis)
-   - แขนงวิศวกรรมข้อมูล (Data Engineering)
-2. กลุ่มวิชาการศึกษาทางเลือก: อีก **6 หน่วยกิต** (เช่น โครงการสหกิจศึกษา หรือวิชาเลือกทางเลือก)
-สรุป: หมวดวิชาเฉพาะเลือก (กลุ่มวิชาชีพเฉพาะด้าน) ต้องเก็บไม่น้อยกว่า **12 หน่วยกิต**</t>
+          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) หมวดวิชาเฉพาะ กลุ่มวิชาชีพเฉพาะด้าน มีจำนวน 12 หน่วยกิต [6]</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
@@ -2551,9 +2565,9 @@
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 349, 352, 7, 351)</t>
         </is>
       </c>
-      <c r="I18" s="22" t="inlineStr">
-        <is>
-          <t>คำตอบสำเร็จรูปที่เขียนไว้ในโค้ด (hard-coded) — ไม่ได้ดึงจากฐานข้อมูลตอนถาม</t>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
       <c r="J18" s="15" t="n">
@@ -2571,12 +2585,12 @@
       </c>
       <c r="M18" s="16" t="inlineStr">
         <is>
-          <t>แยก 12 หน่วยกิต (วิชาชีพเฉพาะด้าน) กับ 6 หน่วยกิต (การศึกษาทางเลือก) ถูกต้อง</t>
+          <t>ตอบ 12 หน่วยกิตถูกในรอบนี้ แต่ไม่คงที่: รันซ้ำ 8 ครั้ง พบเลข 12 ในคำตอบ 5 ครั้ง (ที่เหลือตอบ 6 หน่วยกิตของอีกกลุ่ม) ผ่าน retrieval + LLM</t>
         </is>
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.70s</t>
         </is>
       </c>
       <c r="O18" s="18" t="inlineStr">
@@ -2656,7 +2670,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O19" s="18" t="inlineStr">
@@ -2671,7 +2685,7 @@
           <t>H1</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -2785,7 +2799,7 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
@@ -2797,7 +2811,7 @@
       </c>
       <c r="N20" s="15" t="inlineStr">
         <is>
-          <t>0.07s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O20" s="18" t="inlineStr">
@@ -2812,7 +2826,7 @@
           <t>H2</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -2840,7 +2854,7 @@
       <c r="G21" s="20" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถเรียนวิชาฐานข้อมูลในปีที่ 4 ได้ เนื่องจากหลักสูตร DSBA 2565 มีวิชาบังคับในปีที่ 4 ภาคเรียนที่ 1 คือ 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 ซึ่งเป็นวิชาที่เกี่ยวข้องกับการประยุกต์ใช้ข้อมูลและระบบฐานข้อมูล โดยไม่มีข้อกำหนดวิชาบังคับก่อนที่ห้ามเรียนในปีที่ 4 และมีวิชาเลือกในกลุ่มวิชาศึกษาทั่วไปหรือวิชาเลือกเสรีที่อาจครอบคลุมเนื้อหาด้านฐานข้อมูลได้ แม้จะไม่มีวิชาฐานข้อมูลโดยตรงในปีที่ 4 แต่ไม่มีข้อห้ามใดระบุไว้ จึงถือว่าเรียนได้ตามหลักสูตร.</t>
+นักศึกษาสามารถเรียนวิชา "ระบบฐานข้อมูลแบบกระจาย" (06026246) ในปีที่ 4 ภาคการศึกษาที่ 1 ได้ เนื่องจากเป็นวิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน ซึ่งไม่มีวิชาบังคับก่อนกำหนดไว้ และอยู่ในหลักสูตร DSBA 2565 ภาคการศึกษาที่ 1 ปีที่ 4 โดยมีหน่วยกิต 3 (3-0-6) ประเภทวิชาเลือก.</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -2862,19 +2876,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L21" s="24" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="L21" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M21" s="20" t="inlineStr">
         <is>
-          <t>ตอบ 'ได้' ถูก แต่เหตุผลไม่ชี้วิชาฐานข้อมูลที่เปิดปี 4 จริง (06026246) และอ้างโครงงานว่าเกี่ยวกับฐานข้อมูลโดยไม่มีหลักฐาน</t>
+          <t>ตอบ 'ได้' และชี้วิชา 06026246 ระบบฐานข้อมูลแบบกระจาย ปี 4 ภาค 1 ไม่มีวิชาบังคับก่อน ตรงเฉลย</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>2.07s</t>
+          <t>1.58s</t>
         </is>
       </c>
       <c r="O21" s="18" t="inlineStr">
@@ -2889,7 +2903,7 @@
           <t>H3</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -2917,7 +2931,7 @@
       <c r="G22" s="16" t="inlineStr">
         <is>
           <t>ไม่ได้  
-วิชา 06026212 การสร้างคลังข้อมูล เป็นวิชาบังคับที่ต้องเรียนในปีที่ 3 ภาคการศึกษาที่ 1 และมีข้อกำหนดให้ต้องผ่านวิชา 06066300 แนวคิดระบบฐานข้อมูล ก่อน ซึ่งเป็นวิชาบังคับในปีที่ 2 ภาคการศึกษาที่ 1 ดังนั้นจึงไม่สามารถลงวิชานี้ได้ในปีที่ 2</t>
+วิชา 06026212 การสร้างคลังข้อมูล (DATA WAREHOUSING) เป็นวิชาบังคับในปีที่ 3 ภาคการศึกษาที่ 1 และมีข้อกำหนดให้ต้องผ่านวิชาบังคับก่อนอย่างน้อย 06066300 แนวคิดระบบฐานข้อมูล ซึ่งจัดสอนในปีที่ 2 ภาคการศึกษาที่ 1 ดังนั้นจึงไม่สามารถลงวิชานี้ได้ในปีที่สอง</t>
         </is>
       </c>
       <c r="H22" s="16" t="inlineStr">
@@ -2951,7 +2965,7 @@
       </c>
       <c r="N22" s="15" t="inlineStr">
         <is>
-          <t>1.36s</t>
+          <t>1.53s</t>
         </is>
       </c>
       <c r="O22" s="18" t="inlineStr">
@@ -2966,7 +2980,7 @@
           <t>H4</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3109,7 +3123,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.19s</t>
         </is>
       </c>
       <c r="O23" s="18" t="inlineStr">
@@ -3124,7 +3138,7 @@
           <t>H5</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3151,13 +3165,7 @@
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>ตามโครงสร้างหลักสูตร DSBA 2565 (หน้า 15, 19) หมวดวิชาเฉพาะ (รวม 96 หน่วยกิต) มีข้อกำหนดดังนี้:
-1. กลุ่มวิชาชีพเฉพาะด้าน (หรือวิชาเฉพาะเลือก): กำหนดให้เก็บ **ไม่น้อยกว่า 12 หน่วยกิต** โดยนักศึกษาต้องเลือกลงทะเบียนเรียนในกลุ่มวิชาชีพเฉพาะด้านกลุ่มใดกลุ่มหนึ่งจาก 3 แขนง ได้แก่:
-   - แขนงวิทยาการข้อมูล (Data Science)
-   - แขนงการวิเคราะห์เชิงสถิติ (Statistical Analysis)
-   - แขนงวิศวกรรมข้อมูล (Data Engineering)
-2. กลุ่มวิชาการศึกษาทางเลือก: อีก **6 หน่วยกิต** (เช่น โครงการสหกิจศึกษา หรือวิชาเลือกทางเลือก)
-สรุป: หมวดวิชาเฉพาะเลือก (กลุ่มวิชาชีพเฉพาะด้าน) ต้องเก็บไม่น้อยกว่า **12 หน่วยกิต**</t>
+          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปรับปรุง พ.ศ. 2565 มีหมวดวิชาเฉพาะ (กลุ่มวิชาชีพเฉพาะด้าน) จำนวน 12 หน่วยกิต [7].</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -3166,9 +3174,9 @@
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 349, 351, 352, 7)</t>
         </is>
       </c>
-      <c r="I24" s="22" t="inlineStr">
-        <is>
-          <t>คำตอบสำเร็จรูปที่เขียนไว้ในโค้ด (hard-coded) — ไม่ได้ดึงจากฐานข้อมูลตอนถาม</t>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
       <c r="J24" s="15" t="n">
@@ -3186,12 +3194,12 @@
       </c>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>12 หน่วยกิต (และแยก 6 หน่วยกิตของอีกกลุ่ม) ตรงเฉลย</t>
+          <t>ตอบ 12 หน่วยกิต (รันซ้ำ 8 ครั้ง พบเลข 12 ทุกครั้ง) ผ่าน retrieval + LLM</t>
         </is>
       </c>
       <c r="N24" s="15" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>1.03s</t>
         </is>
       </c>
       <c r="O24" s="18" t="inlineStr">
@@ -3206,7 +3214,7 @@
           <t>H6</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3233,16 +3241,11 @@
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนงผ่านกลุ่มวิชาเลือก 3 กลุ่ม ได้แก่:
-- วิชาเลือกกลุ่มวิทยาการข้อมูล 1 (ELECTIVE IN DATA SCIENCE 1) – รหัส 06026xxx, 3 หน่วยกิต (3-0-6) หรือ (2-2-5) [3]
-- วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 1 (ELECTIVE IN STATISTICAL ANALYSIS 1) – รหัส 06026xxx, 3 หน่วยกิต (3-0-6) หรือ (2-2-5) [3]
-- วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1 (ELECTIVE IN DATA ENGINEERING 1) – รหัส 06026xxx, 3 หน่วยกิต (3-0-6) หรือ (2-2-5) [3]
-ในภาคการศึกษาที่ 2 ปีที่ 3 มีการเลือกเพิ่มเติมจากกลุ่มเดียวกัน ได้แก่:
-- วิชาเลือกกลุ่มวิทยาการข้อมูล 2 (ELECTIVE IN DATA SCIENCE 2) – รหัส 06026xxx, 3 หน่วยกิต (3-0-6) หรือ (2-2-5) [3]
-- วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 2 (ELECTIVE IN STATISTICAL ANALYTICS 2) – รหัส 06026xxx, 3 หน่วยกิต (3-0-6) หรือ (2-2-5) [3]
-- วิชาเลือกกลุ่มวิศวกรรมข้อมูล 2 (ELECTIVE IN DATA ENGINEERING 2) – รหัส 06026xxx, 3 หน่วยกิต (3-0-6) หรือ (2-2-5) [3]
-นอกจากนี้ ยังมีวิชาเลือกในกลุ่มวิชาเลือกกลุ่มวิทยาการข้อมูล 3 และ 4 สำหรับภาคการศึกษาที่ 2 ปีที่ 3 เช่นกัน [4]
-ดังนั้น นักศึกษาต้องเลือกแขนง (หรือโมดูล) จากรายวิชาใน 3 กลุ่มย่อย ได้แก่ วิทยาการข้อมูล, การวิเคราะห์เชิงสถิติ</t>
+          <t>ใช่ หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ได้ โดยมีแขนงให้เลือก 3 แขนง ดังนี้:
+- กลุ่มวิทยาการข้อมูล (Elective in Data Science)  
+- กลุ่มการวิเคราะห์เชิงสถิติ (Elective in Statistical Analytics)  
+- กลุ่มวิศวกรรมข้อมูล (Elective in Data Engineering)  
+[3][4][6]</t>
         </is>
       </c>
       <c r="H25" s="20" t="inlineStr">
@@ -3264,19 +3267,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="L25" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M25" s="20" t="inlineStr">
         <is>
-          <t>ระบุ 3 กลุ่ม (วิทยาการข้อมูล/วิเคราะห์เชิงสถิติ/วิศวกรรมข้อมูล) ได้ แต่ตอบปนรหัสวิชา placeholder 06026xxx ทำให้ไม่ตรงประเด็น</t>
+          <t>ระบุ 3 กลุ่มชัดเจน (วิทยาการข้อมูล/วิเคราะห์เชิงสถิติ/วิศวกรรมข้อมูล) และบอกว่าเลือกได้</t>
         </is>
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>3.98s</t>
+          <t>1.36s</t>
         </is>
       </c>
       <c r="O25" s="18" t="inlineStr">
@@ -3291,7 +3294,7 @@
           <t>H7</t>
         </is>
       </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="B26" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3339,7 +3342,7 @@
       </c>
       <c r="I26" s="16" t="inlineStr">
         <is>
-          <t>คำนวณจากตัวเลขในคำถาม เทียบเกณฑ์ที่ตั้งค่าไว้ในโค้ด (ไม่ผ่าน LLM)</t>
+          <t>คำนวณจากตัวเลขในคำถาม เทียบเกณฑ์ DSBA 2565 ที่ตรวจทานกับ มคอ.2 หน้า 15 (ไม่ผ่าน LLM)</t>
         </is>
       </c>
       <c r="J26" s="15" t="n">
@@ -3362,7 +3365,7 @@
       </c>
       <c r="N26" s="15" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="O26" s="18" t="inlineStr">
@@ -3377,7 +3380,7 @@
           <t>C1</t>
         </is>
       </c>
-      <c r="B27" s="25" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทาย</t>
         </is>
@@ -3404,20 +3407,10 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>การเปรียบเทียบหลักสูตร IT 2560 (เล่มเก่า) กับ IT 2565 (เล่มปัจจุบัน):
-1. การปรับโครงสร้างหน่วยกิตรวมตลอดหลักสูตร:
-   - หลักสูตร IT 2560 (เดิม): กำหนดหน่วยกิตรวมตลอดหลักสูตรไว้ **130 หน่วยกิต** (มคอ.2 หน้า 18)
-   - หลักสูตร IT 2565 (ปัจจุบัน): ปรับลดหน่วยกิตรวมลงเหลือ **129 หน่วยกิต** (มคอ.2 หน้า 20) ปรับลดลง 1 หน่วยกิตเพื่อเพิ่มความยืดหยุ่นในการเรียน
-2. การปรับโครงสร้างแขนงวิชาและกลุ่มวิชาเลือก:
-   - หลักสูตร IT 2560: จัดแบ่งเป็น 3 แขนงวิชาแบบดั้งเดิมอย่างชัดเจน ได้แก่
-     1) วิศวกรรมซอฟต์แวร์ (Software Engineering)
-     2) เทคโนโลยีเครือข่ายและระบบ (Network and System Technology)
-     3) สื่อประสมและการพัฒนาเกม (Multimedia and Game Development)
-   - หลักสูตร IT 2565: ปรับการจัดกลุ่มวิชาใหม่ โดยจัดเป็น 3 กลุ่มวิชาพื้นฐาน และจัดกลุ่มวิชาเลือกเป็น 3 โมดูลอาชีพ (Professional Career Modules) ได้แก่
-     • M1: Full-Stack Web Developer
-     • M2: Network and System Engineer
-     • M3: Game Developer
-     โดยเน้นการเรียนรู้แบบบูรณาการตามเส้นทางอาชีพและโครงงานจริง (หน้า 372)</t>
+          <t>1. หลักสูตร IT 2565 ปรับโครงสร้างหน่วยกิตรวมเพิ่มขึ้น 1 หน่วยกิต (จาก 94 เป็น 93 หน่วยกิต) โดยลดหน่วยกิตกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศจาก 6 เป็น 3 หน่วยกิต และเพิ่มกลุ่มวิชาเลือกเป็น 3 โมดูลอาชีพ พร้อมขยายกลุ่มวิชาเฉพาะด้านจาก 46 เป็น 57 หน่วยกิต
+2. โครงสร้างแขนงวิชาเปลี่ยนจาก "กลุ่มเชี่ยวชาญเฉพาะ" หรือ "แขนงวิชา" แบบบังคับเลือก 3 แขนง (วิศวกรรมซอฟต์แวร์, เทคโนโลยีเครือข่ายและระบบ, การพัฒนาสื่อประสมและเกม) มาเป็น "กลุ่มวิชาพื้นฐาน" 3 กลุ่มที่เน้นทักษะอาชีพ โดยนักศึกษาเลือกผ่าน 1 กลุ่มจาก 3 กลุ่ม ได้แก่ Software Development, IT Infrastructure, และ Multimedia for Interactive Media, Web and Game Development
+3. วิชาที่เพิ่มเข้ามาในหลักสูตรใหม่ เช่น การพัฒนาคลาวด์แอปพลิเคชัน (06016430), การทดสอบอัตโนมัติในรูปแบบอไจล์ (06016433), และการประมวลทางกายภาพ (06016409) จัดอยู่ในกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศ ซึ่งจัดเป็น 3 โมดูลอาชีพ (M1-M3) ตามหลักฐานจากหน้า 378 ของหลักสูตร IT 2565
+4. วิชาที่ยกเลิก เช่น การจัดการโซ่อุปทานและโลจิสติกส์ (06016371) และการพัฒนาเกมขั้นสูง (06016348) ไม่ได้ถูกนำกลับมาในหลักสูตรใหม่ แต่แทนที่ด้วยวิชาใหม่ในโมดูลอาชีพที่สอดคล้องกับแนวโน้มตลาด เช่น M3: Game Developer ซึ่งมีวิชา 06016447 (Fundamental Game Development with Game Engine) เป็นต้น</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">
@@ -3426,32 +3419,32 @@
 (หน้าที่ระบบคืนมา: IT 2560 หน้า 282, 281, 279, 280; IT 2565 หน้า 371, 374, 378, 372)</t>
         </is>
       </c>
-      <c r="I27" s="22" t="inlineStr">
-        <is>
-          <t>คำตอบสำเร็จรูปที่เขียนไว้ในโค้ด (hard-coded) — ไม่ได้ดึงจากฐานข้อมูลตอนถาม</t>
+      <c r="I27" s="20" t="inlineStr">
+        <is>
+          <t>intent เทียบเวอร์ชัน (รายชื่อวิชาจากฐานข้อมูล) → Typhoon เรียบเรียง</t>
         </is>
       </c>
       <c r="J27" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L27" s="24" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="K27" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L27" s="25" t="inlineStr">
+        <is>
+          <t>ผิด</t>
         </is>
       </c>
       <c r="M27" s="20" t="inlineStr">
         <is>
-          <t>130 → 129 หน่วยกิตถูก แต่ส่วนแขนงวิชาแจ้งว่า 2560 มี 3 แขนง และ 2565 เป็น 3 โมดูล ซึ่งต่างจากเฉลย (เฉลยว่า 2565 มี 3 แขนง) ยังไม่ได้ยืนยันกับ PDF ต้นฉบับ</t>
+          <t>ตัวเลขหน่วยกิตรวมผิด/ขัดกันเอง (อ้าง 94→93 หน่วยกิต 'เพิ่มขึ้น 1' ทั้งที่ฐานข้อมูลมี IT 2565 = 129) เพราะ intent เทียบเวอร์ชันจับคู่คำว่า 'เปรียบเทียบ' แล้วป้อนรายชื่อวิชาให้ LLM เรียบเรียง ไม่มีข้อมูลหน่วยกิตรวมของ IT 2560 ในฐานข้อมูล</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>4.86s</t>
         </is>
       </c>
       <c r="O27" s="18" t="inlineStr">
@@ -3466,7 +3459,7 @@
           <t>C2</t>
         </is>
       </c>
-      <c r="B28" s="25" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทาย</t>
         </is>
@@ -3495,12 +3488,11 @@
         <is>
           <t>จากการวิเคราะห์ไฟล์เอกสารหลักสูตรในฐานข้อมูลระบบ (Document Metadata &amp; Cryptographic Hash):
 1. คู่หลักสูตรที่ใช้ไฟล์เอกสารเล่มเดียวกันทุกประการ:
-   - ระดับปริญญาโท: Doctorals_Degree/PH_D_AITBA2569_current.pdf
-   - ระดับปริญญาเอก: Masters_Degree/M_AITBA2569_current.pdf
+   - ไฟล์ที่ 1: Doctorals_Degree/PH_D_AITBA2569_current.pdf (ระดับที่ระบบตรวจพบจากเนื้อหา: master)
+   - ไฟล์ที่ 2: Masters_Degree/M_AITBA2569_current.pdf (ระดับที่ระบบตรวจพบจากเนื้อหา: master)
    ข้อสังเกตเชิงลึก (Provenance &amp; Cryptographic Hash Verification):
    - ค่า Cryptographic Hash (SHA-256) ตรงกันทุกตัวอักษร: 17e982fc74c2c2bc4d9181c0615e6a90c23fff9700ef3652beb37d17f0f9e24b
-   - ขนาดไฟล์เท่ากันทุกไบต์: 12,285,167 ไบต์ และมีจำนวน 252 หน้าเท่ากัน 100%
-   - หน้าปกและเนื้อหาภายในของไฟล์ระดับ ป.เอก ระบุชื่อหลักสูตรเป็น 'หลักสูตรวิทยาศาสตรมหาบัณฑิต' (วท.ม.) เช่นเดียวกับเล่ม ป.โท เนื่องจากผู้จัดทำชุดข้อมูลได้ใช้ไฟล์ของระดับปริญญาโทบรรจุไว้ทั้งสองตำแหน่งตามที่บันทึกไว้ใน readme.txt</t>
+   - ขนาดไฟล์เท่ากันทุกไบต์: 12,285,167 ไบต์ และมีจำนวน 252 หน้าเท่ากัน 100%</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">
@@ -3511,7 +3503,7 @@
       </c>
       <c r="I28" s="16" t="inlineStr">
         <is>
-          <t>ดึงจากตาราง document_relation (SQL) แล้วใส่ในเทมเพลตข้อความ — ไม่ผ่าน LLM</t>
+          <t>ดึงจากตาราง document_relation (SQL) ใส่ในเทมเพลตข้อความ — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J28" s="15" t="n">
@@ -3522,19 +3514,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L28" s="24" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="L28" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M28" s="16" t="inlineStr">
         <is>
-          <t>พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง แต่สลับป้ายกำกับ ป.โท/ป.เอก ของสองไฟล์ (เทมเพลตกำหนดป้ายตามลำดับ from/to ไม่ได้อ่านจาก degree_level)</t>
+          <t>พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง และระบุระดับที่ตรวจพบจากเนื้อหา (master ทั้งคู่) ตามที่ฐานข้อมูลเก็บ</t>
         </is>
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.27s</t>
         </is>
       </c>
       <c r="O28" s="18" t="inlineStr">
@@ -3549,7 +3541,7 @@
           <t>C3</t>
         </is>
       </c>
-      <c r="B29" s="25" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทาย</t>
         </is>
@@ -3576,49 +3568,43 @@
       </c>
       <c r="G29" s="20" t="inlineStr">
         <is>
-          <t>การเปรียบเทียบหลักสูตร DSBA 2565 แผนปกติ (ไม่ทำสหกิจศึกษา) กับ แผนสหกิจศึกษา (มคอ.2 หน้า 15, 22, 29-30):
-1. ภาคเรียนที่มีความแตกต่างกัน:
-   - แตกต่างกันอย่างชัดเจนใน **ชั้นปีที่ 4 ภาคการศึกษาที่ 2** (ส่วนปีที่ 1 ถึงปีที่ 4 ภาคการศึกษาที่ 1 ทั้งสองแผนเรียนวิชาแกนและวิชาบังคับเหมือนกัน)
-2. รายวิชาที่มีความแตกต่างกันในภาคเรียนดังกล่าว:
-   - **แผนปกติ (ไม่ทำสหกิจศึกษา):** นักศึกษาจะลงเรียนรายวิชาในคณะ รวม 6 หน่วยกิต ได้แก่
-     • 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 (PROJECT IN DATA SCIENCE AND BUSINESS ANALYTICS 2) — 3(0-9-0)
-     • วิชาเลือกในกลุ่มวิชาชีพเฉพาะด้าน หรือวิชาเลือกเสรี อีก 1 วิชา — 3 หน่วยกิต
-   - **แผนสหกิจศึกษา:** นักศึกษาจะออกไปปฏิบัติงานเต็มเวลา ณ สถานประกอบการเป็นเวลาไม่น้อยกว่า 16 สัปดาห์ (1 ภาคการศึกษาเต็ม) โดยลงทะเบียนเพียงวิชาเดียว:
-     • 06026245 สหกิจศึกษา (COOPERATIVE EDUCATION) หรือ 06026250 สหกิจศึกษาต่างประเทศ — จำนวน 6 หน่วยกิต</t>
+          <t>1. แผนปกติและแผนสหกิจศึกษาของหลักสูตร DSBA 2565 มีความแตกต่างกันในภาคการศึกษาที่ 3 ของปีที่ 3 และภาคการศึกษาที่ 1 ของปีที่ 4 โดยมีวิชาสหกิจศึกษา (06026259) แทนวิชาเลือกในแผนปกติ
+2. แผนสหกิจศึกษาเปิดภาคเรียนที่ 3 ปีที่ 3 และภาคเรียนที่ 1 ปีที่ 4 สำหรับวิชาสหกิจศึกษา (รหัส 06026259, 6 หน่วยกิต) ซึ่งไม่มีในแผนปกติ ขณะที่แผนปกติใช้วิชาเลือกแทนในช่วงเวลาเดียวกัน ตามโครงสร้างหลักสูตรที่ระบุว่าแผนสหกิจศึกษาต้องเรียนวิชานี้ 6 หน่วยกิต ตั้งแต่ภาคเรียนที่ 3 ปีที่ 3 เป็นต้นไป
+3. อ้างข้อมูลจาก: วิชาบังคับก่อน – ไม่มี, ภาค/ปีที่เปิดสอน – ภาคเรียนที่ 3 ปีที่ 3 และภาคเรียนที่ 1 ปีที่ 4, ประเภทวิชา – บังคับ (สหกิจศึกษา)</t>
         </is>
       </c>
       <c r="H29" s="20" t="inlineStr">
         <is>
           <t>แผนการศึกษาเปรียบเทียบ DSBA 2565 (หน้า 15–17)
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 19, 21, 29, 36)</t>
-        </is>
-      </c>
-      <c r="I29" s="22" t="inlineStr">
-        <is>
-          <t>คำตอบสำเร็จรูปที่เขียนไว้ในโค้ด (hard-coded) — ไม่ได้ดึงจากฐานข้อมูลตอนถาม</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 30, 350, 23, 15)</t>
+        </is>
+      </c>
+      <c r="I29" s="20" t="inlineStr">
+        <is>
+          <t>intent เทียบเวอร์ชัน (รายชื่อวิชาจากฐานข้อมูล) → Typhoon เรียบเรียง</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K29" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L29" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
+      <c r="L29" s="25" t="inlineStr">
+        <is>
+          <t>ไม่ตรงเฉลย</t>
         </is>
       </c>
       <c r="M29" s="20" t="inlineStr">
         <is>
-          <t>ต่างกันที่ปี 4 ภาค 2: แผนปกติเรียนโครงงาน 2 + วิชาเลือก, แผนสหกิจเรียนสหกิจศึกษา 6 หน่วยกิต ตรงเฉลย</t>
+          <t>ตอบว่าต่างกันที่ปี 3 ภาค 3 และปี 4 ภาค 1 ด้วยวิชา 06026259 แต่เฉลยว่าต่างที่ปี 4 ภาค 2 (06026245) ยังไม่ได้ยืนยันกับ PDF ว่าฝั่งไหนถูก; intent เทียบเวอร์ชันถูกจับผิดประเภท (ไม่ใช่การเทียบแผน)</t>
         </is>
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>2.69s</t>
         </is>
       </c>
       <c r="O29" s="18" t="inlineStr">
@@ -3690,12 +3676,12 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>C1: ถูกบางส่วน; C2: ถูกบางส่วน; C3: ถูกครบ</t>
+          <t>C1: ผิด; C2: ถูกครบ; C3: ไม่ตรงเฉลย</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>C1 และ C3 ตอบด้วยข้อความสำเร็จรูปในโค้ด; C2 ดึงจากตาราง document_relation แต่ป้าย ป.โท/ป.เอก สลับ; C1 ส่วนแขนงวิชายังไม่ได้ยืนยันกับ PDF</t>
+          <t>C1: ตัวเลขหน่วยกิตรวมที่ LLM เรียบเรียงผิด/ขัดกันเอง; C3: ไม่ตรงเฉลย (ยังไม่ได้ยืนยันกับ PDF ว่าฝั่งไหนถูก) เพราะ intent เทียบเวอร์ชันถูกจับผิดประเภท; C2: ดึงจากตาราง document_relation ถูกต้อง</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3698,7 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>ระดับยาก 7 ข้อ เฉลี่ย 1.16s ช้าสุด 3.98s · ทั้ง 28 ข้อ ต่ำกว่า 5s 28/28</t>
+          <t>ระดับยาก 7 ข้อ เฉลี่ย 0.86s ช้าสุด 1.58s · ทั้ง 28 ข้อ ต่ำกว่า 5s 28/28</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">

</xml_diff>

<commit_message>
fix(query): handle cross-version credit, multi-version retrieval and prerequisite chains
- rule table: total credits for every bachelor version incl. old editions, each with
  provenance (book page) - DSBA/BIT current values also match teacher GT
- new credit comparison intent across versions/programs (from rule table)
- hybrid retrieval searches every version the question names
- course-name set-diff only when the question really compares versions about courses
- plan/graduate-programme questions no longer routed to topic course search
- prerequisite extractor: catch courses with two prerequisites; show multi-level chains;
  drops 3 false prerequisites (book says none)
- evaluation: 28-question set re-run and re-reviewed (24 correct / 3 partial / 1 wrong);
  20 extra challenge questions written from the book before running, all reported
  (docs/challenge_extended.json, new sheet in tester.xlsx)
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Test Cases &amp; Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenge Criteria (Measured)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenge (extended)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$29</definedName>
@@ -612,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -719,7 +720,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ถูกครบ 25 · ถูกบางส่วน 1 · ผิด/ไม่ตรงเฉลย 2 · ยังไม่ได้ตรวจ 0</t>
+          <t>ถูกครบ 24 · ถูกบางส่วน 3 · ผิด/ไม่ตรงเฉลย 1 · ยังไม่ได้ตรวจ 0</t>
         </is>
       </c>
     </row>
@@ -731,7 +732,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>เฉลี่ย 0.65s · เร็วสุด 0.05s · ช้าสุด 4.86s · ต่ำกว่า 5s 28/28 ข้อ</t>
+          <t>เฉลี่ย 0.77s · เร็วสุด 0.06s · ช้าสุด 3.86s · ต่ำกว่า 5s 28/28 ข้อ</t>
         </is>
       </c>
     </row>
@@ -819,12 +820,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>0.27</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>1.12</t>
         </is>
       </c>
     </row>
@@ -851,12 +852,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>0.70</t>
+          <t>0.74</t>
         </is>
       </c>
     </row>
@@ -873,22 +874,22 @@
         <v>7</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>3.29</t>
         </is>
       </c>
     </row>
@@ -908,19 +909,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>2.61</t>
+          <t>2.52</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>3.86</t>
         </is>
       </c>
     </row>
@@ -937,22 +938,22 @@
         <v>27</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E20" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="10" t="n">
-        <v>2</v>
-      </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>3.86</t>
         </is>
       </c>
     </row>
@@ -987,35 +988,43 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้จึงมาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM) ผลของ C1 และ C3 จึงไม่ดี ซึ่งตรงกับที่ระบบทำได้จริง</t>
+          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ เช่น M8 รันซ้ำ 8 ครั้งพบเลข 12 ในคำตอบ 5 ครั้ง; H5 พบ 8 ครั้งจาก 8</t>
+          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (เขียนเฉลยจากเล่มก่อนรัน รายงานทุกข้อ) อยู่ในแผ่น Challenge (extended)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
+          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
           <t>6) เฉลยข้อ H4 เดิมเขียน 48 วิชา แต่ฐานข้อมูลปัจจุบันให้ 52 (DSBA 2560 71 ชื่อ / 2565 75 ชื่อ) ผลของระบบตรงกับฐานข้อมูล</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="A29:H29"/>
@@ -1222,7 +1231,7 @@
       </c>
       <c r="N2" s="15" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O2" s="18" t="inlineStr">
@@ -1303,7 +1312,7 @@
       </c>
       <c r="N3" s="19" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.24s</t>
         </is>
       </c>
       <c r="O3" s="18" t="inlineStr">
@@ -1382,7 +1391,7 @@
       </c>
       <c r="N4" s="15" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.09s</t>
         </is>
       </c>
       <c r="O4" s="18" t="inlineStr">
@@ -1553,7 +1562,7 @@
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>0.89s</t>
+          <t>1.12s</t>
         </is>
       </c>
       <c r="O6" s="18" t="inlineStr">
@@ -1645,7 +1654,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O7" s="18" t="inlineStr">
@@ -1723,7 +1732,7 @@
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.08s</t>
         </is>
       </c>
       <c r="O8" s="18" t="inlineStr">
@@ -1808,7 +1817,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.28s</t>
         </is>
       </c>
       <c r="O9" s="18" t="inlineStr">
@@ -1886,7 +1895,7 @@
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="O10" s="18" t="inlineStr">
@@ -1964,7 +1973,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O11" s="18" t="inlineStr">
@@ -2049,7 +2058,7 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.32s</t>
         </is>
       </c>
       <c r="O12" s="18" t="inlineStr">
@@ -2138,7 +2147,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.37s</t>
         </is>
       </c>
       <c r="O13" s="18" t="inlineStr">
@@ -2334,7 +2343,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.31s</t>
         </is>
       </c>
       <c r="O15" s="18" t="inlineStr">
@@ -2429,7 +2438,7 @@
       </c>
       <c r="N16" s="15" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O16" s="18" t="inlineStr">
@@ -2556,7 +2565,7 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) หมวดวิชาเฉพาะ กลุ่มวิชาชีพเฉพาะด้าน มีจำนวน 12 หน่วยกิต [6]</t>
+          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) หมวดวิชาเฉพาะ กลุ่มวิชาชีพเฉพาะด้าน มีจำนวนหน่วยกิตทั้งหมด 12 หน่วยกิต [6]</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
@@ -2585,12 +2594,12 @@
       </c>
       <c r="M18" s="16" t="inlineStr">
         <is>
-          <t>ตอบ 12 หน่วยกิตถูกในรอบนี้ แต่ไม่คงที่: รันซ้ำ 8 ครั้ง พบเลข 12 ในคำตอบ 5 ครั้ง (ที่เหลือตอบ 6 หน่วยกิตของอีกกลุ่ม) ผ่าน retrieval + LLM</t>
+          <t>ตอบ 12 หน่วยกิต (กลุ่มวิชาชีพเฉพาะด้าน) ถูกในรอบนี้ แต่ไม่คงที่ ผ่าน retrieval + LLM บางรอบตอบ 6 หน่วยกิตของอีกกลุ่ม</t>
         </is>
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>0.70s</t>
+          <t>0.74s</t>
         </is>
       </c>
       <c r="O18" s="18" t="inlineStr">
@@ -2670,7 +2679,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.20s</t>
         </is>
       </c>
       <c r="O19" s="18" t="inlineStr">
@@ -2811,7 +2820,7 @@
       </c>
       <c r="N20" s="15" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.16s</t>
         </is>
       </c>
       <c r="O20" s="18" t="inlineStr">
@@ -2854,7 +2863,7 @@
       <c r="G21" s="20" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถเรียนวิชา "ระบบฐานข้อมูลแบบกระจาย" (06026246) ในปีที่ 4 ภาคการศึกษาที่ 1 ได้ เนื่องจากเป็นวิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน ซึ่งไม่มีวิชาบังคับก่อนกำหนดไว้ และอยู่ในหลักสูตร DSBA 2565 ภาคการศึกษาที่ 1 ปีที่ 4 โดยมีหน่วยกิต 3 (3-0-6) ประเภทวิชาเลือก.</t>
+นักศึกษาสามารถเรียนวิชาฐานข้อมูลในปีที่ 4 ได้ เนื่องจากหลักสูตร DSBA 2565 มีวิชาบังคับในปีที่ 4 ภาคเรียนที่ 1 คือ 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 ซึ่งเป็นวิชาที่เกี่ยวข้องกับการประยุกต์ใช้ฐานข้อมูล และมีวิชาเลือกในกลุ่มวิชาศึกษาทั่วไปหรือวิชาเลือกเสรีที่อาจครอบคลุมเนื้อหาด้านฐานข้อมูลได้ โดยไม่มีข้อกำหนดวิชาบังคับก่อนที่จำกัดการเรียนวิชานี้ไว้เฉพาะปีก่อนหน้า ทั้งนี้ วิชาที่เกี่ยวข้องกับฐานข้อมูล เช่น 06026246 ระบบฐานข้อมูลแบบกระจาย เปิดสอนในปีที่ 4 ภาคเรียนที่ 2 ภายใต้กลุ่มวิชาการศึกษาทางเลือก ประเภทวิชาเลือก 6 หน่วยกิต สำหรับนักศึกษาที่ไม่เข้าร่วมสหกิจศึกษา จึงยืนยันได้ว่าเรียนวิชาฐานข้อมูลในปีที่ 4 ได้</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -2876,19 +2885,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L21" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
         </is>
       </c>
       <c r="M21" s="20" t="inlineStr">
         <is>
-          <t>ตอบ 'ได้' และชี้วิชา 06026246 ระบบฐานข้อมูลแบบกระจาย ปี 4 ภาค 1 ไม่มีวิชาบังคับก่อน ตรงเฉลย</t>
+          <t>ตอบ 'ได้' ถูก และกล่าวถึง 06026246 ระบบฐานข้อมูลแบบกระจาย แต่ระบุภาคเรียนเป็นปี 4 ภาค 2 (เฉลยว่าปี 4 ภาค 1) และอ้างโครงงาน 2 ว่าเกี่ยวกับฐานข้อมูลโดยไม่มีหลักฐาน</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>1.58s</t>
+          <t>2.52s</t>
         </is>
       </c>
       <c r="O21" s="18" t="inlineStr">
@@ -2965,7 +2974,7 @@
       </c>
       <c r="N22" s="15" t="inlineStr">
         <is>
-          <t>1.53s</t>
+          <t>1.37s</t>
         </is>
       </c>
       <c r="O22" s="18" t="inlineStr">
@@ -3165,7 +3174,18 @@
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปรับปรุง พ.ศ. 2565 มีหมวดวิชาเฉพาะ (กลุ่มวิชาชีพเฉพาะด้าน) จำนวน 12 หน่วยกิต [7].</t>
+          <t>หมวดวิชาเฉพาะในหลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) มีการจัดแบ่งเป็นกลุ่มวิชาชีพเฉพาะด้าน ซึ่งมีจำนวนหน่วยกิตทั้งสิ้น 12 หน่วยกิต [7] โดยกลุ่มนี้ประกอบด้วยรายวิชาที่เน้นทักษะความเชี่ยวชาญเฉพาะทางด้านวิทยาการข้อมูล ได้แก่:
+- ปัญญาประดิษฐ์ (Artificial Intelligence) – 3 หน่วยกิต (3-0-6) [7]  
+- การเรียนรู้ของเครื่อง (Machine Learning) – 3 หน่วยกิต (3-0-6) [7]  
+- การเรียนรู้เชิงลึก (Deep Learning) – 3 หน่วยกิต (2-2-5) [7]  
+- การประมวลผลภาษาธรรมชาติ (Natural Language Processing) – 3 หน่วยกิต (3-0-6) [7]  
+- การทำเหมืองข้อมูลกระบวนการ (Process Mining) – 3 หน่วยกิต (3-0-6) [7]  
+- การค้นคืนสารสนเทศ (Information Retrieval) – 3 หน่วยกิต (3-0-6) [7]  
+- คอมพิวเตอร์วิชัน (Computer Vision) – 3 หน่วยกิต (3-0-6) [7]  
+- การประมวลผลภาพ (Image Processing) – 3 หน่วยกิต (3-0-6) [7]  
+- การแปลงข้อมูลและการรู้จำรูปภาพ (Image Transformation and Recognition) – 3 หน่วยกิต (3-0-6) [7]  
+- การเรียนรู้เชิงลึกสำหรับการวิเคราะห์ภาพและวีดิโอทางการแพทย์ (Deep Learning in Medical Image and Video Analysis) – 3 หน่วยกิต (2-2-5) [7]  
+ทั้งหมดนี้เป็นรายวิชาในกลุ่มวิชาชีพเฉพาะด้าน รวมทั้งสิ้น 12 หน่วยกิต [7]</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -3194,12 +3214,12 @@
       </c>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>ตอบ 12 หน่วยกิต (รันซ้ำ 8 ครั้ง พบเลข 12 ทุกครั้ง) ผ่าน retrieval + LLM</t>
+          <t>ตอบ 12 หน่วยกิต (กลุ่มวิชาชีพเฉพาะด้าน) ถูก ผ่าน retrieval + LLM</t>
         </is>
       </c>
       <c r="N24" s="15" t="inlineStr">
         <is>
-          <t>1.03s</t>
+          <t>3.29s</t>
         </is>
       </c>
       <c r="O24" s="18" t="inlineStr">
@@ -3241,10 +3261,10 @@
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>ใช่ หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ได้ โดยมีแขนงให้เลือก 3 แขนง ดังนี้:
-- กลุ่มวิทยาการข้อมูล (Elective in Data Science)  
-- กลุ่มการวิเคราะห์เชิงสถิติ (Elective in Statistical Analytics)  
-- กลุ่มวิศวกรรมข้อมูล (Elective in Data Engineering)  
+          <t>ใช่ ปีที่ 3 ต้องเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") โดยมี 3 แขนงให้เลือก ได้แก่:
+- กลุ่มวิทยาการข้อมูล (Data Science)  
+- กลุ่มการวิเคราะห์เชิงสถิติ (Statistical Analytics)  
+- กลุ่มวิศวกรรมข้อมูล (Data Engineering)  
 [3][4][6]</t>
         </is>
       </c>
@@ -3274,12 +3294,12 @@
       </c>
       <c r="M25" s="20" t="inlineStr">
         <is>
-          <t>ระบุ 3 กลุ่มชัดเจน (วิทยาการข้อมูล/วิเคราะห์เชิงสถิติ/วิศวกรรมข้อมูล) และบอกว่าเลือกได้</t>
+          <t>ระบุ 3 กลุ่มชัดเจน (วิทยาการข้อมูล/วิเคราะห์เชิงสถิติ/วิศวกรรมข้อมูล) และบอกว่าต้องเลือก</t>
         </is>
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>1.36s</t>
+          <t>1.04s</t>
         </is>
       </c>
       <c r="O25" s="18" t="inlineStr">
@@ -3365,7 +3385,7 @@
       </c>
       <c r="N26" s="15" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="O26" s="18" t="inlineStr">
@@ -3407,44 +3427,43 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>1. หลักสูตร IT 2565 ปรับโครงสร้างหน่วยกิตรวมเพิ่มขึ้น 1 หน่วยกิต (จาก 94 เป็น 93 หน่วยกิต) โดยลดหน่วยกิตกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศจาก 6 เป็น 3 หน่วยกิต และเพิ่มกลุ่มวิชาเลือกเป็น 3 โมดูลอาชีพ พร้อมขยายกลุ่มวิชาเฉพาะด้านจาก 46 เป็น 57 หน่วยกิต
-2. โครงสร้างแขนงวิชาเปลี่ยนจาก "กลุ่มเชี่ยวชาญเฉพาะ" หรือ "แขนงวิชา" แบบบังคับเลือก 3 แขนง (วิศวกรรมซอฟต์แวร์, เทคโนโลยีเครือข่ายและระบบ, การพัฒนาสื่อประสมและเกม) มาเป็น "กลุ่มวิชาพื้นฐาน" 3 กลุ่มที่เน้นทักษะอาชีพ โดยนักศึกษาเลือกผ่าน 1 กลุ่มจาก 3 กลุ่ม ได้แก่ Software Development, IT Infrastructure, และ Multimedia for Interactive Media, Web and Game Development
-3. วิชาที่เพิ่มเข้ามาในหลักสูตรใหม่ เช่น การพัฒนาคลาวด์แอปพลิเคชัน (06016430), การทดสอบอัตโนมัติในรูปแบบอไจล์ (06016433), และการประมวลทางกายภาพ (06016409) จัดอยู่ในกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศ ซึ่งจัดเป็น 3 โมดูลอาชีพ (M1-M3) ตามหลักฐานจากหน้า 378 ของหลักสูตร IT 2565
-4. วิชาที่ยกเลิก เช่น การจัดการโซ่อุปทานและโลจิสติกส์ (06016371) และการพัฒนาเกมขั้นสูง (06016348) ไม่ได้ถูกนำกลับมาในหลักสูตรใหม่ แต่แทนที่ด้วยวิชาใหม่ในโมดูลอาชีพที่สอดคล้องกับแนวโน้มตลาด เช่น M3: Game Developer ซึ่งมีวิชา 06016447 (Fundamental Game Development with Game Engine) เป็นต้น</t>
+          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูล แทนการเลือก "แขนงวิชา" 3 แขนง
+2. หลักสูตร IT 2565 ลดหน่วยกิตรวมจาก 130 เป็น 129 โดยปรับโครงสร้างหมวดวิชาเฉพาะ: กลุ่มวิชาเฉพาะด้านเพิ่มจาก 46 เป็น 57 หน่วยกิต แต่กลุ่มวิชาบังคับเฉพาะแขนงลดจาก 30 เป็น 15 หน่วยกิต และเพิ่มกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศเป็น 9 หน่วยกิต (จากเดิม 6 หน่วยกิต) พร้อมจัดเป็น 3 โมดูลอาชีพ (M1-M3) ตามหลักฐานจากมคอ.2 IT 2565 หน้า 370, 374, 376, 378
+3. ข้อมูลอ้างอิง: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18; IT 2565 หน้า 6), โครงสร้างกลุ่มวิชาเฉพาะ (IT 2565 หน้า 374, 376, 378), ประเภทวิชา (บังคับ/เลือก), ปีที่เปิดสอน (IT 2560 เริ่มภาค 1/2560; IT 2565 เริ่มภาค 1/2565)</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">
         <is>
           <t>IT2560_old.pdf (หน้า 10–18) เปรียบเทียบกับ IT2565_current.pdf (หน้า 15–25, 372)
-(หน้าที่ระบบคืนมา: IT 2560 หน้า 282, 281, 279, 280; IT 2565 หน้า 371, 374, 378, 372)</t>
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 378, 376, 370, 374; IT 2560 หน้า 281, 279, 282, 284)</t>
         </is>
       </c>
       <c r="I27" s="20" t="inlineStr">
         <is>
-          <t>intent เทียบเวอร์ชัน (รายชื่อวิชาจากฐานข้อมูล) → Typhoon เรียบเรียง</t>
+          <t>หน่วยกิตรวมจากตาราง rule + hybrid retrieval → Typhoon เรียบเรียง</t>
         </is>
       </c>
       <c r="J27" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="K27" s="15" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L27" s="25" t="inlineStr">
-        <is>
-          <t>ผิด</t>
+        <v>10</v>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L27" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
         </is>
       </c>
       <c r="M27" s="20" t="inlineStr">
         <is>
-          <t>ตัวเลขหน่วยกิตรวมผิด/ขัดกันเอง (อ้าง 94→93 หน่วยกิต 'เพิ่มขึ้น 1' ทั้งที่ฐานข้อมูลมี IT 2565 = 129) เพราะ intent เทียบเวอร์ชันจับคู่คำว่า 'เปรียบเทียบ' แล้วป้อนรายชื่อวิชาให้ LLM เรียบเรียง ไม่มีข้อมูลหน่วยกิตรวมของ IT 2560 ในฐานข้อมูล</t>
+          <t>หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มี provenance หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่า 2565 มี 3 แขนง) และตัวเลขหน่วยกิตย่อยของกลุ่มวิชามาจาก LLM ยังไม่ได้ยืนยันกับเล่ม</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>4.86s</t>
+          <t>3.86s</t>
         </is>
       </c>
       <c r="O27" s="18" t="inlineStr">
@@ -3526,7 +3545,7 @@
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="O28" s="18" t="inlineStr">
@@ -3568,9 +3587,9 @@
       </c>
       <c r="G29" s="20" t="inlineStr">
         <is>
-          <t>1. แผนปกติและแผนสหกิจศึกษาของหลักสูตร DSBA 2565 มีความแตกต่างกันในภาคการศึกษาที่ 3 ของปีที่ 3 และภาคการศึกษาที่ 1 ของปีที่ 4 โดยมีวิชาสหกิจศึกษา (06026259) แทนวิชาเลือกในแผนปกติ
-2. แผนสหกิจศึกษาเปิดภาคเรียนที่ 3 ปีที่ 3 และภาคเรียนที่ 1 ปีที่ 4 สำหรับวิชาสหกิจศึกษา (รหัส 06026259, 6 หน่วยกิต) ซึ่งไม่มีในแผนปกติ ขณะที่แผนปกติใช้วิชาเลือกแทนในช่วงเวลาเดียวกัน ตามโครงสร้างหลักสูตรที่ระบุว่าแผนสหกิจศึกษาต้องเรียนวิชานี้ 6 หน่วยกิต ตั้งแต่ภาคเรียนที่ 3 ปีที่ 3 เป็นต้นไป
-3. อ้างข้อมูลจาก: วิชาบังคับก่อน – ไม่มี, ภาค/ปีที่เปิดสอน – ภาคเรียนที่ 3 ปีที่ 3 และภาคเรียนที่ 1 ปีที่ 4, ประเภทวิชา – บังคับ (สหกิจศึกษา)</t>
+          <t>1. หลักสูตร DSBA 2565 แผนปกติ (ไม่ทำสหกิจ) และแผนสหกิจศึกษาต่างกันเฉพาะในภาคการศึกษาที่ 3 ปีที่ 3 เป็นต้นไป โดยแผนสหกิจศึกษาต้องเรียนวิชาสหกิจศึกษา (06026259) 6 หน่วยกิต แทนวิชาเลือกเสรีหรือวิชาเฉพาะด้าน
+2. แผนปกติไม่มีวิชาสหกิจศึกษา แต่ต้องเรียนวิชาเลือกเสรี 6 หน่วยกิต ขณะที่แผนสหกิจศึกษาแทนด้วยวิชาสหกิจศึกษา (06026259) ซึ่งเป็นวิชาบังคับก่อนไม่มี และเปิดสอนภาคการศึกษาที่ 3 ปีที่ 3 เป็นต้นไป
+3. วิชาที่ต่างกันคือ 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (6 หน่วยกิต) ประเภทวิชาบังคับ ภาคการศึกษาที่ 3 ปีที่ 3 เป็นต้นไป</t>
         </is>
       </c>
       <c r="H29" s="20" t="inlineStr">
@@ -3581,30 +3600,30 @@
       </c>
       <c r="I29" s="20" t="inlineStr">
         <is>
-          <t>intent เทียบเวอร์ชัน (รายชื่อวิชาจากฐานข้อมูล) → Typhoon เรียบเรียง</t>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K29" s="17" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L29" s="25" t="inlineStr">
         <is>
-          <t>ไม่ตรงเฉลย</t>
+          <t>ผิด</t>
         </is>
       </c>
       <c r="M29" s="20" t="inlineStr">
         <is>
-          <t>ตอบว่าต่างกันที่ปี 3 ภาค 3 และปี 4 ภาค 1 ด้วยวิชา 06026259 แต่เฉลยว่าต่างที่ปี 4 ภาค 2 (06026245) ยังไม่ได้ยืนยันกับ PDF ว่าฝั่งไหนถูก; intent เทียบเวอร์ชันถูกจับผิดประเภท (ไม่ใช่การเทียบแผน)</t>
+          <t>ตอบว่าแผนสหกิจต่างที่ปี 3 ภาค 3 แต่เล่ม (DSBA 2565 หน้า 36) วางสหกิจศึกษา 06026259/06026260 ไว้ที่ปี 4 ภาค 2 หมายเหตุ: เฉลยในไฟล์ทดสอบใช้รหัส 06026245 ซึ่งไม่ตรงกับเล่ม และแผนปกติปี 4 ภาค 2 ในเล่ม (หน้า 29) คือวิชาเลือกศึกษาทั่วไป + เลือกเสรี 2 วิชา รวม 9 หน่วยกิต ไม่ใช่โครงงาน 2</t>
         </is>
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>2.69s</t>
+          <t>3.46s</t>
         </is>
       </c>
       <c r="O29" s="18" t="inlineStr">
@@ -3676,12 +3695,12 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>C1: ผิด; C2: ถูกครบ; C3: ไม่ตรงเฉลย</t>
+          <t>C1: ถูกบางส่วน; C2: ถูกครบ; C3: ผิด</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>C1: ตัวเลขหน่วยกิตรวมที่ LLM เรียบเรียงผิด/ขัดกันเอง; C3: ไม่ตรงเฉลย (ยังไม่ได้ยืนยันกับ PDF ว่าฝั่งไหนถูก) เพราะ intent เทียบเวอร์ชันถูกจับผิดประเภท; C2: ดึงจากตาราง document_relation ถูกต้อง</t>
+          <t>C1: หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มี provenance หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่า 2565 มี 3 แขนง) และตัวเลขหน่วยกิตย่อยของกลุ่มวิชามาจาก LLM ยังไม่ได้ยืนยันกับเล่ม · C2: พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง และระบุระดับที่ตรวจพบจากเนื้อหา (master ทั้งคู่) ตามที่ฐานข้อมูลเก็บ · C3: ตอบว่าแผนสหกิจต่างที่ปี 3 ภาค 3 แต่เล่ม (DSBA 2565 หน้า 36) วางสหกิจศึกษา 06026259/06026260 ไว้ที่ปี 4 ภาค 2 หมายเหตุ: เฉลยในไฟล์ทดสอบใช้รหัส 06026245 ซึ่งไม่ตรงกับเล่ม และแผนปกติปี 4 ภาค 2 ในเล่ม (หน้า 29) คือวิชาเลือกศึกษาทั่วไป + เลือกเสรี 2 วิชา รวม 9 หน่วยกิต ไม่ใช่โครงงาน 2</t>
         </is>
       </c>
     </row>
@@ -3698,13 +3717,1129 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>ระดับยาก 7 ข้อ เฉลี่ย 0.86s ช้าสุด 1.58s · ทั้ง 28 ข้อ ต่ำกว่า 5s 28/28</t>
+          <t>ระดับยาก 7 ข้อ เฉลี่ย 1.26s ช้าสุด 3.29s · ทั้ง 28 ข้อ ต่ำกว่า 5s 28/28</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
           <t>วัดบนเซิร์ฟเวอร์ที่โหลดโมเดลแล้ว (warm); การถามครั้งแรกหลังเปิดเซิร์ฟเวอร์แบบ KATRAG_SKIP_WARMUP=1 จะช้ากว่า (โหลด bge-m3) ราว 0.5–1 นาที</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ข้อท้าทายเพิ่มเติม — บันทึกจากการรันวันที่ 2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>เขียนคำถามและเฉลยจากเล่ม มคอ.2 ก่อนรัน แล้วรายงานทุกข้อที่ลอง (ไม่คัดทิ้ง)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ชุด X (8 ข้อ) — ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>ผลล่าสุด: ถูกครบ 5 · บางส่วน 2 · ผิด 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ชุด Y (6 ข้อ) — เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ผลล่าสุด: ถูกครบ 5 · บางส่วน 1 · ผิด 0  (รอบที่ 1 วัดได้ ถูกครบ 3/6 (Y4, Y5, Y6 ผิด) ก่อนแก้รอบที่ 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>ชุด Z (6 ข้อ) — เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>ผลล่าสุด: ถูกครบ 5 · บางส่วน 1 · ผิด 0  (รอบที่ 2 วัดครั้งแรก ถูกครบ 5/6 (Z3 ผิด))</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>ข้อที่</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>ชุด</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>หลักสูตร</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>คำถาม</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>เฉลย (จากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>หน้าที่มาของเฉลย</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>คำตอบจริงจากเซิร์ฟเวอร์</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>ตรวจโดยคน</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>เวลาตอบ (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>X1</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตรของ DSBA ฉบับ 2560 กับฉบับ 2565 ต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>2560 = 126 หน่วยกิต, 2565 = 132 หน่วยกิต ต่างกัน 6 หน่วยกิต (2565 มากกว่า)</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2560 หน้า 17; DSBA2565 หน้า 15</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
+- DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
+สรุป: DSBA 2565 มากกว่า DSBA 2560 อยู่ 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr"/>
+      <c r="J9" s="15" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตร BIT 2560 กับ BIT 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากันหรือไม่</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>เท่ากัน ทั้งสองฉบับ 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>BIT2560 หน้า 17; BIT2565 หน้า 6</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- BIT 2560: 126 หน่วยกิต (มคอ.2 BIT 2560 หน้า 17)
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+สรุป: เท่ากัน (126 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr"/>
+      <c r="J10" s="15" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>X3</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>ระหว่างหลักสูตร DSBA 2565, AIT 2566 และ BIT 2565 หลักสูตรใดมีหน่วยกิตรวมมากที่สุด</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>DSBA 2565 มากที่สุด 132 หน่วยกิต (BIT 2565 = 126, AIT 2566 = 120)</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 15; BIT2565 หน้า 6; AIT2566 หน้า 5</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
+- AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+สรุป: มากที่สุดคือ DSBA 2565 (132 หน่วยกิต) น้อยที่สุดคือ AIT 2566 (120 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr"/>
+      <c r="J11" s="15" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>X4</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>ในแผนสหกิจศึกษาของ DSBA 2565 ต้องลงทะเบียนวิชาสหกิจศึกษาในภาคไหน และกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>ปีที่ 4 ภาคการศึกษาที่ 2 จำนวน 6 หน่วยกิต (06026259 สหกิจศึกษา หรือ 06026260 สหกิจศึกษาต่างประเทศ)</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 36</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>นักศึกษาต้องลงทะเบียนวิชาสหกิจศึกษา 6 หน่วยกิตในภาคการศึกษาที่ 3 หรือภาคการศึกษาที่ 4 ของปีที่ 3 หรือปีที่ 4 ตามลำดับ [5]</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="inlineStr">
+        <is>
+          <t>ผิด</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>ตอบว่าลงสหกิจภาค 3/ภาค 4 ของปี 3/ปี 4 แต่เล่มหน้า 36 คือปี 4 ภาค 2</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>X5</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท IT 2563 กับ 2568 แบ่งแผนการศึกษาต่างกันอย่างไร</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>2563: แผน ก (แบบ ก1, ก2) และแผน ข; 2568: แผน 1 แบบวิชาการ (แบบ 1.1, 1.2) และแผน 2 แบบวิชาชีพ; ทุกแผนเรียน 36 หน่วยกิตเท่ากัน</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>IT2563 หน้า 16; IT2568 หน้า 5</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2563 (IT 2563) มีแผนการศึกษาแบบ ก 1 และ ก 2 ซึ่งรับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ตั้งแต่ปีการศึกษา 2563 ถึง 2567 โดยแผน ก 1 และ ก 2 มีโครงสร้างการรับนักศึกษาและคาดการณ์การสำเร็จการศึกษาเหมือนกัน คือ รับ 5 คนต่อปี ชั้นปีที่ 1 และสำเร็จการศึกษา 5 คนต่อปี ตั้งแต่ปีการศึกษา 2564 เป็นต้นไป [3]
+ส่วนหลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2568 (IT 2568) มีแผนการศึกษา 3 แบบ ได้แก่ แผน 1 แบบวิชาการ แบบ 1.1, แบบ 1.2 และแผน 2 แบบวิชาชีพ โดยแผน 1 แบบวิชาการ รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ตั้งแต่ปีการศึกษา 2568 เป็นต้นไป คาดว่าจะสำเร็จการศึกษา 3 คนต่อปี ตั้งแต่ปีการศึกษา 2569 เป็นต้นไป ส่วนแผน 2 แบบวิชาชีพ รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ตั้งแต่ปีการศึกษา 2568 เป็นต้นไป คาดว่าจะสำเร็จการศึกษา 30 คนต่อปี ตั้งแต่ปีการศึกษา 2569 เป็นต้นไป [2]
+ดังนั้น ความแตกต่างคือ หลักสูตร 2563 มีเพียงแผน ก 1 และ ก 2 รับคนละ 5 คนต่อปี ส่วนหลักสูตร 2568 มีแผนมากกว่า 3 แบบ โดยมีการแบ่งแยกตามประเภทการศึกษา (วิชาการ/วิชาชีพ) และจำนวนรับนักศึกษาต่อปีแตกต่างกันอย่างชัดเจน [2][3]</t>
+        </is>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>อธิบายแผนของ 2568 ถูก แต่ของ 2563 ขาดแผน ข และตอบจำนวนรับนักศึกษาแทนโครงสร้างแผน</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>X6</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>ถ้าจะเรียนวิชาพื้นฐานการเรียนรู้เชิงลึก (Fundamentals of Deep Learning) ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>ต้องผ่านแคลคูลัส 2 (06046401) และพีชคณิตเชิงเส้น (06046402); แคลคูลัส 2 ต้องผ่านแคลคูลัส 1 (06046400) ก่อน; พีชคณิตเชิงเส้นและแคลคูลัส 1 ไม่มีวิชาบังคับก่อน</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 287-288</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06046401 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
+      ↳ ต้องผ่าน 06046400 แคลคูลัส 1 (CALCULUS 1) ก่อน
+    • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>ไล่วิชาบังคับก่อน 2 ชั้นได้ครบ</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>X7</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>AITBA</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท AITBA 2564 กับ 2569 หน่วยกิตที่เรียนตลอดหลักสูตรต่างกันไหม และชื่อแผนการศึกษาเปลี่ยนไปอย่างไร</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตไม่ต่าง ทุกแผน 36 หน่วยกิต; 2564 ใช้แผน ก (ก1, ก2) และแผน ข; 2569 ใช้แผนวิชาการ (แบบ 1.1, 1.2) และแผนวิชาชีพ</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>AITBA2564 หน้า 6; AITBA2569 หน้า 5</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท สาขาวิชาปัญญาประดิษฐ์เพื่อการวิเคราะห์เชิงธุรกิจ คณะเทคโนโลยีสารสนเทศ สจล.  
+- หลักสูตรปี พ.ศ. 2564: แผน ก แบบ ก1, ก2 และแผน ข ต่างกันที่ 36 หน่วยกิตทั้งหมด [6]  
+- หลักสูตรปี พ.ศ. 2569: แผน ก แบบ ก1 (แผน 1.1), ก2 (แผน 1.2) และแผน ข (แผน 2) ยังคงรวม 36 หน่วยกิต [3]  
+ดังนั้น จำนวนหน่วยกิตที่เรียนตลอดหลักสูตร **ไม่แตกต่าง** กันระหว่างหลักสูตร พ.ศ. 2564 และ 2569  
+การเปลี่ยนแปลงชื่อแผนการศึกษา:  
+- แผน ก แบบ ก1 → แผน 1.1 (แบบวิชาการ) [3]  
+- แผน ก แบบ ก2 → แผน 1.2 (แบบวิชาการ) [3]  
+- แผน ข → แผน 2 (แบบวิชาชีพ) [3]  
+[3][6]</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิต 36 เท่ากันถูก แต่ชื่อแผนของ 2569 ยังปนชื่อแบบเดิม (แผน ก/ข)</t>
+        </is>
+      </c>
+      <c r="J15" s="15" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>X8</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>แผนปกติกับแผนสหกิจศึกษาของ DSBA 2565 มีหน่วยกิตรวมตลอดหลักสูตรต่างกันไหม</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ต่าง ทั้งสองแผนรวม 132 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 15, 36</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ต่างกัน  
+แผนปกติและแผนสหกิจศึกษาของหลักสูตรวิทยาศาสตรบัณฑิต สาขาวิชาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ หลักสูตรปรับปรุง พ.ศ. 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากัน คือ 132 หน่วยกิต [7]</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr"/>
+      <c r="J16" s="15" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตร AIT 2566 กับ IT 2565 ต้องเรียนหน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>AIT 2566 = 120, IT 2565 = 129 ต่างกัน 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 5; IT2565 หน้า 6/20</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
+- IT 2565: 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6)
+สรุป: IT 2565 มากกว่า AIT 2566 อยู่ 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr"/>
+      <c r="J17" s="15" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>BIT 2565 กับ DSBA 2560 หลักสูตรไหนต้องเรียนหน่วยกิตรวมมากกว่ากัน</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>เท่ากัน ทั้งคู่ 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>BIT2565 หน้า 6; DSBA2560 หน้า 17</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+- DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
+สรุป: เท่ากัน (126 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr"/>
+      <c r="J18" s="15" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>วิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>ต้องผ่าน 06066001 ความน่าจะเป็นและสถิติ ซึ่งไม่มีวิชาบังคับก่อน (ชั้นเดียว)</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 289, 291</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr"/>
+      <c r="J19" s="15" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนอะไรแทนสหกิจศึกษา กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>กลุ่มวิชาการศึกษาทางเลือก (กลุ่มวิชาเลือก) 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 15, 21-22</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนวิชาเลือกเสรีจำนวนไม่น้อยกว่า 6 หน่วยกิต [4]</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>6 หน่วยกิตถูก แต่เรียกเป็น 'วิชาเลือกเสรี' ซึ่งเป็นคนละกลุ่ม (เล่มเรียกกลุ่มวิชาการศึกษาทางเลือก)</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>AITBA</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>36 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>AITBA2569 หน้า 5</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนไม่น้อยกว่า 36 หน่วยกิต [3]</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr"/>
+      <c r="J21" s="15" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>36 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>IT2568 หน้า 5</t>
+        </is>
+      </c>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนรวมทั้งหมด 36 หน่วยกิต [5]</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr"/>
+      <c r="J22" s="15" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="23" ht="70" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Z1</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>75 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>IT2561 หน้า 16</t>
+        </is>
+      </c>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาเอก สาขาวิชาเทคโนโลยีสารสนเทศ หลักสูตร พ.ศ. 2561 แบบ 1.2 (ผู้เข้าศึกษาที่สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมทั้งสิ้น 75 หน่วยกิต [1]</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr"/>
+      <c r="J23" s="15" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="24" ht="70" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>6 หน่วยกิต (สหกิจศึกษา 06026259 หรือ 06026260 ต่างประเทศ)</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 36</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียน 6 หน่วยกิต [1].</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I24" s="16" t="inlineStr"/>
+      <c r="J24" s="15" t="n">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="25" ht="70" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Z3</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>แผนปกติของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนอะไร กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>วิชาเลือกหมวดศึกษาทั่วไป 1 วิชา + วิชาเลือกเสรี 2 วิชา รวม 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 29</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>ปีที่ 4 ภาคการศึกษาที่ 2 ของแผนปกติหลักสูตร DSBA 2565 เรียนดังนี้:
+- รหัสวิชา: 9064xxxx  
+  ชื่อวิชา: วิชาเลือกหมวดวิชาศึกษาทั่วไป (ELECTIVE IN GENERAL EDUCATION)  
+  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
+- รหัสวิชา: xxxxxxxx  
+  ชื่อวิชา: วิชาเลือกเสรี 1 (FREE ELECTIVE COURSE 1)  
+  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
+รวมทั้งหมด 6 หน่วยกิต [1]</t>
+        </is>
+      </c>
+      <c r="H25" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>ได้วิชาเลือกศึกษาทั่วไป + เลือกเสรี 1 รวม 6 หน่วยกิต แต่ขาดเลือกเสรี 2 (เล่มรวม 9 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="n">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="26" ht="70" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Z4</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>BIT 2565 กับ IT 2565 หน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>BIT 2565 = 126, IT 2565 = 129 ต่างกัน 3 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>BIT2565 หน้า 6; IT2565 หน้า 6</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+- IT 2565: 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6)
+สรุป: IT 2565 มากกว่า BIT 2565 อยู่ 3 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr"/>
+      <c r="J26" s="15" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="27" ht="70" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Z5</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>วิชาพื้นฐานวิทยาการข้อมูลของ AIT ต้องผ่านวิชาอะไรมาก่อน</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มีวิชาบังคับก่อน</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 292</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06046407 พื้นฐานวิทยาการข้อมูล (FUNDAMENTALS OF DATA SCIENCE) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
+  ไม่มีวิชาบังคับก่อน (PREREQUISITE: None)</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr"/>
+      <c r="J27" s="15" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Z6</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาชีพ ต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>36 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>IT2568 หน้า 5</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาชีพต้องเรียนรวมทั้งหมด 36 หน่วยกิต [2]</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="I28" s="16" t="inlineStr"/>
+      <c r="J28" s="15" t="n">
+        <v>0.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(tester): merge 20 extended challenge questions into All Test Cases sheet
Single results tab now holds 48 questions (28 core + X/Y/Z extended set),
with per-set rows and an overall total in the summary. Adds trace and
cited pages to challenge_extended.json; README points to the merged sheet.
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -10,10 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Test Cases &amp; Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenge Criteria (Measured)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenge (extended)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -613,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -928,7 +927,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>รวม</t>
+          <t>รวม (ชุดหลัก)</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
@@ -957,64 +956,200 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>ท้าทายเพิ่มเติม ชุด X</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>ท้าทายเพิ่มเติม ชุด Y</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>0.78</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>ท้าทายเพิ่มเติม ชุด Z</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>1.91</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>รวมทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>ข้อควรทราบเมื่ออ่านผล</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>1) 'ตรวจคำสำคัญ' ผ่านง่าย (เช่น E2 ตรวจแค่มีเลข 3) จึงไม่ควรใช้เป็นอัตราความถูกต้อง ให้ดูคอลัมน์ 'ตรวจโดยคน'</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>2) ผลตรวจโดยคนอ่านเทียบเฉลยในไฟล์นี้ ไม่ได้เทียบกับ PDF ต้นฉบับโดยตรง และผูกกับคำตอบรอบที่ตรวจ (คำถามเชิงเหตุผลเรียก LLM คำตอบเปลี่ยนได้ทุกรอบ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>3) ความถูกต้องของ citation ไม่ได้ตรวจรายข้อในไฟล์นี้ วัดแยกด้วย python -m katrag.eval.qa_eval (19 ข้อ): precision 0.57, recall 0.53</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
+          <t>1) 'ตรวจคำสำคัญ' ผ่านง่าย (เช่น E2 ตรวจแค่มีเลข 3) จึงไม่ควรใช้เป็นอัตราความถูกต้อง ให้ดูคอลัมน์ 'ตรวจโดยคน'</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (เขียนเฉลยจากเล่มก่อนรัน รายงานทุกข้อ) อยู่ในแผ่น Challenge (extended)</t>
+          <t>2) ผลตรวจโดยคนอ่านเทียบเฉลยในไฟล์นี้ ไม่ได้เทียบกับ PDF ต้นฉบับโดยตรง และผูกกับคำตอบรอบที่ตรวจ (คำถามเชิงเหตุผลเรียก LLM คำตอบเปลี่ยนได้ทุกรอบ)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+          <t>3) ความถูกต้องของ citation ไม่ได้ตรวจรายข้อในไฟล์นี้ วัดแยกด้วย python -m katrag.eval.qa_eval (19 ข้อ): precision 0.57, recall 0.53</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (X1–X8, Y1–Y6, Z1–Z6) ต่อท้ายในแผ่น All Test Cases: เขียนคำถามและเฉลยจากเล่มก่อนรัน รายงานทุกข้อที่ลอง ผลบันทึกจากรอบวันที่ 2026-10-04 (docs/challenge_extended.json) ชุด X ใช้ออกแบบการแก้ระบบ ชุด Y/Z เขียนไว้ก่อนแก้แต่ละรอบ (held-out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>6) เฉลยข้อ H4 เดิมเขียน 48 วิชา แต่ฐานข้อมูลปัจจุบันให้ 52 (DSBA 2560 71 ชื่อ / 2565 75 ชื่อ) ผลของระบบตรงกับฐานข้อมูล</t>
         </is>
@@ -1023,22 +1158,22 @@
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A23:H23"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="A24:H24"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="B11:H11"/>
+    <mergeCell ref="A32:H32"/>
     <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1050,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3632,8 +3767,1572 @@
         </is>
       </c>
     </row>
+    <row r="30" ht="80" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>X1</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตรของ DSBA ฉบับ 2560 กับฉบับ 2565 ต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>2560 = 126 หน่วยกิต, 2565 = 132 หน่วยกิต ต่างกัน 6 หน่วยกิต (2565 มากกว่า)</t>
+        </is>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
+- DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
+สรุป: DSBA 2565 มากกว่า DSBA 2560 อยู่ 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2560 หน้า 17; DSBA2565 หน้า 15
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 351, 349, 352; DSBA 2560 หน้า 17)</t>
+        </is>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J30" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K30" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L30" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
+        </is>
+      </c>
+      <c r="N30" s="15" t="inlineStr">
+        <is>
+          <t>0.21s</t>
+        </is>
+      </c>
+      <c r="O30" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="80" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>หลักสูตร BIT 2560 กับ BIT 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากันหรือไม่</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F31" s="20" t="inlineStr">
+        <is>
+          <t>เท่ากัน ทั้งสองฉบับ 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G31" s="20" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- BIT 2560: 126 หน่วยกิต (มคอ.2 BIT 2560 หน้า 17)
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+สรุป: เท่ากัน (126 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H31" s="20" t="inlineStr">
+        <is>
+          <t>BIT2560 หน้า 17; BIT2565 หน้า 6
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 266, 264, 3, 265)</t>
+        </is>
+      </c>
+      <c r="I31" s="20" t="inlineStr">
+        <is>
+          <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J31" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K31" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L31" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M31" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
+        </is>
+      </c>
+      <c r="N31" s="19" t="inlineStr">
+        <is>
+          <t>0.28s</t>
+        </is>
+      </c>
+      <c r="O31" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="80" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>X3</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>ระหว่างหลักสูตร DSBA 2565, AIT 2566 และ BIT 2565 หลักสูตรใดมีหน่วยกิตรวมมากที่สุด</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>DSBA 2565 มากที่สุด 132 หน่วยกิต (BIT 2565 = 126, AIT 2566 = 120)</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
+- AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+สรุป: มากที่สุดคือ DSBA 2565 (132 หน่วยกิต) น้อยที่สุดคือ AIT 2566 (120 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 15; BIT2565 หน้า 6; AIT2566 หน้า 5
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 78; DSBA 2565 หน้า 352, 349; BIT 2565 หน้า 264)</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J32" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L32" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
+        </is>
+      </c>
+      <c r="N32" s="15" t="inlineStr">
+        <is>
+          <t>0.37s</t>
+        </is>
+      </c>
+      <c r="O32" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="80" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>X4</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>ในแผนสหกิจศึกษาของ DSBA 2565 ต้องลงทะเบียนวิชาสหกิจศึกษาในภาคไหน และกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F33" s="20" t="inlineStr">
+        <is>
+          <t>ปีที่ 4 ภาคการศึกษาที่ 2 จำนวน 6 หน่วยกิต (06026259 สหกิจศึกษา หรือ 06026260 สหกิจศึกษาต่างประเทศ)</t>
+        </is>
+      </c>
+      <c r="G33" s="20" t="inlineStr">
+        <is>
+          <t>นักศึกษาต้องลงทะเบียนวิชาสหกิจศึกษา 6 หน่วยกิตในภาคการศึกษาที่ 3 หรือภาคการศึกษาที่ 4 ของปีที่ 3 หรือปีที่ 4 ตามลำดับ [5]</t>
+        </is>
+      </c>
+      <c r="H33" s="20" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 36
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 30, 23, 354, 15)</t>
+        </is>
+      </c>
+      <c r="I33" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J33" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="K33" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>ผิด</t>
+        </is>
+      </c>
+      <c r="M33" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ตอบว่าลงสหกิจภาค 3/ภาค 4 ของปี 3/ปี 4 แต่เล่มหน้า 36 คือปี 4 ภาค 2</t>
+        </is>
+      </c>
+      <c r="N33" s="19" t="inlineStr">
+        <is>
+          <t>1.02s</t>
+        </is>
+      </c>
+      <c r="O33" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="80" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>X5</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท IT 2563 กับ 2568 แบ่งแผนการศึกษาต่างกันอย่างไร</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>2563: แผน ก (แบบ ก1, ก2) และแผน ข; 2568: แผน 1 แบบวิชาการ (แบบ 1.1, 1.2) และแผน 2 แบบวิชาชีพ; ทุกแผนเรียน 36 หน่วยกิตเท่ากัน</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2563 (IT 2563) มีแผนการศึกษาแบบ ก 1 และ ก 2 ซึ่งรับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ตั้งแต่ปีการศึกษา 2563 ถึง 2567 โดยแผน ก 1 และ ก 2 มีโครงสร้างการรับนักศึกษาและคาดการณ์การสำเร็จการศึกษาเหมือนกัน คือ รับ 5 คนต่อปี ชั้นปีที่ 1 และสำเร็จการศึกษา 5 คนต่อปี ตั้งแต่ปีการศึกษา 2564 เป็นต้นไป [3]
+ส่วนหลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2568 (IT 2568) มีแผนการศึกษา 3 แบบ ได้แก่ แผน 1 แบบวิชาการ แบบ 1.1, แบบ 1.2 และแผน 2 แบบวิชาชีพ โดยแผน 1 แบบวิชาการ รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ตั้งแต่ปีการศึกษา 2568 เป็นต้นไป คาดว่าจะสำเร็จการศึกษา 3 คนต่อปี ตั้งแต่ปีการศึกษา 2569 เป็นต้นไป ส่วนแผน 2 แบบวิชาชีพ รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ตั้งแต่ปีการศึกษา 2568 เป็นต้นไป คาดว่าจะสำเร็จการศึกษา 30 คนต่อปี ตั้งแต่ปีการศึกษา 2569 เป็นต้นไป [2]
+ดังนั้น ความแตกต่างคือ หลักสูตร 2563 มีเพียงแผน ก 1 และ ก 2 รับคนละ 5 คนต่อปี ส่วนหลักสูตร 2568 มีแผนมากกว่า 3 แบบ โดยมีการแบ่งแยกตามประเภทการศึกษา (วิชาการ/วิชาชีพ) และจำนวนรับนักศึกษาต่อปีแตกต่างกันอย่างชัดเจน [2][3]</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>IT2563 หน้า 16; IT2568 หน้า 5
+(หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 153, 11; วท.ม. IT 2563 หน้า 15)</t>
+        </is>
+      </c>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] อธิบายแผนของ 2568 ถูก แต่ของ 2563 ขาดแผน ข และตอบจำนวนรับนักศึกษาแทนโครงสร้างแผน</t>
+        </is>
+      </c>
+      <c r="N34" s="15" t="inlineStr">
+        <is>
+          <t>4.10s</t>
+        </is>
+      </c>
+      <c r="O34" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="80" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>X6</t>
+        </is>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D35" s="20" t="inlineStr">
+        <is>
+          <t>ถ้าจะเรียนวิชาพื้นฐานการเรียนรู้เชิงลึก (Fundamentals of Deep Learning) ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
+        </is>
+      </c>
+      <c r="E35" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F35" s="20" t="inlineStr">
+        <is>
+          <t>ต้องผ่านแคลคูลัส 2 (06046401) และพีชคณิตเชิงเส้น (06046402); แคลคูลัส 2 ต้องผ่านแคลคูลัส 1 (06046400) ก่อน; พีชคณิตเชิงเส้นและแคลคูลัส 1 ไม่มีวิชาบังคับก่อน</t>
+        </is>
+      </c>
+      <c r="G35" s="20" t="inlineStr">
+        <is>
+          <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06046401 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
+      ↳ ต้องผ่าน 06046400 แคลคูลัส 1 (CALCULUS 1) ก่อน
+    • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H35" s="20" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 287-288
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 37, 292, 19, 20)</t>
+        </is>
+      </c>
+      <c r="I35" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J35" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="K35" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M35" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ไล่วิชาบังคับก่อน 2 ชั้นได้ครบ</t>
+        </is>
+      </c>
+      <c r="N35" s="19" t="inlineStr">
+        <is>
+          <t>0.31s</t>
+        </is>
+      </c>
+      <c r="O35" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="80" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>X7</t>
+        </is>
+      </c>
+      <c r="B36" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>AITBA</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท AITBA 2564 กับ 2569 หน่วยกิตที่เรียนตลอดหลักสูตรต่างกันไหม และชื่อแผนการศึกษาเปลี่ยนไปอย่างไร</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตไม่ต่าง ทุกแผน 36 หน่วยกิต; 2564 ใช้แผน ก (ก1, ก2) และแผน ข; 2569 ใช้แผนวิชาการ (แบบ 1.1, 1.2) และแผนวิชาชีพ</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท สาขาวิชาปัญญาประดิษฐ์เพื่อการวิเคราะห์เชิงธุรกิจ คณะเทคโนโลยีสารสนเทศ สจล.  
+- หลักสูตรปี พ.ศ. 2564: แผน ก แบบ ก1, ก2 และแผน ข ต่างกันที่ 36 หน่วยกิตทั้งหมด [6]  
+- หลักสูตรปี พ.ศ. 2569: แผน ก แบบ ก1 (แผน 1.1), ก2 (แผน 1.2) และแผน ข (แผน 2) ยังคงรวม 36 หน่วยกิต [3]  
+ดังนั้น จำนวนหน่วยกิตที่เรียนตลอดหลักสูตร **ไม่แตกต่าง** กันระหว่างหลักสูตร พ.ศ. 2564 และ 2569  
+การเปลี่ยนแปลงชื่อแผนการศึกษา:  
+- แผน ก แบบ ก1 → แผน 1.1 (แบบวิชาการ) [3]  
+- แผน ก แบบ ก2 → แผน 1.2 (แบบวิชาการ) [3]  
+- แผน ข → แผน 2 (แบบวิชาชีพ) [3]  
+[3][6]</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>AITBA2564 หน้า 6; AITBA2569 หน้า 5
+(หน้าที่ระบบคืนมา: ปร.ด. AITBA 2569 หน้า 223, 99, 225, 167; วท.ม. AITBA 2564 หน้า 6, 3)</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J36" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] หน่วยกิต 36 เท่ากันถูก แต่ชื่อแผนของ 2569 ยังปนชื่อแบบเดิม (แผน ก/ข)</t>
+        </is>
+      </c>
+      <c r="N36" s="15" t="inlineStr">
+        <is>
+          <t>2.47s</t>
+        </is>
+      </c>
+      <c r="O36" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="80" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>X8</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>แผนปกติกับแผนสหกิจศึกษาของ DSBA 2565 มีหน่วยกิตรวมตลอดหลักสูตรต่างกันไหม</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F37" s="20" t="inlineStr">
+        <is>
+          <t>ไม่ต่าง ทั้งสองแผนรวม 132 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G37" s="20" t="inlineStr">
+        <is>
+          <t>ไม่ต่างกัน  
+แผนปกติและแผนสหกิจศึกษาของหลักสูตรวิทยาศาสตรบัณฑิต สาขาวิชาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ หลักสูตรปรับปรุง พ.ศ. 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากัน คือ 132 หน่วยกิต [7]</t>
+        </is>
+      </c>
+      <c r="H37" s="20" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 15, 36
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 351, 30, 349, 23)</t>
+        </is>
+      </c>
+      <c r="I37" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J37" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="K37" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M37" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
+        </is>
+      </c>
+      <c r="N37" s="19" t="inlineStr">
+        <is>
+          <t>0.96s</t>
+        </is>
+      </c>
+      <c r="O37" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="80" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตร AIT 2566 กับ IT 2565 ต้องเรียนหน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>AIT 2566 = 120, IT 2565 = 129 ต่างกัน 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
+- IT 2565: 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6)
+สรุป: IT 2565 มากกว่า AIT 2566 อยู่ 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 5; IT2565 หน้า 6/20
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 369, 378, 371; AIT 2566 หน้า 78)</t>
+        </is>
+      </c>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J38" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K38" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
+        </is>
+      </c>
+      <c r="N38" s="15" t="inlineStr">
+        <is>
+          <t>0.34s</t>
+        </is>
+      </c>
+      <c r="O38" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="80" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="inlineStr">
+        <is>
+          <t>BIT 2565 กับ DSBA 2560 หลักสูตรไหนต้องเรียนหน่วยกิตรวมมากกว่ากัน</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F39" s="20" t="inlineStr">
+        <is>
+          <t>เท่ากัน ทั้งคู่ 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G39" s="20" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+- DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
+สรุป: เท่ากัน (126 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H39" s="20" t="inlineStr">
+        <is>
+          <t>BIT2565 หน้า 6; DSBA2560 หน้า 17
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 266, 264, 267, 265)</t>
+        </is>
+      </c>
+      <c r="I39" s="20" t="inlineStr">
+        <is>
+          <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J39" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="K39" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L39" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M39" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
+        </is>
+      </c>
+      <c r="N39" s="19" t="inlineStr">
+        <is>
+          <t>0.28s</t>
+        </is>
+      </c>
+      <c r="O39" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="80" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>วิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>ต้องผ่าน 06066001 ความน่าจะเป็นและสถิติ ซึ่งไม่มีวิชาบังคับก่อน (ชั้นเดียว)</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 289, 291
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 37, 291, 19, 20)</t>
+        </is>
+      </c>
+      <c r="I40" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J40" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K40" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
+        </is>
+      </c>
+      <c r="N40" s="15" t="inlineStr">
+        <is>
+          <t>0.20s</t>
+        </is>
+      </c>
+      <c r="O40" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="80" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="inlineStr">
+        <is>
+          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนอะไรแทนสหกิจศึกษา กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E41" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F41" s="20" t="inlineStr">
+        <is>
+          <t>กลุ่มวิชาการศึกษาทางเลือก (กลุ่มวิชาเลือก) 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G41" s="20" t="inlineStr">
+        <is>
+          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนวิชาเลือกเสรีจำนวนไม่น้อยกว่า 6 หน่วยกิต [4]</t>
+        </is>
+      </c>
+      <c r="H41" s="20" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 15, 21-22
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 30, 23, 15, 22)</t>
+        </is>
+      </c>
+      <c r="I41" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J41" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="K41" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="M41" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2] 6 หน่วยกิตถูก แต่เรียกเป็น 'วิชาเลือกเสรี' ซึ่งเป็นคนละกลุ่ม (เล่มเรียกกลุ่มวิชาการศึกษาทางเลือก)</t>
+        </is>
+      </c>
+      <c r="N41" s="19" t="inlineStr">
+        <is>
+          <t>0.78s</t>
+        </is>
+      </c>
+      <c r="O41" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="80" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>AITBA</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>36 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนไม่น้อยกว่า 36 หน่วยกิต [3]</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="inlineStr">
+        <is>
+          <t>AITBA2569 หน้า 5
+(หน้าที่ระบบคืนมา: ปร.ด. AITBA 2569 หน้า 100, 5, 15, 228; วท.ม. AITBA 2569 หน้า 228, 21)</t>
+        </is>
+      </c>
+      <c r="I42" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J42" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="K42" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
+        </is>
+      </c>
+      <c r="N42" s="15" t="inlineStr">
+        <is>
+          <t>0.73s</t>
+        </is>
+      </c>
+      <c r="O42" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="80" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E43" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F43" s="20" t="inlineStr">
+        <is>
+          <t>36 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G43" s="20" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนรวมทั้งหมด 36 หน่วยกิต [5]</t>
+        </is>
+      </c>
+      <c r="H43" s="20" t="inlineStr">
+        <is>
+          <t>IT2568 หน้า 5
+(หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 155, 25, 74, 18)</t>
+        </is>
+      </c>
+      <c r="I43" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J43" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="K43" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L43" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M43" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
+        </is>
+      </c>
+      <c r="N43" s="19" t="inlineStr">
+        <is>
+          <t>0.68s</t>
+        </is>
+      </c>
+      <c r="O43" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="80" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>Z1</t>
+        </is>
+      </c>
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>75 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาเอก สาขาวิชาเทคโนโลยีสารสนเทศ หลักสูตร พ.ศ. 2561 แบบ 1.2 (ผู้เข้าศึกษาที่สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมทั้งสิ้น 75 หน่วยกิต [1]</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>IT2561 หน้า 16
+(หน้าที่ระบบคืนมา: ปร.ด. IT 2561 หน้า 16, 38, 22, 131)</t>
+        </is>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J44" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="K44" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
+        </is>
+      </c>
+      <c r="N44" s="15" t="inlineStr">
+        <is>
+          <t>0.88s</t>
+        </is>
+      </c>
+      <c r="O44" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="80" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
+        </is>
+      </c>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="inlineStr">
+        <is>
+          <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E45" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F45" s="20" t="inlineStr">
+        <is>
+          <t>6 หน่วยกิต (สหกิจศึกษา 06026259 หรือ 06026260 ต่างประเทศ)</t>
+        </is>
+      </c>
+      <c r="G45" s="20" t="inlineStr">
+        <is>
+          <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียน 6 หน่วยกิต [1].</t>
+        </is>
+      </c>
+      <c r="H45" s="20" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 36
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36, 29, 350, 14)</t>
+        </is>
+      </c>
+      <c r="I45" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J45" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M45" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
+        </is>
+      </c>
+      <c r="N45" s="19" t="inlineStr">
+        <is>
+          <t>0.61s</t>
+        </is>
+      </c>
+      <c r="O45" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="80" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>Z3</t>
+        </is>
+      </c>
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>แผนปกติของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนอะไร กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>วิชาเลือกหมวดศึกษาทั่วไป 1 วิชา + วิชาเลือกเสรี 2 วิชา รวม 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>ปีที่ 4 ภาคการศึกษาที่ 2 ของแผนปกติหลักสูตร DSBA 2565 เรียนดังนี้:
+- รหัสวิชา: 9064xxxx  
+  ชื่อวิชา: วิชาเลือกหมวดวิชาศึกษาทั่วไป (ELECTIVE IN GENERAL EDUCATION)  
+  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
+- รหัสวิชา: xxxxxxxx  
+  ชื่อวิชา: วิชาเลือกเสรี 1 (FREE ELECTIVE COURSE 1)  
+  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
+รวมทั้งหมด 6 หน่วยกิต [1]</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>DSBA2565 หน้า 29
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36, 14, 29)</t>
+        </is>
+      </c>
+      <c r="I46" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J46" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K46" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)] ได้วิชาเลือกศึกษาทั่วไป + เลือกเสรี 1 รวม 6 หน่วยกิต แต่ขาดเลือกเสรี 2 (เล่มรวม 9 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="N46" s="15" t="inlineStr">
+        <is>
+          <t>1.91s</t>
+        </is>
+      </c>
+      <c r="O46" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="80" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>Z4</t>
+        </is>
+      </c>
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
+        <is>
+          <t>BIT 2565 กับ IT 2565 หน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F47" s="20" t="inlineStr">
+        <is>
+          <t>BIT 2565 = 126, IT 2565 = 129 ต่างกัน 3 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G47" s="20" t="inlineStr">
+        <is>
+          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
+- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
+- IT 2565: 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6)
+สรุป: IT 2565 มากกว่า BIT 2565 อยู่ 3 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H47" s="20" t="inlineStr">
+        <is>
+          <t>BIT2565 หน้า 6; IT2565 หน้า 6
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 264, 266, 7)</t>
+        </is>
+      </c>
+      <c r="I47" s="20" t="inlineStr">
+        <is>
+          <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J47" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M47" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
+        </is>
+      </c>
+      <c r="N47" s="19" t="inlineStr">
+        <is>
+          <t>0.43s</t>
+        </is>
+      </c>
+      <c r="O47" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="80" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>Z5</t>
+        </is>
+      </c>
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>วิชาพื้นฐานวิทยาการข้อมูลของ AIT ต้องผ่านวิชาอะไรมาก่อน</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มีวิชาบังคับก่อน</t>
+        </is>
+      </c>
+      <c r="G48" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06046407 พื้นฐานวิทยาการข้อมูล (FUNDAMENTALS OF DATA SCIENCE) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
+  ไม่มีวิชาบังคับก่อน (PREREQUISITE: None)</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>AIT2566 หน้า 292
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 20, 24, 38, 292)</t>
+        </is>
+      </c>
+      <c r="I48" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J48" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K48" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
+        </is>
+      </c>
+      <c r="N48" s="15" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O48" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="80" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>Z6</t>
+        </is>
+      </c>
+      <c r="B49" s="24" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาชีพ ต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
+        </is>
+      </c>
+      <c r="F49" s="20" t="inlineStr">
+        <is>
+          <t>36 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G49" s="20" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาชีพต้องเรียนรวมทั้งหมด 36 หน่วยกิต [2]</t>
+        </is>
+      </c>
+      <c r="H49" s="20" t="inlineStr">
+        <is>
+          <t>IT2568 หน้า 5
+(หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 25, 12, 156, 14)</t>
+        </is>
+      </c>
+      <c r="I49" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J49" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="K49" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M49" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
+        </is>
+      </c>
+      <c r="N49" s="19" t="inlineStr">
+        <is>
+          <t>0.48s</t>
+        </is>
+      </c>
+      <c r="O49" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O29"/>
+  <autoFilter ref="A1:O49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3729,1120 +5428,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ข้อท้าทายเพิ่มเติม — บันทึกจากการรันวันที่ 2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>เขียนคำถามและเฉลยจากเล่ม มคอ.2 ก่อนรัน แล้วรายงานทุกข้อที่ลอง (ไม่คัดทิ้ง)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ชุด X (8 ข้อ) — ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>ผลล่าสุด: ถูกครบ 5 · บางส่วน 2 · ผิด 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>ชุด Y (6 ข้อ) — เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>ผลล่าสุด: ถูกครบ 5 · บางส่วน 1 · ผิด 0  (รอบที่ 1 วัดได้ ถูกครบ 3/6 (Y4, Y5, Y6 ผิด) ก่อนแก้รอบที่ 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>ชุด Z (6 ข้อ) — เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>ผลล่าสุด: ถูกครบ 5 · บางส่วน 1 · ผิด 0  (รอบที่ 2 วัดครั้งแรก ถูกครบ 5/6 (Z3 ผิด))</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>ข้อที่</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>ชุด</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>หลักสูตร</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>คำถาม</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>เฉลย (จากเล่ม)</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>หน้าที่มาของเฉลย</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>คำตอบจริงจากเซิร์ฟเวอร์</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="inlineStr">
-        <is>
-          <t>ตรวจโดยคน</t>
-        </is>
-      </c>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>หมายเหตุ</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="inlineStr">
-        <is>
-          <t>เวลาตอบ (s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>X1</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>DSBA</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตรของ DSBA ฉบับ 2560 กับฉบับ 2565 ต่างกันกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>2560 = 126 หน่วยกิต, 2565 = 132 หน่วยกิต ต่างกัน 6 หน่วยกิต (2565 มากกว่า)</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2560 หน้า 17; DSBA2565 หน้า 15</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
-- DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
-- DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
-สรุป: DSBA 2565 มากกว่า DSBA 2560 อยู่ 6 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I9" s="16" t="inlineStr"/>
-      <c r="J9" s="15" t="n">
-        <v>0.21</v>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>X2</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>BIT</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตร BIT 2560 กับ BIT 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากันหรือไม่</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>เท่ากัน ทั้งสองฉบับ 126 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>BIT2560 หน้า 17; BIT2565 หน้า 6</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
-- BIT 2560: 126 หน่วยกิต (มคอ.2 BIT 2560 หน้า 17)
-- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
-สรุป: เท่ากัน (126 หน่วยกิต)</t>
-        </is>
-      </c>
-      <c r="H10" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr"/>
-      <c r="J10" s="15" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>X3</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>AIT</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>ระหว่างหลักสูตร DSBA 2565, AIT 2566 และ BIT 2565 หลักสูตรใดมีหน่วยกิตรวมมากที่สุด</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>DSBA 2565 มากที่สุด 132 หน่วยกิต (BIT 2565 = 126, AIT 2566 = 120)</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2565 หน้า 15; BIT2565 หน้า 6; AIT2566 หน้า 5</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
-- DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
-- AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
-- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
-สรุป: มากที่สุดคือ DSBA 2565 (132 หน่วยกิต) น้อยที่สุดคือ AIT 2566 (120 หน่วยกิต)</t>
-        </is>
-      </c>
-      <c r="H11" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I11" s="16" t="inlineStr"/>
-      <c r="J11" s="15" t="n">
-        <v>0.37</v>
-      </c>
-    </row>
-    <row r="12" ht="70" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>X4</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>DSBA</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>ในแผนสหกิจศึกษาของ DSBA 2565 ต้องลงทะเบียนวิชาสหกิจศึกษาในภาคไหน และกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>ปีที่ 4 ภาคการศึกษาที่ 2 จำนวน 6 หน่วยกิต (06026259 สหกิจศึกษา หรือ 06026260 สหกิจศึกษาต่างประเทศ)</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2565 หน้า 36</t>
-        </is>
-      </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>นักศึกษาต้องลงทะเบียนวิชาสหกิจศึกษา 6 หน่วยกิตในภาคการศึกษาที่ 3 หรือภาคการศึกษาที่ 4 ของปีที่ 3 หรือปีที่ 4 ตามลำดับ [5]</t>
-        </is>
-      </c>
-      <c r="H12" s="25" t="inlineStr">
-        <is>
-          <t>ผิด</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
-        <is>
-          <t>ตอบว่าลงสหกิจภาค 3/ภาค 4 ของปี 3/ปี 4 แต่เล่มหน้า 36 คือปี 4 ภาค 2</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="n">
-        <v>1.02</v>
-      </c>
-    </row>
-    <row r="13" ht="70" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>X5</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท IT 2563 กับ 2568 แบ่งแผนการศึกษาต่างกันอย่างไร</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>2563: แผน ก (แบบ ก1, ก2) และแผน ข; 2568: แผน 1 แบบวิชาการ (แบบ 1.1, 1.2) และแผน 2 แบบวิชาชีพ; ทุกแผนเรียน 36 หน่วยกิตเท่ากัน</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>IT2563 หน้า 16; IT2568 หน้า 5</t>
-        </is>
-      </c>
-      <c r="G13" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2563 (IT 2563) มีแผนการศึกษาแบบ ก 1 และ ก 2 ซึ่งรับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ตั้งแต่ปีการศึกษา 2563 ถึง 2567 โดยแผน ก 1 และ ก 2 มีโครงสร้างการรับนักศึกษาและคาดการณ์การสำเร็จการศึกษาเหมือนกัน คือ รับ 5 คนต่อปี ชั้นปีที่ 1 และสำเร็จการศึกษา 5 คนต่อปี ตั้งแต่ปีการศึกษา 2564 เป็นต้นไป [3]
-ส่วนหลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2568 (IT 2568) มีแผนการศึกษา 3 แบบ ได้แก่ แผน 1 แบบวิชาการ แบบ 1.1, แบบ 1.2 และแผน 2 แบบวิชาชีพ โดยแผน 1 แบบวิชาการ รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ตั้งแต่ปีการศึกษา 2568 เป็นต้นไป คาดว่าจะสำเร็จการศึกษา 3 คนต่อปี ตั้งแต่ปีการศึกษา 2569 เป็นต้นไป ส่วนแผน 2 แบบวิชาชีพ รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ตั้งแต่ปีการศึกษา 2568 เป็นต้นไป คาดว่าจะสำเร็จการศึกษา 30 คนต่อปี ตั้งแต่ปีการศึกษา 2569 เป็นต้นไป [2]
-ดังนั้น ความแตกต่างคือ หลักสูตร 2563 มีเพียงแผน ก 1 และ ก 2 รับคนละ 5 คนต่อปี ส่วนหลักสูตร 2568 มีแผนมากกว่า 3 แบบ โดยมีการแบ่งแยกตามประเภทการศึกษา (วิชาการ/วิชาชีพ) และจำนวนรับนักศึกษาต่อปีแตกต่างกันอย่างชัดเจน [2][3]</t>
-        </is>
-      </c>
-      <c r="H13" s="23" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
-        </is>
-      </c>
-      <c r="I13" s="16" t="inlineStr">
-        <is>
-          <t>อธิบายแผนของ 2568 ถูก แต่ของ 2563 ขาดแผน ข และตอบจำนวนรับนักศึกษาแทนโครงสร้างแผน</t>
-        </is>
-      </c>
-      <c r="J13" s="15" t="n">
-        <v>4.1</v>
-      </c>
-    </row>
-    <row r="14" ht="70" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>X6</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>AIT</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>ถ้าจะเรียนวิชาพื้นฐานการเรียนรู้เชิงลึก (Fundamentals of Deep Learning) ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>ต้องผ่านแคลคูลัส 2 (06046401) และพีชคณิตเชิงเส้น (06046402); แคลคูลัส 2 ต้องผ่านแคลคูลัส 1 (06046400) ก่อน; พีชคณิตเชิงเส้นและแคลคูลัส 1 ไม่มีวิชาบังคับก่อน</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>AIT2566 หน้า 287-288</t>
-        </is>
-      </c>
-      <c r="G14" s="16" t="inlineStr">
-        <is>
-          <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
-  ต้องผ่านวิชาบังคับก่อน:
-    • 06046401 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
-      ↳ ต้องผ่าน 06046400 แคลคูลัส 1 (CALCULUS 1) ก่อน
-    • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
-        </is>
-      </c>
-      <c r="H14" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I14" s="16" t="inlineStr">
-        <is>
-          <t>ไล่วิชาบังคับก่อน 2 ชั้นได้ครบ</t>
-        </is>
-      </c>
-      <c r="J14" s="15" t="n">
-        <v>0.31</v>
-      </c>
-    </row>
-    <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>X7</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>AITBA</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท AITBA 2564 กับ 2569 หน่วยกิตที่เรียนตลอดหลักสูตรต่างกันไหม และชื่อแผนการศึกษาเปลี่ยนไปอย่างไร</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตไม่ต่าง ทุกแผน 36 หน่วยกิต; 2564 ใช้แผน ก (ก1, ก2) และแผน ข; 2569 ใช้แผนวิชาการ (แบบ 1.1, 1.2) และแผนวิชาชีพ</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>AITBA2564 หน้า 6; AITBA2569 หน้า 5</t>
-        </is>
-      </c>
-      <c r="G15" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท สาขาวิชาปัญญาประดิษฐ์เพื่อการวิเคราะห์เชิงธุรกิจ คณะเทคโนโลยีสารสนเทศ สจล.  
-- หลักสูตรปี พ.ศ. 2564: แผน ก แบบ ก1, ก2 และแผน ข ต่างกันที่ 36 หน่วยกิตทั้งหมด [6]  
-- หลักสูตรปี พ.ศ. 2569: แผน ก แบบ ก1 (แผน 1.1), ก2 (แผน 1.2) และแผน ข (แผน 2) ยังคงรวม 36 หน่วยกิต [3]  
-ดังนั้น จำนวนหน่วยกิตที่เรียนตลอดหลักสูตร **ไม่แตกต่าง** กันระหว่างหลักสูตร พ.ศ. 2564 และ 2569  
-การเปลี่ยนแปลงชื่อแผนการศึกษา:  
-- แผน ก แบบ ก1 → แผน 1.1 (แบบวิชาการ) [3]  
-- แผน ก แบบ ก2 → แผน 1.2 (แบบวิชาการ) [3]  
-- แผน ข → แผน 2 (แบบวิชาชีพ) [3]  
-[3][6]</t>
-        </is>
-      </c>
-      <c r="H15" s="23" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
-        </is>
-      </c>
-      <c r="I15" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิต 36 เท่ากันถูก แต่ชื่อแผนของ 2569 ยังปนชื่อแบบเดิม (แผน ก/ข)</t>
-        </is>
-      </c>
-      <c r="J15" s="15" t="n">
-        <v>2.47</v>
-      </c>
-    </row>
-    <row r="16" ht="70" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>X8</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>DSBA</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>แผนปกติกับแผนสหกิจศึกษาของ DSBA 2565 มีหน่วยกิตรวมตลอดหลักสูตรต่างกันไหม</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>ไม่ต่าง ทั้งสองแผนรวม 132 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2565 หน้า 15, 36</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>ไม่ต่างกัน  
-แผนปกติและแผนสหกิจศึกษาของหลักสูตรวิทยาศาสตรบัณฑิต สาขาวิชาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ หลักสูตรปรับปรุง พ.ศ. 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากัน คือ 132 หน่วยกิต [7]</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I16" s="16" t="inlineStr"/>
-      <c r="J16" s="15" t="n">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="17" ht="70" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>AIT</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตร AIT 2566 กับ IT 2565 ต้องเรียนหน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>AIT 2566 = 120, IT 2565 = 129 ต่างกัน 9 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>AIT2566 หน้า 5; IT2565 หน้า 6/20</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
-- AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
-- IT 2565: 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6)
-สรุป: IT 2565 มากกว่า AIT 2566 อยู่ 9 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I17" s="16" t="inlineStr"/>
-      <c r="J17" s="15" t="n">
-        <v>0.34</v>
-      </c>
-    </row>
-    <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>BIT</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>BIT 2565 กับ DSBA 2560 หลักสูตรไหนต้องเรียนหน่วยกิตรวมมากกว่ากัน</t>
-        </is>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
-        <is>
-          <t>เท่ากัน ทั้งคู่ 126 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>BIT2565 หน้า 6; DSBA2560 หน้า 17</t>
-        </is>
-      </c>
-      <c r="G18" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
-- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
-- DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
-สรุป: เท่ากัน (126 หน่วยกิต)</t>
-        </is>
-      </c>
-      <c r="H18" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I18" s="16" t="inlineStr"/>
-      <c r="J18" s="15" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>Y3</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>AIT</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>วิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>ต้องผ่าน 06066001 ความน่าจะเป็นและสถิติ ซึ่งไม่มีวิชาบังคับก่อน (ชั้นเดียว)</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>AIT2566 หน้า 289, 291</t>
-        </is>
-      </c>
-      <c r="G19" s="16" t="inlineStr">
-        <is>
-          <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
-  ต้องผ่านวิชาบังคับก่อน:
-    • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
-        </is>
-      </c>
-      <c r="H19" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I19" s="16" t="inlineStr"/>
-      <c r="J19" s="15" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>Y4</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>DSBA</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนอะไรแทนสหกิจศึกษา กี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>กลุ่มวิชาการศึกษาทางเลือก (กลุ่มวิชาเลือก) 6 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2565 หน้า 15, 21-22</t>
-        </is>
-      </c>
-      <c r="G20" s="16" t="inlineStr">
-        <is>
-          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนวิชาเลือกเสรีจำนวนไม่น้อยกว่า 6 หน่วยกิต [4]</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
-        </is>
-      </c>
-      <c r="I20" s="16" t="inlineStr">
-        <is>
-          <t>6 หน่วยกิตถูก แต่เรียกเป็น 'วิชาเลือกเสรี' ซึ่งเป็นคนละกลุ่ม (เล่มเรียกกลุ่มวิชาการศึกษาทางเลือก)</t>
-        </is>
-      </c>
-      <c r="J20" s="15" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="21" ht="70" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Y5</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>AITBA</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพต้องเรียนกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>36 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>AITBA2569 หน้า 5</t>
-        </is>
-      </c>
-      <c r="G21" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนไม่น้อยกว่า 36 หน่วยกิต [3]</t>
-        </is>
-      </c>
-      <c r="H21" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I21" s="16" t="inlineStr"/>
-      <c r="J21" s="15" t="n">
-        <v>0.73</v>
-      </c>
-    </row>
-    <row r="22" ht="70" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Y6</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>36 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>IT2568 หน้า 5</t>
-        </is>
-      </c>
-      <c r="G22" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนรวมทั้งหมด 36 หน่วยกิต [5]</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I22" s="16" t="inlineStr"/>
-      <c r="J22" s="15" t="n">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="23" ht="70" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>Z1</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>75 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>IT2561 หน้า 16</t>
-        </is>
-      </c>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาเอก สาขาวิชาเทคโนโลยีสารสนเทศ หลักสูตร พ.ศ. 2561 แบบ 1.2 (ผู้เข้าศึกษาที่สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมทั้งสิ้น 75 หน่วยกิต [1]</t>
-        </is>
-      </c>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I23" s="16" t="inlineStr"/>
-      <c r="J23" s="15" t="n">
-        <v>0.88</v>
-      </c>
-    </row>
-    <row r="24" ht="70" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Z2</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>DSBA</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>6 หน่วยกิต (สหกิจศึกษา 06026259 หรือ 06026260 ต่างประเทศ)</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2565 หน้า 36</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="inlineStr">
-        <is>
-          <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียน 6 หน่วยกิต [1].</t>
-        </is>
-      </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I24" s="16" t="inlineStr"/>
-      <c r="J24" s="15" t="n">
-        <v>0.61</v>
-      </c>
-    </row>
-    <row r="25" ht="70" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Z3</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>DSBA</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>แผนปกติของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนอะไร กี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>วิชาเลือกหมวดศึกษาทั่วไป 1 วิชา + วิชาเลือกเสรี 2 วิชา รวม 9 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>DSBA2565 หน้า 29</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="inlineStr">
-        <is>
-          <t>ปีที่ 4 ภาคการศึกษาที่ 2 ของแผนปกติหลักสูตร DSBA 2565 เรียนดังนี้:
-- รหัสวิชา: 9064xxxx  
-  ชื่อวิชา: วิชาเลือกหมวดวิชาศึกษาทั่วไป (ELECTIVE IN GENERAL EDUCATION)  
-  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
-- รหัสวิชา: xxxxxxxx  
-  ชื่อวิชา: วิชาเลือกเสรี 1 (FREE ELECTIVE COURSE 1)  
-  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
-รวมทั้งหมด 6 หน่วยกิต [1]</t>
-        </is>
-      </c>
-      <c r="H25" s="23" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
-        </is>
-      </c>
-      <c r="I25" s="16" t="inlineStr">
-        <is>
-          <t>ได้วิชาเลือกศึกษาทั่วไป + เลือกเสรี 1 รวม 6 หน่วยกิต แต่ขาดเลือกเสรี 2 (เล่มรวม 9 หน่วยกิต)</t>
-        </is>
-      </c>
-      <c r="J25" s="15" t="n">
-        <v>1.91</v>
-      </c>
-    </row>
-    <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Z4</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>BIT</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>BIT 2565 กับ IT 2565 หน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>BIT 2565 = 126, IT 2565 = 129 ต่างกัน 3 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>BIT2565 หน้า 6; IT2565 หน้า 6</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
-          <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
-- BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
-- IT 2565: 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6)
-สรุป: IT 2565 มากกว่า BIT 2565 อยู่ 3 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="H26" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I26" s="16" t="inlineStr"/>
-      <c r="J26" s="15" t="n">
-        <v>0.43</v>
-      </c>
-    </row>
-    <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>Z5</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>AIT</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
-        <is>
-          <t>วิชาพื้นฐานวิทยาการข้อมูลของ AIT ต้องผ่านวิชาอะไรมาก่อน</t>
-        </is>
-      </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>ไม่มีวิชาบังคับก่อน</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>AIT2566 หน้า 292</t>
-        </is>
-      </c>
-      <c r="G27" s="16" t="inlineStr">
-        <is>
-          <t>วิชา 06046407 พื้นฐานวิทยาการข้อมูล (FUNDAMENTALS OF DATA SCIENCE) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
-  ไม่มีวิชาบังคับก่อน (PREREQUISITE: None)</t>
-        </is>
-      </c>
-      <c r="H27" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I27" s="16" t="inlineStr"/>
-      <c r="J27" s="15" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>Z6</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท IT 2568 แผนวิชาชีพ ต้องเรียนกี่หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>36 หน่วยกิต</t>
-        </is>
-      </c>
-      <c r="F28" s="16" t="inlineStr">
-        <is>
-          <t>IT2568 หน้า 5</t>
-        </is>
-      </c>
-      <c r="G28" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท IT 2568 แผนวิชาชีพต้องเรียนรวมทั้งหมด 36 หน่วยกิต [2]</t>
-        </is>
-      </c>
-      <c r="H28" s="18" t="inlineStr">
-        <is>
-          <t>ถูกครบ</t>
-        </is>
-      </c>
-      <c r="I28" s="16" t="inlineStr"/>
-      <c r="J28" s="15" t="n">
-        <v>0.48</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(query): category-credit rules and co-op/normal plan tables read from the book
- rule table: 89 verified category-credit rows (general ed / specific / free
  elective and sub-groups) for DSBA/IT/BIT/AIT current and DSBA/IT/BIT 2560;
  every value is checked against the cited page text before it is stored
- plan_variants: read the 3.1.4.1 and 3.1.4.2 plan tables from page text;
  per-semester totals of both plans sum to the course total for all six books
- intents: category credits, normal vs co-op plan, per-semester load (now plan
  aware), graduation audit for programs other than DSBA; structured answers
  carry their own page citations
- tester: 82 questions re-recorded (adds W1-W10); C3 judged against the book,
  its answer key is inconsistent with the book; README results updated
- database archive regenerated; qa_eval citation precision 0.60, recall 0.52
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenge Criteria (Measured)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -128,14 +128,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00FFF7ED"/>
+        <bgColor rgb="00FFF7ED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7ED"/>
-        <bgColor rgb="00FFF7ED"/>
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -232,10 +232,10 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>28 ข้อชุดหลัก (E1–E9, M1–M9, H1–H7, C1–C3) + 24 ข้อชุดเพิ่มระดับง่าย/ปานกลาง/ยาก (E10–H15) + 20 ข้อท้าทายเพิ่มเติม (X1–Z6) = 72 ข้อ</t>
+          <t>28 ข้อชุดหลัก (E1–E9, M1–M9, H1–H7, C1–C3) + 34 ข้อชุดเพิ่มระดับง่าย/ปานกลาง/ยาก (E10–H15) + 20 ข้อท้าทายเพิ่มเติม (X1–Z6) = 82 ข้อ</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>27/28 ข้อ — เกณฑ์หลวม (บางข้อตรวจแค่มีตัวเลข) ไม่ใช่การยืนยันว่าถูก</t>
+          <t>28/28 ข้อ — เกณฑ์หลวม (บางข้อตรวจแค่มีตัวเลข) ไม่ใช่การยืนยันว่าถูก</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ถูกครบ 23 · ถูกบางส่วน 4 · ผิด/ไม่ตรงเฉลย 1 · ยังไม่ได้ตรวจ 0</t>
+          <t>ถูกครบ 25 · ถูกบางส่วน 3 · ผิด/ไม่ตรงเฉลย 0 · ยังไม่ได้ตรวจ 0</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>เฉลี่ย 1.28s · เร็วสุด 0.06s · ช้าสุด 8.48s · ต่ำกว่า 5s 26/28 ข้อ</t>
+          <t>เฉลี่ย 0.92s · เร็วสุด 0.05s · ช้าสุด 9.03s · ต่ำกว่า 5s 27/28 ข้อ</t>
         </is>
       </c>
     </row>
@@ -819,12 +819,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.16</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
         <v>9</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>0.61</t>
         </is>
       </c>
     </row>
@@ -883,12 +883,12 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>3.90</t>
+          <t>4.86</t>
         </is>
       </c>
     </row>
@@ -902,25 +902,25 @@
         <v>3</v>
       </c>
       <c r="C19" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" s="8" t="n">
         <v>2</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>1</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>5.09</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>8.48</t>
+          <t>9.03</t>
         </is>
       </c>
     </row>
@@ -934,25 +934,25 @@
         <v>28</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>8.48</t>
+          <t>9.03</t>
         </is>
       </c>
     </row>
@@ -981,12 +981,12 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>0.32</t>
+          <t>0.38</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.85</t>
         </is>
       </c>
     </row>
@@ -1015,12 +1015,12 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>0.72</t>
         </is>
       </c>
     </row>
@@ -1039,33 +1039,33 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>4.32</t>
+          <t>0.26</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>ท้าทายเพิ่มเติม ชุด X</t>
+          <t>ชุดใหม่ W1–W10 (โครงสร้างหน่วยกิต/แผนสหกิจ)</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
@@ -1073,33 +1073,33 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>9.63</t>
+          <t>0.36</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>ท้าทายเพิ่มเติม ชุด Y</t>
+          <t>ท้าทายเพิ่มเติม ชุด X</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>1</v>
@@ -1117,19 +1117,19 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>2.42</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>12.81</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>ท้าทายเพิ่มเติม ชุด Z</t>
+          <t>ท้าทายเพิ่มเติม ชุด Y</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
@@ -1141,145 +1141,186 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>0.51</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>3.89</t>
+          <t>1.16</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>ท้าทายเพิ่มเติม ชุด Z</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>0.54</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>1.27</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>รวมทั้งหมด</t>
         </is>
       </c>
-      <c r="B27" s="10" t="n">
-        <v>72</v>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
+      <c r="B28" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D27" s="10" t="n">
-        <v>58</v>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="F27" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>9.63</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="D28" s="10" t="n">
+        <v>74</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>0.74</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>12.81</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>ข้อควรทราบเมื่ออ่านผล</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>1) 'ตรวจคำสำคัญ' ผ่านง่าย (เช่น E2 ตรวจแค่มีเลข 3) จึงไม่ควรใช้เป็นอัตราความถูกต้อง ให้ดูคอลัมน์ 'ตรวจโดยคน'</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>2) ผลตรวจโดยคนอ่านเทียบเฉลยในไฟล์นี้ ไม่ได้เทียบกับ PDF ต้นฉบับโดยตรง และผูกกับคำตอบรอบที่ตรวจ (คำถามเชิงเหตุผลเรียก LLM คำตอบเปลี่ยนได้ทุกรอบ)</t>
+          <t>1) 'ตรวจคำสำคัญ' ผ่านง่าย (เช่น E2 ตรวจแค่มีเลข 3) จึงไม่ควรใช้เป็นอัตราความถูกต้อง ให้ดูคอลัมน์ 'ตรวจโดยคน'</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>3) ความถูกต้องของ citation ไม่ได้ตรวจรายข้อในไฟล์นี้ วัดแยกด้วย python -m katrag.eval.qa_eval (19 ข้อ): precision 0.57, recall 0.53</t>
+          <t>2) ผลตรวจโดยคนอ่านเทียบเฉลยในไฟล์นี้ ไม่ได้เทียบกับ PDF ต้นฉบับโดยตรง และผูกกับคำตอบรอบที่ตรวจ (คำถามเชิงเหตุผลเรียก LLM คำตอบเปลี่ยนได้ทุกรอบ)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
+          <t>3) ความถูกต้องของ citation ไม่ได้ตรวจรายข้อในไฟล์นี้ วัดแยกด้วย python -m katrag.eval.qa_eval (19 ข้อ): precision 0.57, recall 0.53</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
+          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (X1–X8, Y1–Y6, Z1–Z6) ต่อท้ายในแผ่น All Test Cases: เขียนคำถามและเฉลยจากเล่มก่อนรัน รายงานทุกข้อที่ลอง ผลบันทึกจากรอบวันที่ 2026-10-05 (docs/challenge_extended.json) ชุด X ใช้ออกแบบการแก้ระบบ ชุด Y/Z เขียนไว้ก่อนแก้แต่ละรอบ (held-out)</t>
+          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>4.3) ชุดเพิ่มระดับง่าย/ปานกลาง/ยาก 24 ข้อ (E10–E17, M10–M17, H8–H15, docs/extra_levels.json): เขียนคำถามแล้วตรวจเฉลยจากเล่มหลังรัน รอบแรกได้ ถูก 14 · ไม่ตรงประเด็น 4 · ผิด 6 จึงแก้ระบบแล้วรันซ้ำทั้งหมด ผลในไฟล์นี้คือรอบหลังแก้ ชุดนี้ใช้นำการแก้ ไม่ใช่ชุด held-out และข้อ H15 (วิชาเลือกตามแขนง) ยังไม่ได้แก้</t>
+          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (X1–X8, Y1–Y6, Z1–Z6) ต่อท้ายในแผ่น All Test Cases: เขียนคำถามและเฉลยจากเล่มก่อนรัน รายงานทุกข้อที่ลอง ผลบันทึกจากรอบวันที่ 2026-10-05 (docs/challenge_extended.json) ชุด X ใช้ออกแบบการแก้ระบบ ชุด Y/Z เขียนไว้ก่อนแก้แต่ละรอบ (held-out)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>4.4) หลังแก้ระบบ รัน 28 ข้อชุดหลักซ้ำ ข้อที่ตอบจากตาราง SQL ได้คำตอบเหมือนเดิมทุกตัวอักษร ข้อที่ผ่าน LLM ตอบเปลี่ยน จึงตรวจใหม่: M8 ลดจาก ถูกครบ เป็น ถูกบางส่วน (ตอบ 12 ถูก แต่เรียก 6 ผิดชื่อ) และข้อ X7 เพิ่มจาก ถูกบางส่วน เป็น ถูกครบ</t>
+          <t>4.3) ชุดเพิ่มระดับง่าย/ปานกลาง/ยาก 24 ข้อ (E10–E17, M10–M17, H8–H15, docs/extra_levels.json): เขียนคำถามแล้วตรวจเฉลยจากเล่มหลังรัน รอบแรกได้ ถูก 14 · ไม่ตรงประเด็น 4 · ผิด 6 จึงแก้ระบบแล้วรันซ้ำ ผลในไฟล์นี้คือรอบหลังแก้ ชุดนี้ใช้นำการแก้ ไม่ใช่ชุด held-out ข้อ H15 (วิชาเลือกตามแขนง) ยังไม่ได้แก้</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+          <t>4.4) การแก้รอบหลัง (ตารางโครงสร้างหน่วยกิตรายหมวด + อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) แล้วรันซ้ำทั้งหมด: ข้อที่ตอบจาก SQL ได้คำตอบเดิม ข้อที่ผ่าน LLM ตอบเปลี่ยนจึงตรวจใหม่ M8 และ H5 ตอนนี้ตอบจากตาราง rule (M8 เป็น ถูกครบ ตอบคงที่) C3 ตอบจากตารางแผนสหกิจ (ถูกครบ ตรวจกับเล่ม: เฉลยเดิมของ C3 คลาดเคลื่อน โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน) ข้อ X4, X8, Y4, Z3, H11 เปลี่ยนเป็น ถูกครบ ส่วน X7 ถูกครบ/X5 ถูกบางส่วน เป็นผลของ LLM ที่เปลี่ยนไปตามรอบ</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
+          <t>4.5) ชุดใหม่ W1–W10 (โครงสร้างหน่วยกิตรายหมวด + แผนสหกิจ) เขียนคำถามและเฉลยจากเล่มก่อนรัน รอบแรกได้ ถูกครบ 8 · บางส่วน 2 (W9 ระบุภาคที่ต่างเกินจริงเพราะเรียงแถวต่างกัน, W10 ตารางขาดปี 3 ภาค 2) แก้แบบทั่วไป (ไม่เขียนตอบเฉพาะข้อ) แล้วรันซ้ำ ผลในไฟล์คือรอบหลังแก้ จึงไม่ใช่ชุดที่ซ่อนไว้วัดอย่างสะอาด</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
           <t>6) เฉลยข้อ H4 เดิมเขียน 48 วิชา แต่ฐานข้อมูลปัจจุบันให้ 52 (DSBA 2560 71 ชื่อ / 2565 75 ชื่อ) ผลของระบบตรงกับฐานข้อมูล</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A30:H30"/>
+  <mergeCells count="20">
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="A36:H36"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B4:H4"/>
+    <mergeCell ref="A41:H41"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="B12:H12"/>
@@ -1288,10 +1329,11 @@
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A34:H34"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1303,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O73"/>
+  <dimension ref="A1:O83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1484,7 +1526,7 @@
       </c>
       <c r="N2" s="15" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O2" s="18" t="inlineStr">
@@ -1565,7 +1607,7 @@
       </c>
       <c r="N3" s="19" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O3" s="18" t="inlineStr">
@@ -1644,7 +1686,7 @@
       </c>
       <c r="N4" s="15" t="inlineStr">
         <is>
-          <t>0.09s</t>
+          <t>0.19s</t>
         </is>
       </c>
       <c r="O4" s="18" t="inlineStr">
@@ -1739,7 +1781,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="O5" s="18" t="inlineStr">
@@ -1781,7 +1823,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>ชื่อวิชาภาษาอังกฤษของ "ระบบข้อมูลมหัต" คือ **Big Data Systems** [4]</t>
+          <t>ระบบข้อมูลมหัต (Big Data Systems) [4]</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -1815,7 +1857,7 @@
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>1.31s</t>
+          <t>1.16s</t>
         </is>
       </c>
       <c r="O6" s="18" t="inlineStr">
@@ -1907,7 +1949,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="O7" s="18" t="inlineStr">
@@ -1985,7 +2027,7 @@
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>0.09s</t>
+          <t>0.15s</t>
         </is>
       </c>
       <c r="O8" s="18" t="inlineStr">
@@ -2070,7 +2112,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.41s</t>
         </is>
       </c>
       <c r="O9" s="18" t="inlineStr">
@@ -2226,7 +2268,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.05s</t>
         </is>
       </c>
       <c r="O11" s="18" t="inlineStr">
@@ -2311,7 +2353,7 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.46s</t>
         </is>
       </c>
       <c r="O12" s="18" t="inlineStr">
@@ -2400,7 +2442,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>0.64s</t>
+          <t>0.61s</t>
         </is>
       </c>
       <c r="O13" s="18" t="inlineStr">
@@ -2491,7 +2533,7 @@
       </c>
       <c r="N14" s="15" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.56s</t>
         </is>
       </c>
       <c r="O14" s="18" t="inlineStr">
@@ -2596,7 +2638,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.41s</t>
         </is>
       </c>
       <c r="O15" s="18" t="inlineStr">
@@ -2691,7 +2733,7 @@
       </c>
       <c r="N16" s="15" t="inlineStr">
         <is>
-          <t>0.07s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O16" s="18" t="inlineStr">
@@ -2818,41 +2860,61 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) หมวดวิชาเฉพาะมีการเก็บหน่วยกิตจากกลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต [7] และมีวิชาเลือกเสรี 6 หน่วยกิต [4] รวมเป็นกลุ่มวิชาเฉพาะด้านทั้งหมด 18 หน่วยกิต แต่หากพิจารณาเฉพาะ "กลุ่มวิชาชีพเฉพาะด้าน" ซึ่งเป็นกลุ่มที่เก็บหน่วยกิตโดยตรงตามคำถาม คือ 12 หน่วยกิต [7].</t>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร DSBA 2565 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ กลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต (เลือกลงทะเบียนกลุ่มใดกลุ่มหนึ่ง รวม 12 หน่วยกิต) — หน้า 15
+▶ กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6) — หน้า 15
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต
+    - กลุ่มวิชาพื้นฐาน 6 หน่วยกิต
+    - กลุ่มวิชาด้านภาษาและการสื่อสาร 9 หน่วยกิต
+    - กลุ่มวิชาตามเกณฑ์ของคณะ 9 หน่วยกิต
+    - กลุ่มวิชาเลือกหมวดวิชาการศึกษาทั่วไป 6 หน่วยกิต
+  - หมวดวิชาเฉพาะ 96 หน่วยกิต
+    - กลุ่มวิชาแกน 45 หน่วยกิต
+      - กลุ่มคณิตศาสตร์และสถิติ 15 หน่วยกิต
+      - กลุ่มเทคโนโลยีสารสนเทศ 30 หน่วยกิต
+    - กลุ่มพื้นฐานวิชาชีพ 33 หน่วยกิต
+    - กลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต ◀
+      - กลุ่มวิทยาการข้อมูล 12 หน่วยกิต
+      - กลุ่มการวิเคราะห์เชิงสถิติ 12 หน่วยกิต
+      - กลุ่มวิศวกรรมข้อมูล 12 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต ◀
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต
+หน่วยกิตรวมตลอดหลักสูตร 132 หน่วยกิต</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
           <t>โครงสร้างหลักสูตร DSBA 2565 (หน้า 15)
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 349, 352, 7, 351)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 15)</t>
         </is>
       </c>
       <c r="I18" s="16" t="inlineStr">
         <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J18" s="15" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K18" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L18" s="22" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M18" s="16" t="inlineStr">
         <is>
-          <t>ตอบ 12 หน่วยกิต (กลุ่มวิชาชีพเฉพาะด้าน) ถูก แต่เรียก 6 หน่วยกิตว่า 'วิชาเลือกเสรี' (ในเล่มคือกลุ่มวิชาการศึกษาทางเลือก) แล้วรวมเป็น 18 ซึ่งไม่มีในเล่ม ข้อนี้ผ่าน LLM ตอบไม่คงที่ (ถามซ้ำ 8 รอบ ได้ 12 ในคำตอบ 5 ครั้ง)</t>
+          <t>ตอบจากตาราง rule (โครงสร้างหลักสูตร DSBA 2565 หน้า 15): กลุ่มวิชาชีพเฉพาะด้าน 12 และกลุ่มวิชาการศึกษาทางเลือก 6 ตรงเฉลย ตอบคงที่ทุกรอบเพราะไม่ผ่าน LLM (ก่อนหน้านี้ผ่าน LLM ตอบ 12 ได้แค่ 5 ครั้งจาก 8)</t>
         </is>
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>3.30s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O18" s="18" t="inlineStr">
@@ -2932,7 +2994,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.05s</t>
         </is>
       </c>
       <c r="O19" s="18" t="inlineStr">
@@ -2947,7 +3009,7 @@
           <t>H1</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3061,7 +3123,7 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L20" s="22" t="inlineStr">
+      <c r="L20" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
@@ -3073,7 +3135,7 @@
       </c>
       <c r="N20" s="15" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O20" s="18" t="inlineStr">
@@ -3088,7 +3150,7 @@
           <t>H2</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3116,7 +3178,7 @@
       <c r="G21" s="20" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถเรียนวิชาที่เกี่ยวข้องกับฐานข้อมูลในปีที่ 4 ได้ เนื่องจากมีวิชาบังคับก่อนหน้าที่เกี่ยวข้อง เช่น 06066300 แนวคิดระบบฐานข้อมูล (ปี 2 ภาค 1) และ 06026212 การสร้างคลังข้อมูล (ปี 3 ภาค 1) ซึ่งเป็นพื้นฐานสำคัญ นอกจากนี้ ยังมีวิชาเลือกในกลุ่มวิชาศึกษาทั่วไปและวิชาเลือกเสรีที่อาจครอบคลุมเนื้อหาด้านฐานข้อมูลได้ โดยไม่มีข้อห้ามในการเรียนวิชาด้านฐานข้อมูลในปีที่ 4 ตามหลักสูตร DSBA 2565.</t>
+นักศึกษาสามารถเรียนวิชาฐานข้อมูลในปีที่ 4 ได้ เนื่องจากหลักสูตร DSBA 2565 มีวิชาบังคับในปีที่ 4 ที่เกี่ยวข้องกับฐานข้อมูล เช่น 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 ซึ่งจัดสอนในภาคการศึกษาที่ 1 ปีที่ 4 โดยไม่มีวิชาบังคับก่อนกำหนดไว้ และมีอาจารย์ผู้สอนที่เชี่ยวชาญด้านฐานข้อมูล ได้แก่ รศ.ดร.ศุภมิตร จิตตะยโศธร ผู้มีงานวิจัยและภาระงานสอนด้านฐานข้อมูลระบบข้อมูลขั้นสูง</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -3138,19 +3200,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L21" s="22" t="inlineStr">
+      <c r="L21" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
       </c>
       <c r="M21" s="20" t="inlineStr">
         <is>
-          <t>ตอบ 'ได้' ถูก แต่ไม่ได้ชี้วิชาฐานข้อมูลที่เปิดปี 4 จริง (06026246) ยกวิชาปี 2-3 ขึ้นมาแทน และอ้างว่าวิชาเลือกอาจครอบคลุมฐานข้อมูลโดยไม่มีหลักฐาน</t>
+          <t>ตอบ 'ได้' ถูก ชี้ 06026246/06026247 (หัวข้อพิเศษทางวิศวกรรมข้อมูล) และภาค 1 ตรงเฉลย แต่เรียกว่า 'วิชาบังคับ' (เป็นวิชาเลือก) และอ้างอาจารย์ที่เชี่ยวชาญฐานข้อมูลโดยไม่มีหลักฐานรองรับ ข้อนี้ผ่าน LLM ตอบเปลี่ยนทุกรอบ (รอบก่อนระบุภาค 2 และ 6 หน่วยกิตผิด)</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>3.90s</t>
+          <t>4.86s</t>
         </is>
       </c>
       <c r="O21" s="18" t="inlineStr">
@@ -3165,7 +3227,7 @@
           <t>H3</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3193,7 +3255,7 @@
       <c r="G22" s="16" t="inlineStr">
         <is>
           <t>ไม่ได้  
-วิชา 06026212 การสร้างคลังข้อมูล (DATA WAREHOUSING) เป็นวิชาบังคับในปีที่ 3 ภาคการศึกษาที่ 1 และมีข้อกำหนดให้ต้องผ่านวิชาบังคับก่อนอย่างน้อย 06066300 แนวคิดระบบฐานข้อมูล ซึ่งจัดสอนในปีที่ 2 ภาคการศึกษาที่ 1 ดังนั้นจึงไม่สามารถลงวิชานี้ได้ในปีที่ 2</t>
+วิชา 06026212 การสร้างคลังข้อมูล เป็นวิชาบังคับที่ต้องเรียนในปีที่ 3 ภาคการศึกษาที่ 1 และมีข้อกำหนดให้ต้องผ่านวิชา 06066300 แนวคิดระบบฐานข้อมูล ซึ่งเป็นวิชาบังคับในปีที่ 2 ภาคการศึกษาที่ 1 ก่อนจึงจะสามารถลงทะเบียนได้</t>
         </is>
       </c>
       <c r="H22" s="16" t="inlineStr">
@@ -3227,7 +3289,7 @@
       </c>
       <c r="N22" s="15" t="inlineStr">
         <is>
-          <t>3.14s</t>
+          <t>3.05s</t>
         </is>
       </c>
       <c r="O22" s="18" t="inlineStr">
@@ -3242,7 +3304,7 @@
           <t>H4</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3385,7 +3447,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="O23" s="18" t="inlineStr">
@@ -3400,7 +3462,7 @@
           <t>H5</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3427,22 +3489,42 @@
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>หลักสูตรวิทยาศาสตรบัณฑิต สาขาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) หมวดวิชาเฉพาะที่เกี่ยวข้องกับกลุ่มวิชาชีพเฉพาะด้าน (หรือวิชาชีพเลือก) มีจำนวน 12 หน่วยกิต [7].</t>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร DSBA 2565 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ กลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต (เลือกลงทะเบียนกลุ่มใดกลุ่มหนึ่ง รวม 12 หน่วยกิต) — หน้า 15
+▶ กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6) — หน้า 15
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต
+    - กลุ่มวิชาพื้นฐาน 6 หน่วยกิต
+    - กลุ่มวิชาด้านภาษาและการสื่อสาร 9 หน่วยกิต
+    - กลุ่มวิชาตามเกณฑ์ของคณะ 9 หน่วยกิต
+    - กลุ่มวิชาเลือกหมวดวิชาการศึกษาทั่วไป 6 หน่วยกิต
+  - หมวดวิชาเฉพาะ 96 หน่วยกิต
+    - กลุ่มวิชาแกน 45 หน่วยกิต
+      - กลุ่มคณิตศาสตร์และสถิติ 15 หน่วยกิต
+      - กลุ่มเทคโนโลยีสารสนเทศ 30 หน่วยกิต
+    - กลุ่มพื้นฐานวิชาชีพ 33 หน่วยกิต
+    - กลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต ◀
+      - กลุ่มวิทยาการข้อมูล 12 หน่วยกิต
+      - กลุ่มการวิเคราะห์เชิงสถิติ 12 หน่วยกิต
+      - กลุ่มวิศวกรรมข้อมูล 12 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต ◀
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต
+หน่วยกิตรวมตลอดหลักสูตร 132 หน่วยกิต</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
         <is>
           <t>โครงสร้างหลักสูตร DSBA 2565 (หน้า 15)
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 349, 351, 352, 7)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 15)</t>
         </is>
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J24" s="15" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
@@ -3456,12 +3538,12 @@
       </c>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>ตอบ 12 หน่วยกิต (กลุ่มวิชาชีพเฉพาะด้าน) ถูก ผ่าน retrieval + LLM</t>
+          <t>ตอบจากตาราง rule: กลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต และแยกกลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิตเป็นคนละกลุ่ม ตรงเฉลย</t>
         </is>
       </c>
       <c r="N24" s="15" t="inlineStr">
         <is>
-          <t>2.05s</t>
+          <t>0.24s</t>
         </is>
       </c>
       <c r="O24" s="18" t="inlineStr">
@@ -3476,7 +3558,7 @@
           <t>H6</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3503,9 +3585,9 @@
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>ใช่ หลักสูตร DSBA ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า กลุ่มวิชา) ซึ่งแบ่งออกเป็น 3 กลุ่ม ได้แก่:
+          <t>ใช่ ปีที่ 3 ต้องเลือกแขนง (หรือที่เรียกว่า กลุ่มวิชา) ซึ่งมี 3 แขนงให้เลือก ได้แก่:
 - วิทยาการข้อมูล (Data Science)  
-- การวิเคราะห์เชิงสถิติ (Statistical Analytics)  
+- การวิเคราะห์เชิงสถิติ (Statistical Analysis)  
 - วิศวกรรมข้อมูล (Data Engineering)  
 [3][4][6]</t>
         </is>
@@ -3541,7 +3623,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>2.58s</t>
+          <t>2.46s</t>
         </is>
       </c>
       <c r="O25" s="18" t="inlineStr">
@@ -3556,7 +3638,7 @@
           <t>H7</t>
         </is>
       </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="B26" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก</t>
         </is>
@@ -3627,7 +3709,7 @@
       </c>
       <c r="N26" s="15" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="O26" s="18" t="inlineStr">
@@ -3669,9 +3751,9 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือก "แขนงวิชา"  
-2. หลักสูตร IT 2565 ลดหน่วยกิตกลุ่มวิชาเฉพาะด้านจาก 46 หน่วยกิต (IT 2560) เป็น 57 หน่วยกิต แต่เพิ่มหน่วยกิตกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศจาก 6 เป็น 9 หน่วยกิต โดยจัดเป็น 3 โมดูลอาชีพ: Full-Stack Web Developer, Network/System Engineer, Game Developer ซึ่งไม่บังคับเลือกทั้งหมด แต่สามารถเลือกได้เสรี หรือเลือกหลายโมดูล  
-3. อ้างข้อมูลจาก: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18, IT 2565 หน้า 6), โครงสร้างหลักสูตร (มคอ.2 IT 2565 หน้า 371, 374, 376, 378), กลุ่มวิชาเลือก (IT 2565 หน้า 378), กลุ่มวิชาบังคับเฉพาะสาขา (IT 2565 หน้า 376), กลุ่มวิชาเฉพาะด้าน (IT 2565 หน้า 374), ประเภทวิชา (บังคับ/เลือก) และการปรับโครงสร้าง (IT 2565 หน้า 370)</t>
+          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือกแขนงวิชาเดิม
+2. หลักสูตร IT 2565 ปรับลดหน่วยกิตรวมจาก 130 เหลือ 129 หน่วยกิต โดยลดหน่วยกิตในกลุ่มวิชาเฉพาะด้านจาก 94 เป็น 93 หน่วยกิต และลดหน่วยกิตกลุ่มวิชาบังคับเฉพาะแขนงจาก 30 เป็น 15 หน่วยกิต พร้อมเพิ่มกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศเป็น 9 หน่วยกิต (จากเดิม 6 หน่วยกิต) ซึ่งจัดเป็น 3 โมดูลอาชีพ ได้แก่ Full-Stack Web Developer, Network/System Engineer และ Game Developer
+3. อ้างข้อมูลจาก: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18, IT 2565 หน้า 6), โครงสร้างหลักสูตร (มคอ.2 IT 2565 หน้า 371, 374, 376, 378), คำอธิบายการปรับโครงสร้าง (มคอ.2 IT 2565 หน้า 370) — ประเภทวิชา: บังคับ/เลือก, ภาค/ปีที่เปิดสอน: ปีการศึกษา 2560 (IT 2560), 2565 (IT 2565)</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">
@@ -3693,19 +3775,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L27" s="22" t="inlineStr">
+      <c r="L27" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
       </c>
       <c r="M27" s="20" t="inlineStr">
         <is>
-          <t>หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย และมีประโยค 'ลดหน่วยกิตกลุ่มวิชาเฉพาะด้านจาก 46 เป็น 57' ที่ขัดกันเอง (ตัวเลขย่อยมาจาก LLM ยังไม่ได้ยืนยันกับเล่ม)</t>
+          <t>หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่ามี 3 แขนง) ตัวเลขย่อยรอบนี้ (เฉพาะด้าน 94→93, บังคับเฉพาะแขนง 30→15, เลือก IT 6→9) ตรงกับโครงสร้างในเล่ม ข้อนี้ผ่าน LLM ตัวเลขย่อยเปลี่ยนทุกรอบ (รอบก่อนมีประโยคที่ขัดกันเอง)</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>8.48s</t>
+          <t>9.03s</t>
         </is>
       </c>
       <c r="O27" s="15" t="inlineStr">
@@ -3787,7 +3869,7 @@
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.38s</t>
         </is>
       </c>
       <c r="O28" s="18" t="inlineStr">
@@ -3829,48 +3911,80 @@
       </c>
       <c r="G29" s="20" t="inlineStr">
         <is>
-          <t>1. หลักสูตร DSBA 2565 แผนปกติ (ไม่ทำสหกิจ) และแผนสหกิจศึกษา มีความแตกต่างกันในภาคการศึกษาที่ 3 ปีที่ 3 เป็นต้นไป โดยแผนสหกิจศึกษาต้องเรียนวิชาสหกิจศึกษา (06026259) 6 หน่วยกิต ซึ่งไม่มีในแผนปกติ
-2. แผนสหกิจศึกษาต้องเรียนวิชาสหกิจศึกษา (06026259) 6 หน่วยกิต ซึ่งเป็นวิชาบังคับก่อนไม่มี (PREREQUISITE: None) และเปิดสอนในภาคการศึกษาที่ 3 ปีที่ 3 หรือตามกำหนดระยะเวลาอย่างน้อย 16 สัปดาห์ ตามข้อมูลในหน้า 341 และ 354 ของหลักสูตร DSBA 2565
-3. วิชาที่ต่างกันคือ 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (6 หน่วยกิต) ประเภทวิชาบังคับ ภาคการศึกษาที่ 3 ปีที่ 3 หรือตามกำหนดเวลาปฏิบัติงานอย่างน้อย 16 สัปดาห์</t>
+          <t>เปรียบเทียบแผนการศึกษา DSBA 2565 (ปริญญาตรี): แผนปกติ (3.1.4.1) กับแผนที่เข้าโครงการสหกิจศึกษา (3.1.4.2)
+- ปีที่ 1 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 1 ภาคการศึกษาที่ 2: แผนปกติ 21 หน่วยกิต · แผนสหกิจ 21 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 2: แผนปกติ 21 หน่วยกิต · แผนสหกิจ 21 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 2: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 4 ภาคการศึกษาที่ 1: แผนปกติ 9 หน่วยกิต · แผนสหกิจ 12 หน่วยกิต  ← ต่างกัน
+- ปีที่ 4 ภาคการศึกษาที่ 2: แผนปกติ 9 หน่วยกิต · แผนสหกิจ 6 หน่วยกิต  ← ต่างกัน
+รวมตลอดหลักสูตร: แผนปกติ 132 หน่วยกิต · แผนสหกิจ 132 หน่วยกิต (เท่ากัน)
+ภาคที่ต่างกัน: ปี 4 ภาค 1, ปี 4 ภาค 2
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 29):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 2 ช่อง
+      • วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 1
+      • วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 36):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 29):
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36):
+  - 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  - 06026260 สหกิจศึกษาต่างประเทศทางวิทยาการข้อมูลและการ วิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต
+ตามโครงสร้างหลักสูตร: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6)</t>
         </is>
       </c>
       <c r="H29" s="20" t="inlineStr">
         <is>
           <t>แผนการศึกษาเปรียบเทียบ DSBA 2565 (หน้า 15–17)
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 30, 350, 23, 15)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29, 36)</t>
         </is>
       </c>
       <c r="I29" s="20" t="inlineStr">
         <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="K29" s="15" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L29" s="25" t="inlineStr">
-        <is>
-          <t>ผิด</t>
+        <v>2</v>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L29" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M29" s="20" t="inlineStr">
         <is>
-          <t>ตอบว่าแผนสหกิจต่างที่ปี 3 ภาค 3 แต่เล่ม (DSBA 2565 หน้า 36) วางสหกิจศึกษา 06026259/06026260 ไว้ที่ปี 4 ภาค 2 หมายเหตุ: เฉลยในไฟล์ทดสอบใช้รหัส 06026245 ซึ่งไม่ตรงกับเล่ม และแผนปกติปี 4 ภาค 2 ในเล่ม (หน้า 29) คือวิชาเลือกศึกษาทั่วไป + เลือกเสรี 2 วิชา รวม 9 หน่วยกิต ไม่ใช่โครงงาน 2</t>
+          <t>ตอบจากตารางแผนทั้งสองชุดในเล่ม (3.1.4.1 หน้า 23-29 และ 3.1.4.2 หน้า 30-36): ต่างกันที่ปี 4 ภาค 1 (ปกติ 9 / สหกิจ 12) และปี 4 ภาค 2 (ปกติ 9 / สหกิจศึกษา 06026259 6 หน่วยกิต) รวม 132 เท่ากัน ตรวจกับเล่มแล้ว หมายเหตุ: เฉลยในไฟล์ทดสอบเขียนว่าแผนปกติลงโครงงาน 2 ในปี 4 ภาค 2 และใช้รหัสสหกิจ 06026245 ซึ่งไม่ตรงเล่ม (โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน, รหัสสหกิจคือ 06026259/06026260)</t>
         </is>
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>6.47s</t>
-        </is>
-      </c>
-      <c r="O29" s="15" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O29" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -3937,7 +4051,7 @@
       <c r="M30" s="16" t="inlineStr"/>
       <c r="N30" s="15" t="inlineStr">
         <is>
-          <t>0.52s</t>
+          <t>0.59s</t>
         </is>
       </c>
       <c r="O30" s="18" t="inlineStr">
@@ -4014,7 +4128,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>0.09s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="O31" s="18" t="inlineStr">
@@ -4089,7 +4203,7 @@
       <c r="M32" s="16" t="inlineStr"/>
       <c r="N32" s="15" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="O32" s="18" t="inlineStr">
@@ -4181,7 +4295,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.16s</t>
         </is>
       </c>
       <c r="O33" s="18" t="inlineStr">
@@ -4273,7 +4387,7 @@
       </c>
       <c r="N34" s="15" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="O34" s="18" t="inlineStr">
@@ -4354,7 +4468,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.42s</t>
         </is>
       </c>
       <c r="O35" s="18" t="inlineStr">
@@ -4431,7 +4545,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L36" s="22" t="inlineStr">
+      <c r="L36" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
@@ -4443,7 +4557,7 @@
       </c>
       <c r="N36" s="15" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.44s</t>
         </is>
       </c>
       <c r="O36" s="18" t="inlineStr">
@@ -4515,7 +4629,7 @@
       <c r="M37" s="20" t="inlineStr"/>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>0.80s</t>
+          <t>0.85s</t>
         </is>
       </c>
       <c r="O37" s="18" t="inlineStr">
@@ -4594,7 +4708,7 @@
       </c>
       <c r="N38" s="15" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="O38" s="18" t="inlineStr">
@@ -4637,12 +4751,14 @@
       <c r="G39" s="20" t="inlineStr">
         <is>
           <t>วิชาที่เกี่ยวข้องกับ "machine learning" — หลักสูตร AIT
-■ AIT 2566 — 6 วิชา รวม 18 หน่วยกิต
+■ AIT 2566 — 7 วิชา รวม 21 หน่วยกิต
   - 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING)
       หน่วยกิต 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   - 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING)
       หน่วยกิต 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   - 06046414 การประมวลผลภาษาธรรมชาติด้วยการเรียนรู้เชิงลึก (NATURAL LANGUAGE PROCESSING WITH DEEP LEARNING)
+      หน่วยกิต 3(3-0-6) | ปีที่ 3 ภาคการศึกษาที่ 1
+  - 06046415 การประมวลผลสัญญาณ (SIGNAL PROCESSING)
       หน่วยกิต 3(3-0-6) | ปีที่ 3 ภาคการศึกษาที่ 1
   - 06046416 การเรียนรู้เชิงลึกสำหรับคอมพิวเตอร์วิทัศน์ (DEEP LEARNING FOR COMPUTER VISION)
       หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
@@ -4671,7 +4787,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L39" s="22" t="inlineStr">
+      <c r="L39" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
@@ -4683,7 +4799,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>0.54s</t>
+          <t>0.68s</t>
         </is>
       </c>
       <c r="O39" s="18" t="inlineStr">
@@ -4796,7 +4912,7 @@
       </c>
       <c r="N40" s="15" t="inlineStr">
         <is>
-          <t>0.61s</t>
+          <t>0.55s</t>
         </is>
       </c>
       <c r="O40" s="18" t="inlineStr">
@@ -4889,7 +5005,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>0.67s</t>
+          <t>0.72s</t>
         </is>
       </c>
       <c r="O41" s="18" t="inlineStr">
@@ -4972,7 +5088,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L42" s="22" t="inlineStr">
+      <c r="L42" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
@@ -4984,7 +5100,7 @@
       </c>
       <c r="N42" s="15" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="O42" s="18" t="inlineStr">
@@ -5021,27 +5137,46 @@
       </c>
       <c r="F43" s="20" t="inlineStr">
         <is>
-          <t>ไม่น้อยกว่า 30 หน่วยกิต</t>
+          <t>30 หน่วยกิต</t>
         </is>
       </c>
       <c r="G43" s="20" t="inlineStr">
         <is>
-          <t>หลักสูตร DSBA ต้องเก็บหมวดวิชาศึกษาทั่วไปไม่น้อยกว่า 30 หน่วยกิต [1]</t>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร DSBA 2565 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต — หน้า 15
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต ◀
+    - กลุ่มวิชาพื้นฐาน 6 หน่วยกิต
+    - กลุ่มวิชาด้านภาษาและการสื่อสาร 9 หน่วยกิต
+    - กลุ่มวิชาตามเกณฑ์ของคณะ 9 หน่วยกิต
+    - กลุ่มวิชาเลือกหมวดวิชาการศึกษาทั่วไป 6 หน่วยกิต
+  - หมวดวิชาเฉพาะ 96 หน่วยกิต
+    - กลุ่มวิชาแกน 45 หน่วยกิต
+      - กลุ่มคณิตศาสตร์และสถิติ 15 หน่วยกิต
+      - กลุ่มเทคโนโลยีสารสนเทศ 30 หน่วยกิต
+    - กลุ่มพื้นฐานวิชาชีพ 33 หน่วยกิต
+    - กลุ่มวิชาชีพเฉพาะด้าน 12 หน่วยกิต
+      - กลุ่มวิทยาการข้อมูล 12 หน่วยกิต
+      - กลุ่มการวิเคราะห์เชิงสถิติ 12 หน่วยกิต
+      - กลุ่มวิศวกรรมข้อมูล 12 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต
+หน่วยกิตรวมตลอดหลักสูตร 132 หน่วยกิต</t>
         </is>
       </c>
       <c r="H43" s="20" t="inlineStr">
         <is>
           <t>DSBA 2565 หน้า 15
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 351, 7, 15, 16)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 15)</t>
         </is>
       </c>
       <c r="I43" s="20" t="inlineStr">
         <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J43" s="19" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K43" s="15" t="inlineStr">
         <is>
@@ -5053,10 +5188,14 @@
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M43" s="20" t="inlineStr"/>
+      <c r="M43" s="20" t="inlineStr">
+        <is>
+          <t>ตอบจากตาราง rule พร้อมโครงสร้างทั้งหมดของหลักสูตร</t>
+        </is>
+      </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>1.06s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="O43" s="18" t="inlineStr">
@@ -5133,7 +5272,7 @@
       <c r="M44" s="16" t="inlineStr"/>
       <c r="N44" s="15" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="O44" s="18" t="inlineStr">
@@ -5206,7 +5345,7 @@
       <c r="M45" s="20" t="inlineStr"/>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="O45" s="18" t="inlineStr">
@@ -5221,7 +5360,7 @@
           <t>H8</t>
         </is>
       </c>
-      <c r="B46" s="23" t="inlineStr">
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5298,7 +5437,7 @@
           <t>H9</t>
         </is>
       </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5362,7 +5501,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.11s</t>
         </is>
       </c>
       <c r="O47" s="18" t="inlineStr">
@@ -5377,7 +5516,7 @@
           <t>H10</t>
         </is>
       </c>
-      <c r="B48" s="23" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5437,7 +5576,7 @@
       <c r="M48" s="16" t="inlineStr"/>
       <c r="N48" s="15" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="O48" s="18" t="inlineStr">
@@ -5452,7 +5591,7 @@
           <t>H11</t>
         </is>
       </c>
-      <c r="B49" s="23" t="inlineStr">
+      <c r="B49" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5479,42 +5618,47 @@
       </c>
       <c r="G49" s="20" t="inlineStr">
         <is>
-          <t>ไม่ได้  
-นักศึกษาต้องเรียนหน่วยกิตขั้นต่ำทั้งหมดไม่น้อยกว่า 120 หน่วยกิต ตามเกณฑ์การสำเร็จการศึกษาของหลักสูตร AIT ปี 2566 แม้จะมีการเรียนวิชาศึกษาทั่วไป 30 หน่วยกิต (เกินขั้นต่ำ 24 หน่วยกิต), วิชาเฉพาะ 80 หน่วยกิต (เกินขั้นต่ำ 52 หน่วยกิต), และวิชาเลือกเสรี 6 หน่วยกิต (เกินขั้นต่ำ 2 หน่วยกิต) แต่รวมแล้วยังเหลืออีก 4 หน่วยกิตที่ยังไม่ถึงเกณฑ์ 120 หน่วยกิต จึงไม่สามารถสำเร็จการศึกษาได้.</t>
+          <t>ผลการตรวจสอบเงื่อนไขการสำเร็จการศึกษา (หลักสูตร AIT 2566 (ปริญญาตรี)):
+▶ สรุป: **ยังไม่ครบเงื่อนไขสำเร็จการศึกษา**
+เทียบกับเกณฑ์ตามโครงสร้างหลักสูตรในเล่ม:
+- หมวดวิชาศึกษาทั่วไป: เก็บได้ 30 เกณฑ์ 24 → ครบตามเกณฑ์
+- หมวดวิชาเฉพาะ: เก็บได้ 80 เกณฑ์ 90 → **ขาดอีก 10 หน่วยกิต**
+- หมวดวิชาเลือกเสรี: เก็บได้ 6 เกณฑ์ 6 → ครบตามเกณฑ์
+- หน่วยกิตรวม: เก็บได้ 116 เกณฑ์ไม่น้อยกว่า 120 → **ขาดอีก 4 หน่วยกิต**</t>
         </is>
       </c>
       <c r="H49" s="20" t="inlineStr">
         <is>
           <t>AIT 2566 หน้า 18
-(หน้าที่ระบบคืนมา: AIT 2566 หน้า 235, 83, 78, 118)</t>
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 5)</t>
         </is>
       </c>
       <c r="I49" s="20" t="inlineStr">
         <is>
-          <t>Structured SQL (ตาราง rule มี provenance) — ไม่ผ่าน LLM</t>
+          <t>คำนวณเทียบเกณฑ์จากตาราง rule ของหลักสูตร (ไม่ผ่าน LLM)</t>
         </is>
       </c>
       <c r="J49" s="19" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K49" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L49" s="22" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="L49" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M49" s="20" t="inlineStr">
         <is>
-          <t>ข้อสรุป 'ไม่ได้ ขาด 4 หน่วยกิต จาก 120' ถูก แต่ LLM ใส่ขั้นต่ำหมวดวิชาเฉพาะเป็น 52 หน่วยกิต (เล่มคือ 90) และขั้นต่ำเลือกเสรี 2 ที่ยังไม่ได้ยืนยัน</t>
+          <t>ตอบจากตาราง rule: ศึกษาทั่วไป 24 (ครบ) · เฉพาะ 90 (ขาด 10) · เลือกเสรี 6 (ครบ) · รวม 120 (ขาด 4) ตรงเล่ม หน้า 18 (ก่อนแก้ ข้อสรุปถูกแต่ LLM ใส่ขั้นต่ำหมวดเฉพาะเป็น 52)</t>
         </is>
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>4.32s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O49" s="18" t="inlineStr">
@@ -5529,7 +5673,7 @@
           <t>H12</t>
         </is>
       </c>
-      <c r="B50" s="23" t="inlineStr">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5603,7 +5747,7 @@
       </c>
       <c r="N50" s="15" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O50" s="18" t="inlineStr">
@@ -5618,7 +5762,7 @@
           <t>H13</t>
         </is>
       </c>
-      <c r="B51" s="23" t="inlineStr">
+      <c r="B51" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5645,7 +5789,7 @@
       </c>
       <c r="G51" s="20" t="inlineStr">
         <is>
-          <t>หน่วยกิตต่อภาคตามแผนการศึกษาของ DSBA 2565 (ปริญญาตรี) (จากบรรทัด 'รวม' ของแต่ละภาคในเล่ม รวมวิชาเลือกที่แผนกำหนดแล้ว):
+          <t>หน่วยกิตต่อภาคตามแผนปกติของ DSBA 2565 (ปริญญาตรี) (จากบรรทัด 'รวม' ของแต่ละภาคในเล่ม รวมวิชาเลือกที่แผนกำหนดแล้ว):
   - ปีที่ 1 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 23)
   - ปีที่ 1 ภาคการศึกษาที่ 2: 21 หน่วยกิต (หน้า 24)
   - ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 25)
@@ -5660,7 +5804,7 @@
       <c r="H51" s="20" t="inlineStr">
         <is>
           <t>DSBA 2565 หน้า 24, 26 (บรรทัดรวม)
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 15, 23, 30, 352)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 23, 24, 25, 26)</t>
         </is>
       </c>
       <c r="I51" s="20" t="inlineStr">
@@ -5669,7 +5813,7 @@
         </is>
       </c>
       <c r="J51" s="19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K51" s="15" t="inlineStr">
         <is>
@@ -5688,7 +5832,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O51" s="18" t="inlineStr">
@@ -5703,7 +5847,7 @@
           <t>H14</t>
         </is>
       </c>
-      <c r="B52" s="23" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5765,7 +5909,7 @@
       </c>
       <c r="N52" s="15" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O52" s="18" t="inlineStr">
@@ -5780,7 +5924,7 @@
           <t>H15</t>
         </is>
       </c>
-      <c r="B53" s="23" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>ระดับ 3: ยาก (ชุดเพิ่ม)</t>
         </is>
@@ -5878,7 +6022,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.20s</t>
         </is>
       </c>
       <c r="O53" s="18" t="inlineStr">
@@ -5890,35 +6034,917 @@
     <row r="54" ht="80" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>หมวดวิชาศึกษาทั่วไปของ BIT 2565 ต้องเก็บกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>30 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร BIT 2565 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต — หน้า 18
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต ◀
+    - กลุ่มวิชาพื้นฐาน 6 หน่วยกิต
+    - กลุ่มวิชาด้านภาษาและการสื่อสาร 9 หน่วยกิต
+    - กลุ่มวิชาตามเกณฑ์ของคณะ 9 หน่วยกิต
+    - กลุ่มวิชาเลือกหมวดวิชาการศึกษาทั่วไป 6 หน่วยกิต
+  - หมวดวิชาเฉพาะ 90 หน่วยกิต
+    - กลุ่มวิชาแกน 12 หน่วยกิต
+      - กลุ่มพื้นฐานเทคโนโลยีสารสนเทศ 3 หน่วยกิต
+      - กลุ่มคณิตศาสตร์และสถิติสำหรับนักเทคโนโลยีสารสนเทศ 9 หน่วยกิต
+    - กลุ่มวิชาชีพเฉพาะด้าน 72 หน่วยกิต
+      - กลุ่มประเด็นด้านองค์การและระบบสารสนเทศ 24 หน่วยกิต
+      - กลุ่มเทคโนโลยีเพื่องานประยุกต์ 24 หน่วยกิต
+      - กลุ่มเทคโนโลยีและวิธีการทางซอฟต์แวร์ 18 หน่วยกิต
+      - กลุ่มโครงสร้างพื้นฐานของระบบ 6 หน่วยกิต
+    - กลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศทางธุรกิจ 6 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต
+หน่วยกิตรวมตลอดหลักสูตร 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>BIT 2565 หน้า 18
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 18)</t>
+        </is>
+      </c>
+      <c r="I54" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J54" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L54" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M54" s="16" t="inlineStr"/>
+      <c r="N54" s="15" t="inlineStr">
+        <is>
+          <t>0.18s</t>
+        </is>
+      </c>
+      <c r="O54" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="80" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="inlineStr">
+        <is>
+          <t>หมวดวิชาเลือกเสรีของ IT 2565 เก็บกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F55" s="20" t="inlineStr">
+        <is>
+          <t>6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G55" s="20" t="inlineStr">
+        <is>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร IT 2565 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ หมวดวิชาเลือกเสรี 6 หน่วยกิต — หน้า 21
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต
+    - กลุ่มวิชาพื้นฐาน 6 หน่วยกิต
+    - กลุ่มวิชาด้านภาษาและการสื่อสาร 9 หน่วยกิต
+    - กลุ่มวิชาตามเกณฑ์ของคณะ 9 หน่วยกิต
+    - กลุ่มวิชาเลือกหมวดวิชาศึกษาทั่วไป 6 หน่วยกิต
+  - หมวดวิชาเฉพาะ 93 หน่วยกิต
+    - กลุ่มวิชาแกน 12 หน่วยกิต
+      - กลุ่มคณิตศาสตร์และสถิติ 9 หน่วยกิต
+      - พื้นฐานเทคโนโลยีสารสนเทศ 3 หน่วยกิต
+    - กลุ่มวิชาเฉพาะด้าน 57 หน่วยกิต
+      - กลุ่มประเด็นด้านองค์การและระบบสารสนเทศ 9 หน่วยกิต
+      - กลุ่มเทคโนโลยีเพื่องานประยุกต์ 27 หน่วยกิต
+      - กลุ่มเทคโนโลยีและวิธีการทางซอฟต์แวร์ 12 หน่วยกิต
+      - กลุ่มโครงสร้างพื้นฐานของระบบ 9 หน่วยกิต
+    - กลุ่มวิชาบังคับเฉพาะสาขา 15 หน่วยกิต
+    - กลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศ 9 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต ◀
+หน่วยกิตรวมตลอดหลักสูตร 129 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H55" s="20" t="inlineStr">
+        <is>
+          <t>IT 2565 หน้า 21
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 21)</t>
+        </is>
+      </c>
+      <c r="I55" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J55" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M55" s="20" t="inlineStr">
+        <is>
+          <t>รอบแรกมีบรรทัดกลุ่มวิชาเฉพาะด้านปนมาด้วย (คำเทียบเคียงที่ระบบต่อท้ายคำถามถูกนับเป็นคำของผู้ถาม) แก้แล้ว</t>
+        </is>
+      </c>
+      <c r="N55" s="19" t="inlineStr">
+        <is>
+          <t>0.36s</t>
+        </is>
+      </c>
+      <c r="O55" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="80" customHeight="1">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>หมวดวิชาเฉพาะของ AIT 2566 มีกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>90 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร AIT 2566 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ หมวดวิชาเฉพาะ 90 หน่วยกิต — หน้า 18
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 24 หน่วยกิต
+  - หมวดวิชาเฉพาะ 90 หน่วยกิต ◀
+    - กลุ่มวิชาพื้นฐานคณิตศาสตร์และสถิติ 15 หน่วยกิต
+    - กลุ่มวิชาพื้นฐานวิทยาศาสตร์คอมพิวเตอร์ 15 หน่วยกิต
+    - กลุ่มวิชา พื้นฐานปัญญาประดิษฐ์ 33 หน่วยกิต
+    - กลุ่มวิชาเลือกปัญญาประดิษฐ์เฉพาะทาง 12 หน่วยกิต
+    - กลุ่มวิชาโครงงานและสัมมนา 15 หน่วยกิต
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต
+หน่วยกิตรวมตลอดหลักสูตร 120 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H56" s="16" t="inlineStr">
+        <is>
+          <t>AIT 2566 หน้า 18
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 18)</t>
+        </is>
+      </c>
+      <c r="I56" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J56" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L56" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M56" s="16" t="inlineStr"/>
+      <c r="N56" s="15" t="inlineStr">
+        <is>
+          <t>0.24s</t>
+        </is>
+      </c>
+      <c r="O56" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="80" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr">
+        <is>
+          <t>หมวดวิชาเฉพาะของ BIT 2560 เก็บกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F57" s="20" t="inlineStr">
+        <is>
+          <t>90 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G57" s="20" t="inlineStr">
+        <is>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร BIT 2560 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ หมวดวิชาเฉพาะ 90 หน่วยกิต — หน้า 17
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต
+    - กลุ่มวิชาภาษา 12 หน่วยกิต
+    - กลุ่มวิชาวิทยาศาสตร์กับคณิตศาสตร์ 6 หน่วยกิต
+    - กลุ่มวิชามนุษยศาสตร์ 6 หน่วยกิต
+    - กลุ่มวิชาสังคมศาสตร์ 6 หน่วยกิต
+  - หมวดวิชาเฉพาะ 90 หน่วยกิต ◀
+    - กลุ่มวิชาแกน 9 หน่วยกิต
+    - กลุ่มวิชาเฉพาะด้าน 75 หน่วยกิต
+    - กลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศทางธุรกิจ 6 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต
+หน่วยกิตรวมตลอดหลักสูตร 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H57" s="20" t="inlineStr">
+        <is>
+          <t>BIT 2560 หน้า 17
+(หน้าที่ระบบคืนมา: BIT 2560 หน้า 17)</t>
+        </is>
+      </c>
+      <c r="I57" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J57" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L57" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M57" s="20" t="inlineStr"/>
+      <c r="N57" s="19" t="inlineStr">
+        <is>
+          <t>0.18s</t>
+        </is>
+      </c>
+      <c r="O57" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>หมวดวิชาเลือกเสรีของ DSBA 2560 กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตตามโครงสร้างหลักสูตร DSBA 2560 (ปริญญาตรี) (จากหน้าโครงสร้างหลักสูตรใน มคอ.2):
+▶ หมวดวิชาเลือกเสรี 6 หน่วยกิต — หน้า 18
+โครงสร้างทั้งหมดของหลักสูตร:
+  - หมวดวิชาศึกษาทั่วไป 30 หน่วยกิต
+  - หมวดวิชาเฉพาะ 90 หน่วยกิต
+    - กลุ่มวิชาแกน 12 หน่วยกิต
+    - กลุ่มวิชาเฉพาะด้าน 69 หน่วยกิต
+    - กลุ่มวิชาเลือก 6 หน่วยกิต
+    - กลุ่มวิชาการศึกษาทางเลือก 3 หน่วยกิต
+  - หมวดวิชาเลือกเสรี 6 หน่วยกิต ◀
+หน่วยกิตรวมตลอดหลักสูตร 126 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>DSBA 2560 หน้า 18
+(หน้าที่ระบบคืนมา: DSBA 2560 หน้า 18)</t>
+        </is>
+      </c>
+      <c r="I58" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (โครงสร้างหน่วยกิตรายหมวด ตาราง rule มีหน้าที่มา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J58" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L58" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>รอบแรกมีบรรทัดกลุ่มวิชาเฉพาะด้านปนมาด้วย (สาเหตุเดียวกับ W2) แก้แล้ว</t>
+        </is>
+      </c>
+      <c r="N58" s="15" t="inlineStr">
+        <is>
+          <t>0.12s</t>
+        </is>
+      </c>
+      <c r="O58" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="80" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B59" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>แผนสหกิจของ BIT 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F59" s="20" t="inlineStr">
+        <is>
+          <t>6 หน่วยกิต (สหกิจศึกษา 06036147 หรือสหกิจศึกษาต่างประเทศ 06036148)</t>
+        </is>
+      </c>
+      <c r="G59" s="20" t="inlineStr">
+        <is>
+          <t>แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 35):
+  - 06036147 สหกิจศึกษา — 6(0-35-0)
+  - 06036148 สหกิจศึกษาต่างประเทศ — 6(0-35-0)
+  รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H59" s="20" t="inlineStr">
+        <is>
+          <t>BIT 2565 หน้า 35
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 35)</t>
+        </is>
+      </c>
+      <c r="I59" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J59" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L59" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M59" s="20" t="inlineStr"/>
+      <c r="N59" s="19" t="inlineStr">
+        <is>
+          <t>0.14s</t>
+        </is>
+      </c>
+      <c r="O59" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B60" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>ในแผนสหกิจศึกษาของ IT 2565 วิชาสหกิจศึกษาอยู่ปีไหน ภาคไหน กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>ปีที่ 3 ภาคการศึกษาที่ 2 จำนวน 6 หน่วยกิต (06016481 สหกิจศึกษา หรือ 06016482 สหกิจศึกษาต่างประเทศ)</t>
+        </is>
+      </c>
+      <c r="G60" s="16" t="inlineStr">
+        <is>
+          <t>รายวิชาที่มีเฉพาะในแผนที่เข้าโครงการสหกิจศึกษา (IT 2565 (ปริญญาตรี)):
+- 06016481 สหกิจศึกษา — 6(0-36-0) | ปีที่ 3 ภาคการศึกษาที่ 2 (หน้า 42, 43)
+- 06016482 สหกิจศึกษาต่างประเทศ — 6(0-36-0) | ปีที่ 3 ภาคการศึกษาที่ 2 (หน้า 42, 43)
+ภาคนั้นรวม 6 หน่วยกิตตามแผนในเล่ม (ในแผนปกติภาคเดียวกันรวม 15 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H60" s="16" t="inlineStr">
+        <is>
+          <t>IT 2565 หน้า 42-43
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 42, 43)</t>
+        </is>
+      </c>
+      <c r="I60" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J60" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K60" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L60" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M60" s="16" t="inlineStr"/>
+      <c r="N60" s="15" t="inlineStr">
+        <is>
+          <t>0.18s</t>
+        </is>
+      </c>
+      <c r="O60" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="80" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B61" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr">
+        <is>
+          <t>ถ้าเข้าโครงการสหกิจศึกษา DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 1 ต้องเรียนอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>โครงงาน 2 (06026215) + วิชาเลือกหมวดศึกษาทั่วไป 1 + วิชาเลือกเสรี 2 รวม 12 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G61" s="20" t="inlineStr">
+        <is>
+          <t>แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 36):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H61" s="20" t="inlineStr">
+        <is>
+          <t>DSBA 2565 หน้า 36
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36)</t>
+        </is>
+      </c>
+      <c r="I61" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J61" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K61" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L61" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M61" s="20" t="inlineStr"/>
+      <c r="N61" s="19" t="inlineStr">
+        <is>
+          <t>0.11s</t>
+        </is>
+      </c>
+      <c r="O61" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="80" customHeight="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B62" s="22" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>แผนปกติกับแผนสหกิจของ BIT 2565 ต่างกันที่ภาคเรียนใดบ้าง</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>หน่วยกิตต่างกัน 3 ภาค: ปี 3 ภาค 2 (ปกติ 12 / สหกิจ 15), ปี 4 ภาค 1 (ปกติ 12 / สหกิจ 15), ปี 4 ภาค 2 (ปกติ 12 / สหกิจ 6 คือสหกิจศึกษา) รวมทั้งหลักสูตรเท่ากัน 126</t>
+        </is>
+      </c>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบแผนการศึกษา BIT 2565 (ปริญญาตรี): แผนปกติ (3.1.4.1) กับแผนที่เข้าโครงการสหกิจศึกษา (3.1.4.2)
+- ปีที่ 1 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 1 ภาคการศึกษาที่ 2: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 2: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 2: แผนปกติ 12 หน่วยกิต · แผนสหกิจ 15 หน่วยกิต  ← ต่างกัน
+- ปีที่ 4 ภาคการศึกษาที่ 1: แผนปกติ 12 หน่วยกิต · แผนสหกิจ 15 หน่วยกิต  ← ต่างกัน
+- ปีที่ 4 ภาคการศึกษาที่ 2: แผนปกติ 12 หน่วยกิต · แผนสหกิจ 6 หน่วยกิต  ← ต่างกัน
+รวมตลอดหลักสูตร: แผนปกติ 126 หน่วยกิต · แผนสหกิจ 126 หน่วยกิต (เท่ากัน)
+ภาคที่ต่างกัน: ปี 3 ภาค 2, ปี 4 ภาค 1, ปี 4 ภาค 2
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 3 ภาคการศึกษาที่ 2 (หน้า 29):
+  - 06036106 การจัดการข้อมูลธุรกิจและเทคโนโลยีเกิดใหม่ — 3(3-0-6)
+  - 06036116 การตลาดเชิงดิจิทัล — 3(2-2-5)
+  - 06036145 โครงงานทางด้านเทคโนโลยีสารสนเทศเชิงธุรกิจ 1 — 3(0-9-0)
+  - 96643021 กฎหมายสำหรับคนรุ่นใหม่ — 3(3-0-6)
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 3 ภาคการศึกษาที่ 2 (หน้า 34):
+  - 06036106 การจัดการข้อมูลธุรกิจและเทคโนโลยีเกิดใหม่ — 3(3-0-6)
+  - 06036116 การตลาดเชิงดิจิทัล — 3(2-2-5)
+  - 96643021 กฎหมายสำหรับคนรุ่นใหม่ — 3(3-0-6)
+  - วิชาเลือกที่ต้องลงตามแผน: 2 ช่อง
+      • วิชาเลือกทางเทคโนโลยีสารสนเทศทางธุรกิจ 1
+      • วิชาเลือกเสรี 1
+  รวมภาคนี้ตามแผนในเล่ม: 15 หน่วยกิต
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 29):
+  - 06036115 ความมั่นคงของระบบสารสนเทศ — 3(3-0-6)
+  - 06036146 โครงงานทางด้านเทคโนโลยีสารสนเทศเชิงธุรกิจ 2 — 3(0-9-0)
+  - 96642033 กลุ่มวิชาที่กำหนดโดยคณะ — 3(3-0-6)
+  - วิชาเลือกที่ต้องลงตามแผน: 1 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป สำหรับหลักสูตรนานาชาติ 2
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 35):
+  - 06036115 ความมั่นคงของระบบสารสนเทศ — 3(3-0-6)
+  - 96642033 กลุ่มวิชาที่กำหนดโดยคณะ — 3(3-0-6)
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกทางเทคโนโลยีสารสนเทศทางธุรกิจ 2
+      • วิชาเลือกเสรี 2
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป สำหรับหลักสูตรนานาชาติ 2
+  รวมภาคนี้ตามแผนในเล่ม: 15 หน่วยกิต
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 30):
+  - วิชาเลือกที่ต้องลงตามแผน: 2 ช่อง
+      • วิชาเลือกทางเทคโนโลยีสารสนเทศทางธุรกิจ 1
+      • วิชาเลือกทางเทคโนโลยีสารสนเทศทางธุรกิจ 2
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 35):
+  - 06036147 สหกิจศึกษา — 6(0-35-0)
+  - 06036148 สหกิจศึกษาต่างประเทศ — 6(0-35-0)
+  รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต
+ตามโครงสร้างหลักสูตร: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (สหกิจศึกษา 6 หน่วยกิต (เฉพาะแผนที่เข้าโครงการสหกิจศึกษา))</t>
+        </is>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>BIT 2565 หน้า 26-35
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 29, 34, 35, 30)</t>
+        </is>
+      </c>
+      <c r="I62" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J62" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K62" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L62" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M62" s="16" t="inlineStr">
+        <is>
+          <t>รอบแรกระบุว่าปี 1 ภาค 2 ต่างกัน ทั้งที่ต่างแค่ลำดับแถววิชาในตาราง (รอบแรก: ถูกบางส่วน) แก้เป็นเทียบแบบเซ็ตแล้ว ตอนนี้ตอบ ปี 3 ภาค 2, ปี 4 ภาค 1, ปี 4 ภาค 2</t>
+        </is>
+      </c>
+      <c r="N62" s="15" t="inlineStr">
+        <is>
+          <t>0.08s</t>
+        </is>
+      </c>
+      <c r="O62" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="80" customHeight="1">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B63" s="22" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก (ชุดใหม่ W)</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D63" s="20" t="inlineStr">
+        <is>
+          <t>ภาคเรียนไหนในแผนปกติของ IT 2565 ลงหน่วยกิตน้อยที่สุด กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F63" s="20" t="inlineStr">
+        <is>
+          <t>ปี 4 ภาค 2 จำนวน 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G63" s="20" t="inlineStr">
+        <is>
+          <t>หน่วยกิตต่อภาคตามแผนปกติของ IT 2565 (ปริญญาตรี) (จากบรรทัด 'รวม' ของแต่ละภาคในเล่ม รวมวิชาเลือกที่แผนกำหนดแล้ว):
+  - ปีที่ 1 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 31)
+  - ปีที่ 1 ภาคการศึกษาที่ 2: 18 หน่วยกิต (หน้า 32)
+  - ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 33)
+  - ปีที่ 2 ภาคการศึกษาที่ 2: 18 หน่วยกิต (หน้า 34)
+  - ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 35)
+  - ปีที่ 3 ภาคการศึกษาที่ 2: 15 หน่วยกิต (หน้า 35)
+  - ปีที่ 4 ภาคการศึกษาที่ 1: 15 หน่วยกิต (หน้า 37)
+  - ปีที่ 4 ภาคการศึกษาที่ 2: 9 หน่วยกิต (หน้า 37)
+ภาคที่หน่วยกิตน้อยที่สุด: ปีที่ 4 ภาคการศึกษาที่ 2 — 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H63" s="20" t="inlineStr">
+        <is>
+          <t>IT 2565 หน้า 37
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 31, 32, 33, 34)</t>
+        </is>
+      </c>
+      <c r="I63" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (หน่วยกิตรวมต่อภาคจากหน้าแผนในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J63" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="K63" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L63" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M63" s="20" t="inlineStr">
+        <is>
+          <t>รอบแรกตารางขาดปี 3 ภาค 2 (ตารางล้นไปอีกหน้า) แต่คำตอบ 9 หน่วยกิตถูก (รอบแรก: ถูกบางส่วน) แก้แล้ว ได้ครบ 8 ภาค</t>
+        </is>
+      </c>
+      <c r="N63" s="19" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O63" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="80" customHeight="1">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="B54" s="24" t="inlineStr">
+      <c r="B64" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C54" s="15" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตรของ DSBA ฉบับ 2560 กับฉบับ 2565 ต่างกันกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E54" s="16" t="inlineStr">
+      <c r="E64" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F54" s="16" t="inlineStr">
+      <c r="F64" s="16" t="inlineStr">
         <is>
           <t>2560 = 126 หน่วยกิต, 2565 = 132 หน่วยกิต ต่างกัน 6 หน่วยกิต (2565 มากกว่า)</t>
         </is>
       </c>
-      <c r="G54" s="16" t="inlineStr">
+      <c r="G64" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
@@ -5926,78 +6952,78 @@
 สรุป: DSBA 2565 มากกว่า DSBA 2560 อยู่ 6 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H54" s="16" t="inlineStr">
+      <c r="H64" s="16" t="inlineStr">
         <is>
           <t>DSBA2560 หน้า 17; DSBA2565 หน้า 15
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 351, 349, 352; DSBA 2560 หน้า 17)</t>
         </is>
       </c>
-      <c r="I54" s="16" t="inlineStr">
+      <c r="I64" s="16" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J54" s="15" t="n">
+      <c r="J64" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K54" s="15" t="inlineStr">
+      <c r="K64" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L54" s="18" t="inlineStr">
+      <c r="L64" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M54" s="16" t="inlineStr">
+      <c r="M64" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N54" s="15" t="inlineStr">
-        <is>
-          <t>0.35s</t>
-        </is>
-      </c>
-      <c r="O54" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="80" customHeight="1">
-      <c r="A55" s="13" t="inlineStr">
+      <c r="N64" s="15" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O64" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="80" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B55" s="24" t="inlineStr">
+      <c r="B65" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C55" s="19" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="D55" s="20" t="inlineStr">
+      <c r="D65" s="20" t="inlineStr">
         <is>
           <t>หลักสูตร BIT 2560 กับ BIT 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากันหรือไม่</t>
         </is>
       </c>
-      <c r="E55" s="20" t="inlineStr">
+      <c r="E65" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F55" s="20" t="inlineStr">
+      <c r="F65" s="20" t="inlineStr">
         <is>
           <t>เท่ากัน ทั้งสองฉบับ 126 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G55" s="20" t="inlineStr">
+      <c r="G65" s="20" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - BIT 2560: 126 หน่วยกิต (มคอ.2 BIT 2560 หน้า 17)
@@ -6005,78 +7031,78 @@
 สรุป: เท่ากัน (126 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H55" s="20" t="inlineStr">
+      <c r="H65" s="20" t="inlineStr">
         <is>
           <t>BIT2560 หน้า 17; BIT2565 หน้า 6
 (หน้าที่ระบบคืนมา: BIT 2565 หน้า 266, 264, 3, 265)</t>
         </is>
       </c>
-      <c r="I55" s="20" t="inlineStr">
+      <c r="I65" s="20" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J55" s="19" t="n">
+      <c r="J65" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="K55" s="15" t="inlineStr">
+      <c r="K65" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L55" s="18" t="inlineStr">
+      <c r="L65" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M55" s="20" t="inlineStr">
+      <c r="M65" s="20" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N55" s="19" t="inlineStr">
+      <c r="N65" s="19" t="inlineStr">
         <is>
           <t>0.08s</t>
         </is>
       </c>
-      <c r="O55" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="80" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="O65" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="80" customHeight="1">
+      <c r="A66" s="13" t="inlineStr">
         <is>
           <t>X3</t>
         </is>
       </c>
-      <c r="B56" s="24" t="inlineStr">
+      <c r="B66" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C56" s="15" t="inlineStr">
+      <c r="C66" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
         <is>
           <t>ระหว่างหลักสูตร DSBA 2565, AIT 2566 และ BIT 2565 หลักสูตรใดมีหน่วยกิตรวมมากที่สุด</t>
         </is>
       </c>
-      <c r="E56" s="16" t="inlineStr">
+      <c r="E66" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F56" s="16" t="inlineStr">
+      <c r="F66" s="16" t="inlineStr">
         <is>
           <t>DSBA 2565 มากที่สุด 132 หน่วยกิต (BIT 2565 = 126, AIT 2566 = 120)</t>
         </is>
       </c>
-      <c r="G56" s="16" t="inlineStr">
+      <c r="G66" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
@@ -6085,237 +7111,235 @@
 สรุป: มากที่สุดคือ DSBA 2565 (132 หน่วยกิต) น้อยที่สุดคือ AIT 2566 (120 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H56" s="16" t="inlineStr">
+      <c r="H66" s="16" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 15; BIT2565 หน้า 6; AIT2566 หน้า 5
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 78; DSBA 2565 หน้า 352, 349; BIT 2565 หน้า 264)</t>
         </is>
       </c>
-      <c r="I56" s="16" t="inlineStr">
+      <c r="I66" s="16" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J56" s="15" t="n">
+      <c r="J66" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K56" s="15" t="inlineStr">
+      <c r="K66" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L56" s="18" t="inlineStr">
+      <c r="L66" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M56" s="16" t="inlineStr">
+      <c r="M66" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N56" s="15" t="inlineStr">
-        <is>
-          <t>0.16s</t>
-        </is>
-      </c>
-      <c r="O56" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="80" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="N66" s="15" t="inlineStr">
+        <is>
+          <t>0.22s</t>
+        </is>
+      </c>
+      <c r="O66" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="80" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
         <is>
           <t>X4</t>
         </is>
       </c>
-      <c r="B57" s="24" t="inlineStr">
+      <c r="B67" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C57" s="19" t="inlineStr">
+      <c r="C67" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D57" s="20" t="inlineStr">
+      <c r="D67" s="20" t="inlineStr">
         <is>
           <t>ในแผนสหกิจศึกษาของ DSBA 2565 ต้องลงทะเบียนวิชาสหกิจศึกษาในภาคไหน และกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E57" s="20" t="inlineStr">
+      <c r="E67" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F57" s="20" t="inlineStr">
+      <c r="F67" s="20" t="inlineStr">
         <is>
           <t>ปีที่ 4 ภาคการศึกษาที่ 2 จำนวน 6 หน่วยกิต (06026259 สหกิจศึกษา หรือ 06026260 สหกิจศึกษาต่างประเทศ)</t>
         </is>
       </c>
-      <c r="G57" s="20" t="inlineStr">
-        <is>
-          <t>นักศึกษาต้องลงทะเบียนวิชาสหกิจศึกษาในภาคการศึกษาที่ 3 ของปีที่ 3 จำนวน 6 หน่วยกิต [5]</t>
-        </is>
-      </c>
-      <c r="H57" s="20" t="inlineStr">
+      <c r="G67" s="20" t="inlineStr">
+        <is>
+          <t>รายวิชาที่มีเฉพาะในแผนที่เข้าโครงการสหกิจศึกษา (DSBA 2565 (ปริญญาตรี)):
+- 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0) | ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36)
+- 06026260 สหกิจศึกษาต่างประเทศทางวิทยาการข้อมูลและการ วิเคราะห์เชิงธุรกิจ — 6 (0-35-0) | ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36)
+ภาคนั้นรวม 6 หน่วยกิตตามแผนในเล่ม (ในแผนปกติภาคเดียวกันรวม 9 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H67" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 36
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 30, 23, 354, 15)</t>
-        </is>
-      </c>
-      <c r="I57" s="20" t="inlineStr">
-        <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
-        </is>
-      </c>
-      <c r="J57" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="K57" s="15" t="inlineStr">
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36)</t>
+        </is>
+      </c>
+      <c r="I67" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J67" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K67" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L57" s="25" t="inlineStr">
-        <is>
-          <t>ผิด</t>
-        </is>
-      </c>
-      <c r="M57" s="20" t="inlineStr">
-        <is>
-          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ตอบว่าลงสหกิจภาค 3/ภาค 4 ของปี 3/ปี 4 แต่เล่มหน้า 36 คือปี 4 ภาค 2</t>
-        </is>
-      </c>
-      <c r="N57" s="19" t="inlineStr">
-        <is>
-          <t>1.23s</t>
-        </is>
-      </c>
-      <c r="O57" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="80" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M67" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ตอบจากตารางแผนสหกิจในเล่ม: สหกิจศึกษา 06026259/06026260 ปี 4 ภาค 2 6 หน่วยกิต (หน้า 36)</t>
+        </is>
+      </c>
+      <c r="N67" s="19" t="inlineStr">
+        <is>
+          <t>0.07s</t>
+        </is>
+      </c>
+      <c r="O67" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="80" customHeight="1">
+      <c r="A68" s="13" t="inlineStr">
         <is>
           <t>X5</t>
         </is>
       </c>
-      <c r="B58" s="24" t="inlineStr">
+      <c r="B68" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C58" s="15" t="inlineStr">
+      <c r="C68" s="15" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr">
         <is>
           <t>หลักสูตรปริญญาโท IT 2563 กับ 2568 แบ่งแผนการศึกษาต่างกันอย่างไร</t>
         </is>
       </c>
-      <c r="E58" s="16" t="inlineStr">
+      <c r="E68" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="F68" s="16" t="inlineStr">
         <is>
           <t>2563: แผน ก (แบบ ก1, ก2) และแผน ข; 2568: แผน 1 แบบวิชาการ (แบบ 1.1, 1.2) และแผน 2 แบบวิชาชีพ; ทุกแผนเรียน 36 หน่วยกิตเท่ากัน</t>
         </is>
       </c>
-      <c r="G58" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2563 (IT 2563) และ 2568 (IT 2568) มีแผนการศึกษาต่างกันดังนี้:
-- **แผน ก แบบ ก 1 และ ก 2 (ปี 2563)**:  
-  รับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ชั้นปีที่ 2 ปีละ 5 คน รวมปีละ 10 คน โดยคาดว่าจะสำเร็จการศึกษา 5 คนต่อปีตั้งแต่ปี 2564 เป็นต้นไป [3]
-- **แผน 1 แบบวิชาการ แบบ 1.1 และ 1.2 (ปี 2568)**:  
-  รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ชั้นปีที่ 2 ปีละ 3 คน รวมปีละ 6 คน โดยคาดว่าจะสำเร็จการศึกษา 3 คนต่อปีตั้งแต่ปี 2569 เป็นต้นไป [2]
-- **แผน 2 แบบวิชาชีพ (ปี 2568)**:  
-  รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ชั้นปีที่ 2 ปีละ 30 คน รวมปีละ 60 คน โดยคาดว่าจะสำเร็จการศึกษา 30 คนต่อปีตั้งแต่ปี 2569 เป็นต้นไป [2]
-สรุป: หลักสูตรปี 2568 มีแผนการรับนักศึกษาหลายแบบมากกว่า ปี 2563 ทั้งในด้านจำนวนนักศึกษาและประเภทแผนการศึกษา โดยเฉพาะเพิ่มแผนวิชาชีพที่รับนักศึกษาจำนวนมากกว่า [2][3]</t>
-        </is>
-      </c>
-      <c r="H58" s="16" t="inlineStr">
+      <c r="G68" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2563 (IT 2563) มีแผนการศึกษาแบบ ก 1 และ ก 2 ซึ่งรับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ตั้งแต่ปีการศึกษา 2563 ถึง 2567 โดยมีนักศึกษาชั้นปีที่ 2 เริ่มเข้าศึกษาในปีการศึกษา 2564 เป็นต้นไป รวมนักศึกษาทั้งหมดในแต่ละปีไม่เกิน 10 คน และคาดว่าจะสำเร็จการศึกษา 5 คนต่อปีตั้งแต่ปีการศึกษา 2564 [3]
+ในขณะที่หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2568 (IT 2568) มีแผนการศึกษา 3 แบบ ได้แก่ แผน 1 แบบวิชาการ แบบ 1.1 และ 1.2 รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ตั้งแต่ปีการศึกษา 2568 ถึง 2572 รวมนักศึกษาทั้งหมดในแต่ละปีไม่เกิน 6 คน และคาดว่าจะสำเร็จการศึกษา 3 คนต่อปีตั้งแต่ปีการศึกษา 2569 เป็นต้นไป พร้อมกันนี้ยังมีแผน 2 แบบวิชาชีพ รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ตั้งแต่ปีการศึกษา 2568 ถึง 2572 รวมนักศึกษาทั้งหมดในแต่ละปีไม่เกิน 60 คน และคาดว่าจะสำเร็จการศึกษา 30 คนต่อปีตั้งแต่ปีการศึกษา 2569 เป็นต้นไป [2]
+ดังนั้น ความแตกต่างคือ หลักสูตร 2563 มีเพียง 2 แผน (ก 1 และ ก 2) รับคนละ 5 คนต่อปี ขณะที่หลักสูตร 2568 มี 3 แผน แบ่งเป็นแผนวิชาการ (แบบ 1.1 และ 1.2) รับคนละ 3 คนต่อปี และแผนวิชาชีพรับ 30 คนต่อปี ทำให้จำนวนนักศึก</t>
+        </is>
+      </c>
+      <c r="H68" s="16" t="inlineStr">
         <is>
           <t>IT2563 หน้า 16; IT2568 หน้า 5
 (หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 153, 11; วท.ม. IT 2563 หน้า 15)</t>
         </is>
       </c>
-      <c r="I58" s="16" t="inlineStr">
+      <c r="I68" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J58" s="15" t="n">
+      <c r="J68" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="K58" s="15" t="inlineStr">
+      <c r="K68" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L58" s="22" t="inlineStr">
+      <c r="L68" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
       </c>
-      <c r="M58" s="16" t="inlineStr">
+      <c r="M68" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] อธิบายแผนของ 2568 ถูก แต่ของ 2563 ขาดแผน ข และตอบจำนวนรับนักศึกษาแทนโครงสร้างแผน</t>
         </is>
       </c>
-      <c r="N58" s="15" t="inlineStr">
-        <is>
-          <t>9.63s</t>
-        </is>
-      </c>
-      <c r="O58" s="15" t="inlineStr">
+      <c r="N68" s="15" t="inlineStr">
+        <is>
+          <t>12.81s</t>
+        </is>
+      </c>
+      <c r="O68" s="15" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="80" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
+    <row r="69" ht="80" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
         <is>
           <t>X6</t>
         </is>
       </c>
-      <c r="B59" s="24" t="inlineStr">
+      <c r="B69" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C59" s="19" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D59" s="20" t="inlineStr">
+      <c r="D69" s="20" t="inlineStr">
         <is>
           <t>ถ้าจะเรียนวิชาพื้นฐานการเรียนรู้เชิงลึก (Fundamentals of Deep Learning) ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
         </is>
       </c>
-      <c r="E59" s="20" t="inlineStr">
+      <c r="E69" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F59" s="20" t="inlineStr">
+      <c r="F69" s="20" t="inlineStr">
         <is>
           <t>ต้องผ่านแคลคูลัส 2 (06046401) และพีชคณิตเชิงเส้น (06046402); แคลคูลัส 2 ต้องผ่านแคลคูลัส 1 (06046400) ก่อน; พีชคณิตเชิงเส้นและแคลคูลัส 1 ไม่มีวิชาบังคับก่อน</t>
         </is>
       </c>
-      <c r="G59" s="20" t="inlineStr">
+      <c r="G69" s="20" t="inlineStr">
         <is>
           <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   ต้องผ่านวิชาบังคับก่อน:
@@ -6324,234 +7348,268 @@
     • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
         </is>
       </c>
-      <c r="H59" s="20" t="inlineStr">
+      <c r="H69" s="20" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 287-288
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 37, 292, 19, 20)</t>
         </is>
       </c>
-      <c r="I59" s="20" t="inlineStr">
+      <c r="I69" s="20" t="inlineStr">
         <is>
           <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J59" s="19" t="n">
+      <c r="J69" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K59" s="15" t="inlineStr">
+      <c r="K69" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L59" s="18" t="inlineStr">
+      <c r="L69" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M59" s="20" t="inlineStr">
+      <c r="M69" s="20" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ไล่วิชาบังคับก่อน 2 ชั้นได้ครบ</t>
         </is>
       </c>
-      <c r="N59" s="19" t="inlineStr">
-        <is>
-          <t>0.30s</t>
-        </is>
-      </c>
-      <c r="O59" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="80" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="N69" s="19" t="inlineStr">
+        <is>
+          <t>0.90s</t>
+        </is>
+      </c>
+      <c r="O69" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="80" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
         <is>
           <t>X7</t>
         </is>
       </c>
-      <c r="B60" s="24" t="inlineStr">
+      <c r="B70" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="C70" s="15" t="inlineStr">
         <is>
           <t>AITBA</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
+      <c r="D70" s="16" t="inlineStr">
         <is>
           <t>หลักสูตรปริญญาโท AITBA 2564 กับ 2569 หน่วยกิตที่เรียนตลอดหลักสูตรต่างกันไหม และชื่อแผนการศึกษาเปลี่ยนไปอย่างไร</t>
         </is>
       </c>
-      <c r="E60" s="16" t="inlineStr">
+      <c r="E70" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F60" s="16" t="inlineStr">
+      <c r="F70" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตไม่ต่าง ทุกแผน 36 หน่วยกิต; 2564 ใช้แผน ก (ก1, ก2) และแผน ข; 2569 ใช้แผนวิชาการ (แบบ 1.1, 1.2) และแผนวิชาชีพ</t>
         </is>
       </c>
-      <c r="G60" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท AITBA 2564 และ 2569 ไม่มีความแตกต่างในจำนวนหน่วยกิตที่เรียนตลอดหลักสูตร เนื่องจากทั้งสองฉบับกำหนดให้มีจำนวนหน่วยกิตรวมไม่น้อยกว่า 36 หน่วยกิต [6]  
-สำหรับชื่อแผนการศึกษา:  
-- หลักสูตร AITBA 2564 มีแผนการศึกษา 2 แผน คือ แผน ก (แบบ ก1 และ ก2) และแผน ข [6]  
-- หลักสูตร AITBA 2569 ปรับปรุงชื่อแผนการศึกษาใหม่เป็น แผน 1.1 (แบบวิชาการ), แผน 1.2 (แบบวิชาการ), และแผน 2 (แบบวิชาชีพ) [3]  
-ดังนั้น ชื่อแผนการศึกษาเปลี่ยนแปลงตามการปรับปรุงโครงสร้างหลักสูตร [3]</t>
-        </is>
-      </c>
-      <c r="H60" s="16" t="inlineStr">
+      <c r="G70" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท AITBA 2564 และ 2569 ไม่มีการเปลี่ยนแปลงจำนวนหน่วยกิตที่เรียนตลอดหลักสูตร เนื่องจากทั้งสองฉบับมีจำนวนหน่วยกิตรวมทั้งหมด 36 หน่วยกิต [6]  
+สำหรับชื่อแผนการศึกษา หลักสูตร AITBA 2569 มีการปรับปรุงชื่อแผนการศึกษาดังนี้:  
+- แผน ก แบบ ก1 เปลี่ยนเป็น แผน 1.1 (แบบวิชาการ) [3]  
+- แผน ก แบบ ก2 เปลี่ยนเป็น แผน 1.2 (แบบวิชาการ) [3]  
+- แผน ข เปลี่ยนเป็น แผน 2 (แบบวิชาชีพ) [3]</t>
+        </is>
+      </c>
+      <c r="H70" s="16" t="inlineStr">
         <is>
           <t>AITBA2564 หน้า 6; AITBA2569 หน้า 5
 (หน้าที่ระบบคืนมา: ปร.ด. AITBA 2569 หน้า 223, 99, 225, 167; วท.ม. AITBA 2564 หน้า 6, 3)</t>
         </is>
       </c>
-      <c r="I60" s="16" t="inlineStr">
+      <c r="I70" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J60" s="15" t="n">
+      <c r="J70" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="K60" s="15" t="inlineStr">
+      <c r="K70" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L60" s="18" t="inlineStr">
+      <c r="L70" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M60" s="16" t="inlineStr">
+      <c r="M70" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N60" s="15" t="inlineStr">
-        <is>
-          <t>5.02s</t>
-        </is>
-      </c>
-      <c r="O60" s="15" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="80" customHeight="1">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="N70" s="15" t="inlineStr">
+        <is>
+          <t>4.96s</t>
+        </is>
+      </c>
+      <c r="O70" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="80" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>X8</t>
         </is>
       </c>
-      <c r="B61" s="24" t="inlineStr">
+      <c r="B71" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C61" s="19" t="inlineStr">
+      <c r="C71" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D61" s="20" t="inlineStr">
+      <c r="D71" s="20" t="inlineStr">
         <is>
           <t>แผนปกติกับแผนสหกิจศึกษาของ DSBA 2565 มีหน่วยกิตรวมตลอดหลักสูตรต่างกันไหม</t>
         </is>
       </c>
-      <c r="E61" s="20" t="inlineStr">
+      <c r="E71" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F61" s="20" t="inlineStr">
+      <c r="F71" s="20" t="inlineStr">
         <is>
           <t>ไม่ต่าง ทั้งสองแผนรวม 132 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G61" s="20" t="inlineStr">
-        <is>
-          <t>ไม่ต่างกัน แผนปกติและแผนสหกิจศึกษาของหลักสูตรวิทยาศาสตรบัณฑิต สาขาวิชาวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ หลักสูตรปรับปรุง พ.ศ. 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากัน คือ 132 หน่วยกิต [7]</t>
-        </is>
-      </c>
-      <c r="H61" s="20" t="inlineStr">
+      <c r="G71" s="20" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบแผนการศึกษา DSBA 2565 (ปริญญาตรี): แผนปกติ (3.1.4.1) กับแผนที่เข้าโครงการสหกิจศึกษา (3.1.4.2)
+- ปีที่ 1 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 1 ภาคการศึกษาที่ 2: แผนปกติ 21 หน่วยกิต · แผนสหกิจ 21 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 2: แผนปกติ 21 หน่วยกิต · แผนสหกิจ 21 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 2: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 4 ภาคการศึกษาที่ 1: แผนปกติ 9 หน่วยกิต · แผนสหกิจ 12 หน่วยกิต  ← ต่างกัน
+- ปีที่ 4 ภาคการศึกษาที่ 2: แผนปกติ 9 หน่วยกิต · แผนสหกิจ 6 หน่วยกิต  ← ต่างกัน
+รวมตลอดหลักสูตร: แผนปกติ 132 หน่วยกิต · แผนสหกิจ 132 หน่วยกิต (เท่ากัน)
+ภาคที่ต่างกัน: ปี 4 ภาค 1, ปี 4 ภาค 2
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 29):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 2 ช่อง
+      • วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 1
+      • วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 36):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 29):
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36):
+  - 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  - 06026260 สหกิจศึกษาต่างประเทศทางวิทยาการข้อมูลและการ วิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต
+ตามโครงสร้างหลักสูตร: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6)</t>
+        </is>
+      </c>
+      <c r="H71" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 15, 36
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 351, 30, 349, 23)</t>
-        </is>
-      </c>
-      <c r="I61" s="20" t="inlineStr">
-        <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
-        </is>
-      </c>
-      <c r="J61" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="K61" s="15" t="inlineStr">
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29, 36)</t>
+        </is>
+      </c>
+      <c r="I71" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J71" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K71" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L61" s="18" t="inlineStr">
+      <c r="L71" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M61" s="20" t="inlineStr">
-        <is>
-          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
-        </is>
-      </c>
-      <c r="N61" s="19" t="inlineStr">
-        <is>
-          <t>2.31s</t>
-        </is>
-      </c>
-      <c r="O61" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="80" customHeight="1">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="M71" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ตอบเป็นตารางเทียบหน่วยกิตรายภาคของสองแผน รวมทั้งหลักสูตรเท่ากัน 132</t>
+        </is>
+      </c>
+      <c r="N71" s="19" t="inlineStr">
+        <is>
+          <t>0.21s</t>
+        </is>
+      </c>
+      <c r="O71" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="80" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="B62" s="24" t="inlineStr">
+      <c r="B72" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C62" s="15" t="inlineStr">
+      <c r="C72" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D72" s="16" t="inlineStr">
         <is>
           <t>หลักสูตร AIT 2566 กับ IT 2565 ต้องเรียนหน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr">
+      <c r="E72" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="F72" s="16" t="inlineStr">
         <is>
           <t>AIT 2566 = 120, IT 2565 = 129 ต่างกัน 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G62" s="16" t="inlineStr">
+      <c r="G72" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
@@ -6559,78 +7617,78 @@
 สรุป: IT 2565 มากกว่า AIT 2566 อยู่ 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H62" s="16" t="inlineStr">
+      <c r="H72" s="16" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 5; IT2565 หน้า 6/20
 (หน้าที่ระบบคืนมา: IT 2565 หน้า 369, 378, 371; AIT 2566 หน้า 78)</t>
         </is>
       </c>
-      <c r="I62" s="16" t="inlineStr">
+      <c r="I72" s="16" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J62" s="15" t="n">
+      <c r="J72" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K62" s="15" t="inlineStr">
+      <c r="K72" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L62" s="18" t="inlineStr">
+      <c r="L72" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M62" s="16" t="inlineStr">
+      <c r="M72" s="16" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N62" s="15" t="inlineStr">
-        <is>
-          <t>0.46s</t>
-        </is>
-      </c>
-      <c r="O62" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="80" customHeight="1">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="N72" s="15" t="inlineStr">
+        <is>
+          <t>0.43s</t>
+        </is>
+      </c>
+      <c r="O72" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="80" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="B63" s="24" t="inlineStr">
+      <c r="B73" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C63" s="19" t="inlineStr">
+      <c r="C73" s="19" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="D63" s="20" t="inlineStr">
+      <c r="D73" s="20" t="inlineStr">
         <is>
           <t>BIT 2565 กับ DSBA 2560 หลักสูตรไหนต้องเรียนหน่วยกิตรวมมากกว่ากัน</t>
         </is>
       </c>
-      <c r="E63" s="20" t="inlineStr">
+      <c r="E73" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F63" s="20" t="inlineStr">
+      <c r="F73" s="20" t="inlineStr">
         <is>
           <t>เท่ากัน ทั้งคู่ 126 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G63" s="20" t="inlineStr">
+      <c r="G73" s="20" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
@@ -6638,619 +7696,654 @@
 สรุป: เท่ากัน (126 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H63" s="20" t="inlineStr">
+      <c r="H73" s="20" t="inlineStr">
         <is>
           <t>BIT2565 หน้า 6; DSBA2560 หน้า 17
 (หน้าที่ระบบคืนมา: BIT 2565 หน้า 266, 264, 267, 265)</t>
         </is>
       </c>
-      <c r="I63" s="20" t="inlineStr">
+      <c r="I73" s="20" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J63" s="19" t="n">
+      <c r="J73" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K63" s="15" t="inlineStr">
+      <c r="K73" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L63" s="18" t="inlineStr">
+      <c r="L73" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M63" s="20" t="inlineStr">
+      <c r="M73" s="20" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N63" s="19" t="inlineStr">
-        <is>
-          <t>0.11s</t>
-        </is>
-      </c>
-      <c r="O63" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="80" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="N73" s="19" t="inlineStr">
+        <is>
+          <t>0.17s</t>
+        </is>
+      </c>
+      <c r="O73" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="80" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="B64" s="24" t="inlineStr">
+      <c r="B74" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
         <is>
           <t>วิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
         </is>
       </c>
-      <c r="E64" s="16" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F64" s="16" t="inlineStr">
+      <c r="F74" s="16" t="inlineStr">
         <is>
           <t>ต้องผ่าน 06066001 ความน่าจะเป็นและสถิติ ซึ่งไม่มีวิชาบังคับก่อน (ชั้นเดียว)</t>
         </is>
       </c>
-      <c r="G64" s="16" t="inlineStr">
+      <c r="G74" s="16" t="inlineStr">
         <is>
           <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   ต้องผ่านวิชาบังคับก่อน:
     • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
         </is>
       </c>
-      <c r="H64" s="16" t="inlineStr">
+      <c r="H74" s="16" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 289, 291
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 37, 291, 19, 20)</t>
         </is>
       </c>
-      <c r="I64" s="16" t="inlineStr">
+      <c r="I74" s="16" t="inlineStr">
         <is>
           <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J64" s="15" t="n">
+      <c r="J74" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="K64" s="15" t="inlineStr">
+      <c r="K74" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L64" s="18" t="inlineStr">
+      <c r="L74" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M64" s="16" t="inlineStr">
+      <c r="M74" s="16" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N64" s="15" t="inlineStr">
-        <is>
-          <t>0.12s</t>
-        </is>
-      </c>
-      <c r="O64" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="80" customHeight="1">
-      <c r="A65" s="13" t="inlineStr">
+      <c r="N74" s="15" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O74" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="80" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="B65" s="24" t="inlineStr">
+      <c r="B75" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C65" s="19" t="inlineStr">
+      <c r="C75" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D65" s="20" t="inlineStr">
+      <c r="D75" s="20" t="inlineStr">
         <is>
           <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนอะไรแทนสหกิจศึกษา กี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E65" s="20" t="inlineStr">
+      <c r="E75" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F65" s="20" t="inlineStr">
+      <c r="F75" s="20" t="inlineStr">
         <is>
           <t>กลุ่มวิชาการศึกษาทางเลือก (กลุ่มวิชาเลือก) 6 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G65" s="20" t="inlineStr">
-        <is>
-          <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนวิชาเลือกเสรีจำนวนไม่น้อยกว่า 6 หน่วยกิต [4]</t>
-        </is>
-      </c>
-      <c r="H65" s="20" t="inlineStr">
+      <c r="G75" s="20" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบแผนการศึกษา DSBA 2565 (ปริญญาตรี): แผนปกติ (3.1.4.1) กับแผนที่เข้าโครงการสหกิจศึกษา (3.1.4.2)
+- ปีที่ 1 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 1 ภาคการศึกษาที่ 2: แผนปกติ 21 หน่วยกิต · แผนสหกิจ 21 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 2 ภาคการศึกษาที่ 2: แผนปกติ 21 หน่วยกิต · แผนสหกิจ 21 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 3 ภาคการศึกษาที่ 2: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
+- ปีที่ 4 ภาคการศึกษาที่ 1: แผนปกติ 9 หน่วยกิต · แผนสหกิจ 12 หน่วยกิต  ← ต่างกัน
+- ปีที่ 4 ภาคการศึกษาที่ 2: แผนปกติ 9 หน่วยกิต · แผนสหกิจ 6 หน่วยกิต  ← ต่างกัน
+รวมตลอดหลักสูตร: แผนปกติ 132 หน่วยกิต · แผนสหกิจ 132 หน่วยกิต (เท่ากัน)
+ภาคที่ต่างกัน: ปี 4 ภาค 1, ปี 4 ภาค 2
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 29):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 2 ช่อง
+      • วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 1
+      • วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 1 (หน้า 36):
+  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 — 3(0-9-0)
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 12 หน่วยกิต
+แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 29):
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต
+แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36):
+  - 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  - 06026260 สหกิจศึกษาต่างประเทศทางวิทยาการข้อมูลและการ วิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต
+ตามโครงสร้างหลักสูตร: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6)</t>
+        </is>
+      </c>
+      <c r="H75" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 15, 21-22
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 30, 23, 15, 22)</t>
-        </is>
-      </c>
-      <c r="I65" s="20" t="inlineStr">
-        <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
-        </is>
-      </c>
-      <c r="J65" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="K65" s="15" t="inlineStr">
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29, 36)</t>
+        </is>
+      </c>
+      <c r="I75" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J75" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K75" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L65" s="22" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
-        </is>
-      </c>
-      <c r="M65" s="20" t="inlineStr">
-        <is>
-          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2] 6 หน่วยกิตถูก แต่เรียกเป็น 'วิชาเลือกเสรี' ซึ่งเป็นคนละกลุ่ม (เล่มเรียกกลุ่มวิชาการศึกษาทางเลือก)</t>
-        </is>
-      </c>
-      <c r="N65" s="19" t="inlineStr">
-        <is>
-          <t>1.36s</t>
-        </is>
-      </c>
-      <c r="O65" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="80" customHeight="1">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="L75" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M75" s="20" t="inlineStr">
+        <is>
+          <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2] ตอบเป็นตารางเทียบสองแผนทั้งหมด ส่วนที่ถามอยู่ท้ายคำตอบ: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน)</t>
+        </is>
+      </c>
+      <c r="N75" s="19" t="inlineStr">
+        <is>
+          <t>0.06s</t>
+        </is>
+      </c>
+      <c r="O75" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="80" customHeight="1">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="B66" s="24" t="inlineStr">
+      <c r="B76" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C66" s="15" t="inlineStr">
+      <c r="C76" s="15" t="inlineStr">
         <is>
           <t>AITBA</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
+      <c r="D76" s="16" t="inlineStr">
         <is>
           <t>ปริญญาโท AITBA 2569 แผนวิชาชีพต้องเรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E66" s="16" t="inlineStr">
+      <c r="E76" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F66" s="16" t="inlineStr">
+      <c r="F76" s="16" t="inlineStr">
         <is>
           <t>36 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G66" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท หลักสูตร AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนรวมไม่น้อยกว่า 36 หน่วยกิต [3]</t>
-        </is>
-      </c>
-      <c r="H66" s="16" t="inlineStr">
+      <c r="G76" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนไม่น้อยกว่า 36 หน่วยกิต [3]</t>
+        </is>
+      </c>
+      <c r="H76" s="16" t="inlineStr">
         <is>
           <t>AITBA2569 หน้า 5
 (หน้าที่ระบบคืนมา: ปร.ด. AITBA 2569 หน้า 100, 5, 15, 228; วท.ม. AITBA 2569 หน้า 228, 21)</t>
         </is>
       </c>
-      <c r="I66" s="16" t="inlineStr">
+      <c r="I76" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J66" s="15" t="n">
+      <c r="J76" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="K66" s="15" t="inlineStr">
+      <c r="K76" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L66" s="18" t="inlineStr">
+      <c r="L76" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M66" s="16" t="inlineStr">
+      <c r="M76" s="16" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N66" s="15" t="inlineStr">
-        <is>
-          <t>1.30s</t>
-        </is>
-      </c>
-      <c r="O66" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="80" customHeight="1">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="N76" s="15" t="inlineStr">
+        <is>
+          <t>1.16s</t>
+        </is>
+      </c>
+      <c r="O76" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="80" customHeight="1">
+      <c r="A77" s="13" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
-      <c r="B67" s="24" t="inlineStr">
+      <c r="B77" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="C77" s="19" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D67" s="20" t="inlineStr">
+      <c r="D77" s="20" t="inlineStr">
         <is>
           <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E67" s="20" t="inlineStr">
+      <c r="E77" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F67" s="20" t="inlineStr">
+      <c r="F77" s="20" t="inlineStr">
         <is>
           <t>36 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G67" s="20" t="inlineStr">
+      <c r="G77" s="20" t="inlineStr">
         <is>
           <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนรวมทั้งหมด 36 หน่วยกิต [5]</t>
         </is>
       </c>
-      <c r="H67" s="20" t="inlineStr">
+      <c r="H77" s="20" t="inlineStr">
         <is>
           <t>IT2568 หน้า 5
 (หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 155, 25, 74, 18)</t>
         </is>
       </c>
-      <c r="I67" s="20" t="inlineStr">
+      <c r="I77" s="20" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J67" s="19" t="n">
+      <c r="J77" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K67" s="15" t="inlineStr">
+      <c r="K77" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L67" s="18" t="inlineStr">
+      <c r="L77" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M67" s="20" t="inlineStr">
+      <c r="M77" s="20" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N67" s="19" t="inlineStr">
-        <is>
-          <t>1.13s</t>
-        </is>
-      </c>
-      <c r="O67" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="80" customHeight="1">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="N77" s="19" t="inlineStr">
+        <is>
+          <t>1.11s</t>
+        </is>
+      </c>
+      <c r="O77" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="80" customHeight="1">
+      <c r="A78" s="13" t="inlineStr">
         <is>
           <t>Z1</t>
         </is>
       </c>
-      <c r="B68" s="24" t="inlineStr">
+      <c r="B78" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C78" s="15" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E68" s="16" t="inlineStr">
+      <c r="E78" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F68" s="16" t="inlineStr">
+      <c r="F78" s="16" t="inlineStr">
         <is>
           <t>75 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G68" s="16" t="inlineStr">
+      <c r="G78" s="16" t="inlineStr">
         <is>
           <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวม 75 หน่วยกิต [1]</t>
         </is>
       </c>
-      <c r="H68" s="16" t="inlineStr">
+      <c r="H78" s="16" t="inlineStr">
         <is>
           <t>IT2561 หน้า 16
 (หน้าที่ระบบคืนมา: ปร.ด. IT 2561 หน้า 16, 38, 22, 131)</t>
         </is>
       </c>
-      <c r="I68" s="16" t="inlineStr">
+      <c r="I78" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J68" s="15" t="n">
+      <c r="J78" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="K68" s="15" t="inlineStr">
+      <c r="K78" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L68" s="18" t="inlineStr">
+      <c r="L78" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M68" s="16" t="inlineStr">
+      <c r="M78" s="16" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N68" s="15" t="inlineStr">
-        <is>
-          <t>1.21s</t>
-        </is>
-      </c>
-      <c r="O68" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="80" customHeight="1">
-      <c r="A69" s="13" t="inlineStr">
+      <c r="N78" s="15" t="inlineStr">
+        <is>
+          <t>1.27s</t>
+        </is>
+      </c>
+      <c r="O78" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="80" customHeight="1">
+      <c r="A79" s="13" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="B69" s="24" t="inlineStr">
+      <c r="B79" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C69" s="19" t="inlineStr">
+      <c r="C79" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D69" s="20" t="inlineStr">
+      <c r="D79" s="20" t="inlineStr">
         <is>
           <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E69" s="20" t="inlineStr">
+      <c r="E79" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F69" s="20" t="inlineStr">
+      <c r="F79" s="20" t="inlineStr">
         <is>
           <t>6 หน่วยกิต (สหกิจศึกษา 06026259 หรือ 06026260 ต่างประเทศ)</t>
         </is>
       </c>
-      <c r="G69" s="20" t="inlineStr">
-        <is>
-          <t>แผนสหกิจศึกษาของหลักสูตร DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 มีจำนวน 6 หน่วยกิต [1]</t>
-        </is>
-      </c>
-      <c r="H69" s="20" t="inlineStr">
+      <c r="G79" s="20" t="inlineStr">
+        <is>
+          <t>แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36):
+  - 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  - 06026260 สหกิจศึกษาต่างประเทศทางวิทยาการข้อมูลและการ วิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
+  รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H79" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 36
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36, 29, 350, 14)</t>
-        </is>
-      </c>
-      <c r="I69" s="20" t="inlineStr">
-        <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
-        </is>
-      </c>
-      <c r="J69" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="K69" s="15" t="inlineStr">
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36)</t>
+        </is>
+      </c>
+      <c r="I79" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J79" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K79" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L69" s="18" t="inlineStr">
+      <c r="L79" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M69" s="20" t="inlineStr">
+      <c r="M79" s="20" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N69" s="19" t="inlineStr">
-        <is>
-          <t>1.26s</t>
-        </is>
-      </c>
-      <c r="O69" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="80" customHeight="1">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="N79" s="19" t="inlineStr">
+        <is>
+          <t>0.17s</t>
+        </is>
+      </c>
+      <c r="O79" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="80" customHeight="1">
+      <c r="A80" s="13" t="inlineStr">
         <is>
           <t>Z3</t>
         </is>
       </c>
-      <c r="B70" s="24" t="inlineStr">
+      <c r="B80" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C70" s="15" t="inlineStr">
+      <c r="C80" s="15" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>แผนปกติของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนอะไร กี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E70" s="16" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F70" s="16" t="inlineStr">
+      <c r="F80" s="16" t="inlineStr">
         <is>
           <t>วิชาเลือกหมวดศึกษาทั่วไป 1 วิชา + วิชาเลือกเสรี 2 วิชา รวม 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G70" s="16" t="inlineStr">
-        <is>
-          <t>ปีที่ 4 ภาคการศึกษาที่ 2 ของแผนปกติหลักสูตร DSBA 2565 เรียนดังนี้:
-- รหัสวิชา: 9064xxxx  
-  ชื่อวิชา: วิชาเลือกหมวดวิชาศึกษาทั่วไป (ELECTIVE IN GENERAL EDUCATION)  
-  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
-- รหัสวิชา: xxxxxxxx  
-  ชื่อวิชา: วิชาเลือกเสรี 1 (FREE ELECTIVE COURSE 1)  
-  หน่วยกิต: 3 (3-0-6) หรือ 3 (2-2-5)  
-รวมทั้งหมด 6 หน่วยกิต [1]</t>
-        </is>
-      </c>
-      <c r="H70" s="16" t="inlineStr">
+      <c r="G80" s="16" t="inlineStr">
+        <is>
+          <t>แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 29):
+  - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
+      • วิชาเลือกหมวดวิชาศึกษาทั่วไป
+      • วิชาเลือกเสรี 1
+      • วิชาเลือกเสรี 2
+  รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="H80" s="16" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 29
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36, 14, 29)</t>
-        </is>
-      </c>
-      <c r="I70" s="16" t="inlineStr">
-        <is>
-          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
-        </is>
-      </c>
-      <c r="J70" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="K70" s="15" t="inlineStr">
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29)</t>
+        </is>
+      </c>
+      <c r="I80" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J80" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L70" s="22" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
-        </is>
-      </c>
-      <c r="M70" s="16" t="inlineStr">
-        <is>
-          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)] ได้วิชาเลือกศึกษาทั่วไป + เลือกเสรี 1 รวม 6 หน่วยกิต แต่ขาดเลือกเสรี 2 (เล่มรวม 9 หน่วยกิต)</t>
-        </is>
-      </c>
-      <c r="N70" s="15" t="inlineStr">
-        <is>
-          <t>3.89s</t>
-        </is>
-      </c>
-      <c r="O70" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="80" customHeight="1">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M80" s="16" t="inlineStr">
+        <is>
+          <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)] ตอบ 3 ช่อง (วิชาเลือกศึกษาทั่วไป 1 + เลือกเสรี 2) รวม 9 หน่วยกิต ตรงเฉลย</t>
+        </is>
+      </c>
+      <c r="N80" s="15" t="inlineStr">
+        <is>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="O80" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="80" customHeight="1">
+      <c r="A81" s="13" t="inlineStr">
         <is>
           <t>Z4</t>
         </is>
       </c>
-      <c r="B71" s="24" t="inlineStr">
+      <c r="B81" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C71" s="19" t="inlineStr">
+      <c r="C81" s="19" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="D71" s="20" t="inlineStr">
+      <c r="D81" s="20" t="inlineStr">
         <is>
           <t>BIT 2565 กับ IT 2565 หน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E71" s="20" t="inlineStr">
+      <c r="E81" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F71" s="20" t="inlineStr">
+      <c r="F81" s="20" t="inlineStr">
         <is>
           <t>BIT 2565 = 126, IT 2565 = 129 ต่างกัน 3 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G71" s="20" t="inlineStr">
+      <c r="G81" s="20" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
@@ -7258,201 +8351,201 @@
 สรุป: IT 2565 มากกว่า BIT 2565 อยู่ 3 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H71" s="20" t="inlineStr">
+      <c r="H81" s="20" t="inlineStr">
         <is>
           <t>BIT2565 หน้า 6; IT2565 หน้า 6
 (หน้าที่ระบบคืนมา: BIT 2565 หน้า 264, 266, 7)</t>
         </is>
       </c>
-      <c r="I71" s="20" t="inlineStr">
+      <c r="I81" s="20" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J71" s="19" t="n">
+      <c r="J81" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K71" s="15" t="inlineStr">
+      <c r="K81" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L71" s="18" t="inlineStr">
+      <c r="L81" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M71" s="20" t="inlineStr">
+      <c r="M81" s="20" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N71" s="19" t="inlineStr">
-        <is>
-          <t>0.39s</t>
-        </is>
-      </c>
-      <c r="O71" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="80" customHeight="1">
-      <c r="A72" s="13" t="inlineStr">
+      <c r="N81" s="19" t="inlineStr">
+        <is>
+          <t>0.30s</t>
+        </is>
+      </c>
+      <c r="O81" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="80" customHeight="1">
+      <c r="A82" s="13" t="inlineStr">
         <is>
           <t>Z5</t>
         </is>
       </c>
-      <c r="B72" s="24" t="inlineStr">
+      <c r="B82" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C72" s="15" t="inlineStr">
+      <c r="C82" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D72" s="16" t="inlineStr">
+      <c r="D82" s="16" t="inlineStr">
         <is>
           <t>วิชาพื้นฐานวิทยาการข้อมูลของ AIT ต้องผ่านวิชาอะไรมาก่อน</t>
         </is>
       </c>
-      <c r="E72" s="16" t="inlineStr">
+      <c r="E82" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F72" s="16" t="inlineStr">
+      <c r="F82" s="16" t="inlineStr">
         <is>
           <t>ไม่มีวิชาบังคับก่อน</t>
         </is>
       </c>
-      <c r="G72" s="16" t="inlineStr">
+      <c r="G82" s="16" t="inlineStr">
         <is>
           <t>วิชา 06046407 พื้นฐานวิทยาการข้อมูล (FUNDAMENTALS OF DATA SCIENCE) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
   ไม่มีวิชาบังคับก่อน (PREREQUISITE: None)</t>
         </is>
       </c>
-      <c r="H72" s="16" t="inlineStr">
+      <c r="H82" s="16" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 292
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 20, 24, 38, 292)</t>
         </is>
       </c>
-      <c r="I72" s="16" t="inlineStr">
+      <c r="I82" s="16" t="inlineStr">
         <is>
           <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J72" s="15" t="n">
+      <c r="J82" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K72" s="15" t="inlineStr">
+      <c r="K82" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L72" s="18" t="inlineStr">
+      <c r="L82" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M72" s="16" t="inlineStr">
+      <c r="M82" s="16" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N72" s="15" t="inlineStr">
-        <is>
-          <t>0.12s</t>
-        </is>
-      </c>
-      <c r="O72" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="80" customHeight="1">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="N82" s="15" t="inlineStr">
+        <is>
+          <t>0.18s</t>
+        </is>
+      </c>
+      <c r="O82" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="80" customHeight="1">
+      <c r="A83" s="13" t="inlineStr">
         <is>
           <t>Z6</t>
         </is>
       </c>
-      <c r="B73" s="24" t="inlineStr">
+      <c r="B83" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C73" s="19" t="inlineStr">
+      <c r="C83" s="19" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D73" s="20" t="inlineStr">
+      <c r="D83" s="20" t="inlineStr">
         <is>
           <t>ปริญญาโท IT 2568 แผนวิชาชีพ ต้องเรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E73" s="20" t="inlineStr">
+      <c r="E83" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F73" s="20" t="inlineStr">
+      <c r="F83" s="20" t="inlineStr">
         <is>
           <t>36 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G73" s="20" t="inlineStr">
-        <is>
-          <t>ปริญญาโท IT 2568 แผนวิชาชีพต้องเรียนทั้งหมด 36 หน่วยกิต [2]</t>
-        </is>
-      </c>
-      <c r="H73" s="20" t="inlineStr">
+      <c r="G83" s="20" t="inlineStr">
+        <is>
+          <t>ปริญญาโท IT 2568 แผนวิชาชีพต้องเรียนรวมทั้งหมด 36 หน่วยกิต [2]</t>
+        </is>
+      </c>
+      <c r="H83" s="20" t="inlineStr">
         <is>
           <t>IT2568 หน้า 5
 (หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 25, 12, 156, 14)</t>
         </is>
       </c>
-      <c r="I73" s="20" t="inlineStr">
+      <c r="I83" s="20" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J73" s="19" t="n">
+      <c r="J83" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="K73" s="15" t="inlineStr">
+      <c r="K83" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L73" s="18" t="inlineStr">
+      <c r="L83" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M73" s="20" t="inlineStr">
+      <c r="M83" s="20" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N73" s="19" t="inlineStr">
-        <is>
-          <t>1.02s</t>
-        </is>
-      </c>
-      <c r="O73" s="18" t="inlineStr">
+      <c r="N83" s="19" t="inlineStr">
+        <is>
+          <t>1.17s</t>
+        </is>
+      </c>
+      <c r="O83" s="18" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O73"/>
+  <autoFilter ref="A1:O83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7514,12 +8607,12 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>C1: ถูกบางส่วน; C2: ถูกครบ; C3: ผิด</t>
+          <t>C1: ถูกบางส่วน; C2: ถูกครบ; C3: ถูกครบ</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>C1: หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย และมีประโยค 'ลดหน่วยกิตกลุ่มวิชาเฉพาะด้านจาก 46 เป็น 57' ที่ขัดกันเอง (ตัวเลขย่อยมาจาก LLM ยังไม่ได้ยืนยันกับเล่ม) · C2: พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง และระบุระดับที่ตรวจพบจากเนื้อหา (master ทั้งคู่) ตามที่ฐานข้อมูลเก็บ · C3: ตอบว่าแผนสหกิจต่างที่ปี 3 ภาค 3 แต่เล่ม (DSBA 2565 หน้า 36) วางสหกิจศึกษา 06026259/06026260 ไว้ที่ปี 4 ภาค 2 หมายเหตุ: เฉลยในไฟล์ทดสอบใช้รหัส 06026245 ซึ่งไม่ตรงกับเล่ม และแผนปกติปี 4 ภาค 2 ในเล่ม (หน้า 29) คือวิชาเลือกศึกษาทั่วไป + เลือกเสรี 2 วิชา รวม 9 หน่วยกิต ไม่ใช่โครงงาน 2</t>
+          <t>C1: หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่ามี 3 แขนง) ตัวเลขย่อยรอบนี้ (เฉพาะด้าน 94→93, บังคับเฉพาะแขนง 30→15, เลือก IT 6→9) ตรงกับโครงสร้างในเล่ม ข้อนี้ผ่าน LLM ตัวเลขย่อยเปลี่ยนทุกรอบ (รอบก่อนมีประโยคที่ขัดกันเอง) · C2: พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง และระบุระดับที่ตรวจพบจากเนื้อหา (master ทั้งคู่) ตามที่ฐานข้อมูลเก็บ · C3: ตอบจากตารางแผนทั้งสองชุดในเล่ม (3.1.4.1 หน้า 23-29 และ 3.1.4.2 หน้า 30-36): ต่างกันที่ปี 4 ภาค 1 (ปกติ 9 / สหกิจ 12) และปี 4 ภาค 2 (ปกติ 9 / สหกิจศึกษา 06026259 6 หน่วยกิต) รวม 132 เท่ากัน ตรวจกับเล่มแล้ว หมายเหตุ: เฉลยในไฟล์ทดสอบเขียนว่าแผนปกติลงโครงงาน 2 ในปี 4 ภาค 2 และใช้รหัสสหกิจ 06026245 ซึ่งไม่ตรงเล่ม (โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน, รหัสสหกิจคือ 06026259/06026260)</t>
         </is>
       </c>
     </row>
@@ -7536,7 +8629,7 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>ระดับยาก 7 ข้อ เฉลี่ย 1.78s ช้าสุด 3.90s · ทั้ง 28 ข้อ ต่ำกว่า 5s 26/28</t>
+          <t>ระดับยาก 7 ข้อ เฉลี่ย 1.60s ช้าสุด 4.86s · ทั้ง 28 ข้อ ต่ำกว่า 5s 27/28</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">

</xml_diff>

<commit_message>
test: record 92 questions after tester-feedback fixes; course answers cite table pages too
- tester: 92 questions re-recorded (adds T1-T10 from tester comments); E16 and
  H15 now fully correct, T10 partial; all LLM-path answers re-reviewed
- course answers: cite the course-list and description pages for the code in
  addition to the plan/group pages (qa_eval recall had dropped to 0.46)
- qa_eval: citation precision 0.60, recall 0.50, retrieval hit 17/19
- README: tester-feedback section, results tables, limitations
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenge Criteria (Measured)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Test Cases &amp; Results'!$A$1:$O$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,14 +76,8 @@
       <color rgb="00B45309"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00B91C1C"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -144,12 +138,6 @@
         <bgColor rgb="00FAF5FF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-        <bgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -177,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,9 +227,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -612,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -695,7 +680,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>28 ข้อชุดหลัก (E1–E9, M1–M9, H1–H7, C1–C3) + 34 ข้อชุดเพิ่มระดับง่าย/ปานกลาง/ยาก (E10–H15) + 20 ข้อท้าทายเพิ่มเติม (X1–Z6) = 82 ข้อ</t>
+          <t>28 ข้อชุดหลัก (E1–E9, M1–M9, H1–H7, C1–C3) + 44 ข้อชุดเพิ่ม (ระดับง่าย/ปานกลาง/ยาก E10–H15, ชุดใหม่ W1–W10 และชุดจาก tester T1–T10) + 20 ข้อท้าทายเพิ่มเติม (X1–Z6) = 92 ข้อ</t>
         </is>
       </c>
     </row>
@@ -731,7 +716,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>เฉลี่ย 0.92s · เร็วสุด 0.05s · ช้าสุด 9.03s · ต่ำกว่า 5s 27/28 ข้อ</t>
+          <t>เฉลี่ย 0.86s · เร็วสุด 0.06s · ช้าสุด 7.52s · ต่ำกว่า 5s 26/28 ข้อ</t>
         </is>
       </c>
     </row>
@@ -819,12 +804,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>0.73</t>
         </is>
       </c>
     </row>
@@ -851,12 +836,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>0.60</t>
         </is>
       </c>
     </row>
@@ -883,12 +868,12 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>5.40</t>
         </is>
       </c>
     </row>
@@ -915,12 +900,12 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>3.17</t>
+          <t>2.66</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>9.03</t>
+          <t>7.52</t>
         </is>
       </c>
     </row>
@@ -947,12 +932,12 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>0.92</t>
+          <t>0.86</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>9.03</t>
+          <t>7.52</t>
         </is>
       </c>
     </row>
@@ -971,22 +956,22 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>0.38</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.75</t>
         </is>
       </c>
     </row>
@@ -1015,12 +1000,12 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>0.36</t>
+          <t>0.37</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.90</t>
         </is>
       </c>
     </row>
@@ -1039,13 +1024,13 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
@@ -1054,7 +1039,7 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.34</t>
         </is>
       </c>
     </row>
@@ -1083,23 +1068,23 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.09</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>0.36</t>
+          <t>0.16</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>ท้าทายเพิ่มเติม ชุด X</t>
+          <t>ชุดจาก tester T1–T10 (ถามวิชาด้วยชื่อ/แขนง/อาจารย์)</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
@@ -1107,7 +1092,7 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>1</v>
@@ -1117,23 +1102,23 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>2.42</t>
+          <t>0.22</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>12.81</t>
+          <t>1.37</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>ท้าทายเพิ่มเติม ชุด Y</t>
+          <t>ท้าทายเพิ่มเติม ชุด X</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
@@ -1141,29 +1126,29 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>0.51</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>10.78</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>ท้าทายเพิ่มเติม ชุด Z</t>
+          <t>ท้าทายเพิ่มเติม ชุด Y</t>
         </is>
       </c>
       <c r="B27" s="8" t="n">
@@ -1195,125 +1180,166 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>ท้าทายเพิ่มเติม ชุด Z</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>รวมทั้งหมด</t>
         </is>
       </c>
-      <c r="B28" s="10" t="n">
-        <v>82</v>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
+      <c r="B29" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D28" s="10" t="n">
-        <v>74</v>
-      </c>
-      <c r="E28" s="10" t="n">
+      <c r="D29" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="E29" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="F28" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="10" t="inlineStr">
-        <is>
-          <t>0.74</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>12.81</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="F29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>0.61</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>10.78</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>ข้อควรทราบเมื่ออ่านผล</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>1) 'ตรวจคำสำคัญ' ผ่านง่าย (เช่น E2 ตรวจแค่มีเลข 3) จึงไม่ควรใช้เป็นอัตราความถูกต้อง ให้ดูคอลัมน์ 'ตรวจโดยคน'</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>2) ผลตรวจโดยคนอ่านเทียบเฉลยในไฟล์นี้ ไม่ได้เทียบกับ PDF ต้นฉบับโดยตรง และผูกกับคำตอบรอบที่ตรวจ (คำถามเชิงเหตุผลเรียก LLM คำตอบเปลี่ยนได้ทุกรอบ)</t>
+          <t>1) 'ตรวจคำสำคัญ' ผ่านง่าย (เช่น E2 ตรวจแค่มีเลข 3) จึงไม่ควรใช้เป็นอัตราความถูกต้อง ให้ดูคอลัมน์ 'ตรวจโดยคน'</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>3) ความถูกต้องของ citation ไม่ได้ตรวจรายข้อในไฟล์นี้ วัดแยกด้วย python -m katrag.eval.qa_eval (19 ข้อ): precision 0.57, recall 0.53</t>
+          <t>2) ผลตรวจโดยคนอ่านเทียบเฉลยในไฟล์นี้ ไม่ได้เทียบกับ PDF ต้นฉบับโดยตรง และผูกกับคำตอบรอบที่ตรวจ (คำถามเชิงเหตุผลเรียก LLM คำตอบเปลี่ยนได้ทุกรอบ)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
+          <t>3) ความถูกต้องของ citation ไม่ได้ตรวจรายข้อในไฟล์นี้ วัดแยกด้วย python -m katrag.eval.qa_eval (19 ข้อ): precision 0.57, recall 0.53</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
+          <t>4) คำตอบสำเร็จรูปที่เคยเขียนไว้ในโค้ดสำหรับ M8, H5, C1, C3 ถูกถอดออกแล้ว ผลในไฟล์นี้มาจาก pipeline จริง (ฐานข้อมูล / retrieval + LLM)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (X1–X8, Y1–Y6, Z1–Z6) ต่อท้ายในแผ่น All Test Cases: เขียนคำถามและเฉลยจากเล่มก่อนรัน รายงานทุกข้อที่ลอง ผลบันทึกจากรอบวันที่ 2026-10-05 (docs/challenge_extended.json) ชุด X ใช้ออกแบบการแก้ระบบ ชุด Y/Z เขียนไว้ก่อนแก้แต่ละรอบ (held-out)</t>
+          <t>4.1) ข้อที่เรียก LLM ตอบไม่เหมือนเดิมทุกรอบ (เช่น M8, H2) ผลตรวจโดยคนผูกกับคำตอบของรอบที่ตรวจ</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>4.3) ชุดเพิ่มระดับง่าย/ปานกลาง/ยาก 24 ข้อ (E10–E17, M10–M17, H8–H15, docs/extra_levels.json): เขียนคำถามแล้วตรวจเฉลยจากเล่มหลังรัน รอบแรกได้ ถูก 14 · ไม่ตรงประเด็น 4 · ผิด 6 จึงแก้ระบบแล้วรันซ้ำ ผลในไฟล์นี้คือรอบหลังแก้ ชุดนี้ใช้นำการแก้ ไม่ใช่ชุด held-out ข้อ H15 (วิชาเลือกตามแขนง) ยังไม่ได้แก้</t>
+          <t>4.2) ข้อท้าทายเพิ่มเติม 20 ข้อ (X1–X8, Y1–Y6, Z1–Z6) ต่อท้ายในแผ่น All Test Cases: เขียนคำถามและเฉลยจากเล่มก่อนรัน รายงานทุกข้อที่ลอง ผลบันทึกจากรอบวันที่ 2026-10-05 (docs/challenge_extended.json) ชุด X ใช้ออกแบบการแก้ระบบ ชุด Y/Z เขียนไว้ก่อนแก้แต่ละรอบ (held-out)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>4.4) การแก้รอบหลัง (ตารางโครงสร้างหน่วยกิตรายหมวด + อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) แล้วรันซ้ำทั้งหมด: ข้อที่ตอบจาก SQL ได้คำตอบเดิม ข้อที่ผ่าน LLM ตอบเปลี่ยนจึงตรวจใหม่ M8 และ H5 ตอนนี้ตอบจากตาราง rule (M8 เป็น ถูกครบ ตอบคงที่) C3 ตอบจากตารางแผนสหกิจ (ถูกครบ ตรวจกับเล่ม: เฉลยเดิมของ C3 คลาดเคลื่อน โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน) ข้อ X4, X8, Y4, Z3, H11 เปลี่ยนเป็น ถูกครบ ส่วน X7 ถูกครบ/X5 ถูกบางส่วน เป็นผลของ LLM ที่เปลี่ยนไปตามรอบ</t>
+          <t>4.3) ชุดเพิ่มระดับง่าย/ปานกลาง/ยาก 24 ข้อ (E10–E17, M10–M17, H8–H15, docs/extra_levels.json): เขียนคำถามแล้วตรวจเฉลยจากเล่มหลังรัน รอบแรกได้ ถูก 14 · ไม่ตรงประเด็น 4 · ผิด 6 จึงแก้ระบบแล้วรันซ้ำ ผลในไฟล์นี้คือรอบหลังแก้ ชุดนี้ใช้นำการแก้ ไม่ใช่ชุด held-out ข้อ H15 (วิชาเลือกตามแขนง) ยังไม่ได้แก้</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>4.5) ชุดใหม่ W1–W10 (โครงสร้างหน่วยกิตรายหมวด + แผนสหกิจ) เขียนคำถามและเฉลยจากเล่มก่อนรัน รอบแรกได้ ถูกครบ 8 · บางส่วน 2 (W9 ระบุภาคที่ต่างเกินจริงเพราะเรียงแถวต่างกัน, W10 ตารางขาดปี 3 ภาค 2) แก้แบบทั่วไป (ไม่เขียนตอบเฉพาะข้อ) แล้วรันซ้ำ ผลในไฟล์คือรอบหลังแก้ จึงไม่ใช่ชุดที่ซ่อนไว้วัดอย่างสะอาด</t>
+          <t>4.4) การแก้รอบหลัง (ตารางโครงสร้างหน่วยกิตรายหมวด + อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) แล้วรันซ้ำทั้งหมด: ข้อที่ตอบจาก SQL ได้คำตอบเดิม ข้อที่ผ่าน LLM ตอบเปลี่ยนจึงตรวจใหม่ M8 และ H5 ตอนนี้ตอบจากตาราง rule (M8 เป็น ถูกครบ ตอบคงที่) C3 ตอบจากตารางแผนสหกิจ (ถูกครบ ตรวจกับเล่ม: เฉลยเดิมของ C3 คลาดเคลื่อน โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน) ข้อ X4, X8, Y4, Z3, H11 เปลี่ยนเป็น ถูกครบ ส่วน X7 ถูกครบ/X5 ถูกบางส่วน เป็นผลของ LLM ที่เปลี่ยนไปตามรอบ</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+          <t>4.5) ชุดใหม่ W1–W10 (โครงสร้างหน่วยกิตรายหมวด + แผนสหกิจ) เขียนคำถามและเฉลยจากเล่มก่อนรัน รอบแรกได้ ถูกครบ 8 · บางส่วน 2 (W9 ระบุภาคที่ต่างเกินจริงเพราะเรียงแถวต่างกัน, W10 ตารางขาดปี 3 ภาค 2) แก้แบบทั่วไป (ไม่เขียนตอบเฉพาะข้อ) แล้วรันซ้ำ ผลในไฟล์คือรอบหลังแก้ จึงไม่ใช่ชุดที่ซ่อนไว้วัดอย่างสะอาด</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
+          <t>4.6) ชุด T1–T10 เขียนจาก comment ของผู้ทดสอบ (วิชาที่ถามด้วยชื่อ/แขนง/โมดูล/อาจารย์/เลขประจำตัว) เฉลยจากเล่ม ใช้เป็นแนวทางแก้ระบบ จึงไม่ใช่ชุดซ่อนวัด หลังแก้ ข้อ H15, E16 ถูกครบ และ T10 ถูกบางส่วน (ตอบเฉพาะวุฒิปริญญาตรี) รันซ้ำทั้งหมด 92 ข้อ ไม่พบเลขประจำตัวประชาชนหรืออักษรจีนในคำตอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>5) คอลัมน์ 'เส้นทางประมวลผล' ได้จากการ trace โค้ด pipeline (นับว่ามีการเรียก LLM หรือไม่) ไม่ใช่ข้อมูลที่ API ส่งกลับมา</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
           <t>6) เฉลยข้อ H4 เดิมเขียน 48 วิชา แต่ฐานข้อมูลปัจจุบันให้ 52 (DSBA 2560 71 ชื่อ / 2565 75 ชื่อ) ผลของระบบตรงกับฐานข้อมูล</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="B6:H6"/>
@@ -1324,15 +1350,16 @@
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A33:H33"/>
     <mergeCell ref="B11:H11"/>
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="A35:H35"/>
     <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="B10:H10"/>
-    <mergeCell ref="A31:H31"/>
     <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1345,7 +1372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1526,7 +1553,7 @@
       </c>
       <c r="N2" s="15" t="inlineStr">
         <is>
-          <t>0.07s</t>
+          <t>0.73s</t>
         </is>
       </c>
       <c r="O2" s="18" t="inlineStr">
@@ -1568,27 +1595,26 @@
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>วิชาที่เกี่ยวข้องกับ "แคลคูลัส 2" — หลักสูตร DSBA
-■ DSBA 2565 — 2 วิชา รวม 6 หน่วยกิต
-  - 06026200 แคลคูลัส 1 (CALCULUS 1)
-      หน่วยกิต 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1
-  - 06026201 แคลคูลัส 2 (CALCULUS 2)
-      หน่วยกิต 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2</t>
+          <t>วิชา 06026201 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) หน่วยกิต · หลักสูตร DSBA 2565 (ปริญญาตรี)
+อยู่ในกลุ่มคณิตศาสตร์และสถิติ (ส่วนของกลุ่มวิชาแกน) (หน้า 17)
+เรียนตามแผนการศึกษา:
+  - ปีที่ 1 ภาคการศึกษาที่ 2 (ทั้งแผนปกติและแผนสหกิจ, หน้า 24, 31)
+วิชาบังคับก่อน: 06026200 แคลคูลัส 1</t>
         </is>
       </c>
       <c r="H3" s="20" t="inlineStr">
         <is>
           <t>ตารางรายวิชา DSBA 2565 (หน้า 12)
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 17, 68, 314, 353)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 17, 24, 31, 68)</t>
         </is>
       </c>
       <c r="I3" s="20" t="inlineStr">
         <is>
-          <t>ค้นวิชาด้วย bge-m3 → จัดรูปคำตอบเอง (ไม่ผ่าน LLM)</t>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J3" s="19" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K3" s="17" t="inlineStr">
         <is>
@@ -1602,12 +1628,12 @@
       </c>
       <c r="M3" s="20" t="inlineStr">
         <is>
-          <t>แคลคูลัส 2 = 3(3-0-6) ถูก แต่ตอบพ่วงแคลคูลัส 1 มาด้วย (ส่วนเกิน)</t>
+          <t>ตอบจากตารางรายวิชาและแผนในเล่ม: แคลคูลัส 2 = 3 หน่วยกิต ปี 1 ภาค 2 พร้อมวิชาบังคับก่อน</t>
         </is>
       </c>
       <c r="N3" s="19" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="O3" s="18" t="inlineStr">
@@ -1649,10 +1675,11 @@
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>วิชาที่เกี่ยวข้องกับ "การสร้างคลังข้อมูล" — หลักสูตร DSBA
-■ DSBA 2565 — 1 วิชา รวม 3 หน่วยกิต
-  - 06026212 การสร้างคลังข้อมูล (DATA WAREHOUSING)
-      หน่วยกิต 3(2-2-5) | ปีที่ 3 ภาคการศึกษาที่ 1</t>
+          <t>วิชา 06026212 การสร้างคลังข้อมูล (DATA WAREHOUSING) — 3(2-2-5) หน่วยกิต · หลักสูตร DSBA 2565 (ปริญญาตรี)
+อยู่ในกลุ่มพื้นฐานวิชาชีพ (หน้า 18)
+เรียนตามแผนการศึกษา:
+  - ปีที่ 3 ภาคการศึกษาที่ 1 (ทั้งแผนปกติและแผนสหกิจ, หน้า 27, 34)
+วิชาบังคับก่อน: 06066300 แนวคิดระบบฐานข้อมูล</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
@@ -1663,7 +1690,7 @@
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>ค้นวิชาด้วย bge-m3 → จัดรูปคำตอบเอง (ไม่ผ่าน LLM)</t>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J4" s="15" t="n">
@@ -1681,12 +1708,12 @@
       </c>
       <c r="M4" s="16" t="inlineStr">
         <is>
-          <t>ปีที่ 3 ภาคการศึกษาที่ 1 ตรงเฉลย</t>
+          <t>ตอบจากตารางแผนในเล่ม: การสร้างคลังข้อมูล ปี 3 ภาค 1 พร้อมวิชาบังคับก่อน</t>
         </is>
       </c>
       <c r="N4" s="15" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="O4" s="18" t="inlineStr">
@@ -1781,7 +1808,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.31s</t>
         </is>
       </c>
       <c r="O5" s="18" t="inlineStr">
@@ -1823,7 +1850,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>ระบบข้อมูลมหัต (Big Data Systems) [4]</t>
+          <t>ระบบข้อมูลมหัต (Big Data Systems)</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -1857,7 +1884,7 @@
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>1.16s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="O6" s="18" t="inlineStr">
@@ -1949,7 +1976,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O7" s="18" t="inlineStr">
@@ -2027,7 +2054,7 @@
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="O8" s="18" t="inlineStr">
@@ -2112,7 +2139,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.38s</t>
         </is>
       </c>
       <c r="O9" s="18" t="inlineStr">
@@ -2190,7 +2217,7 @@
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="O10" s="18" t="inlineStr">
@@ -2268,7 +2295,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.11s</t>
         </is>
       </c>
       <c r="O11" s="18" t="inlineStr">
@@ -2353,7 +2380,7 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.33s</t>
         </is>
       </c>
       <c r="O12" s="18" t="inlineStr">
@@ -2442,7 +2469,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>0.61s</t>
+          <t>0.60s</t>
         </is>
       </c>
       <c r="O13" s="18" t="inlineStr">
@@ -2533,7 +2560,7 @@
       </c>
       <c r="N14" s="15" t="inlineStr">
         <is>
-          <t>0.56s</t>
+          <t>0.50s</t>
         </is>
       </c>
       <c r="O14" s="18" t="inlineStr">
@@ -2638,7 +2665,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.32s</t>
         </is>
       </c>
       <c r="O15" s="18" t="inlineStr">
@@ -2733,7 +2760,7 @@
       </c>
       <c r="N16" s="15" t="inlineStr">
         <is>
-          <t>0.06s</t>
+          <t>0.11s</t>
         </is>
       </c>
       <c r="O16" s="18" t="inlineStr">
@@ -2818,7 +2845,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>0.06s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O17" s="18" t="inlineStr">
@@ -2914,7 +2941,7 @@
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>0.07s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O18" s="18" t="inlineStr">
@@ -2994,7 +3021,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.09s</t>
         </is>
       </c>
       <c r="O19" s="18" t="inlineStr">
@@ -3135,7 +3162,7 @@
       </c>
       <c r="N20" s="15" t="inlineStr">
         <is>
-          <t>0.06s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O20" s="18" t="inlineStr">
@@ -3178,7 +3205,7 @@
       <c r="G21" s="20" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถเรียนวิชาฐานข้อมูลในปีที่ 4 ได้ เนื่องจากหลักสูตร DSBA 2565 มีวิชาบังคับในปีที่ 4 ที่เกี่ยวข้องกับฐานข้อมูล เช่น 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 ซึ่งจัดสอนในภาคการศึกษาที่ 1 ปีที่ 4 โดยไม่มีวิชาบังคับก่อนกำหนดไว้ และมีอาจารย์ผู้สอนที่เชี่ยวชาญด้านฐานข้อมูล ได้แก่ รศ.ดร.ศุภมิตร จิตตะยโศธร ผู้มีงานวิจัยและภาระงานสอนด้านฐานข้อมูลระบบข้อมูลขั้นสูง</t>
+นักศึกษาสามารถเรียนวิชาที่เกี่ยวข้องกับฐานข้อมูลในปีที่ 4 ได้ เนื่องจากมีวิชาบังคับก่อนหน้า เช่น 06066300 แนวคิดระบบฐานข้อมูล (ปี 2 ภาค 1) และ 06026212 การสร้างคลังข้อมูล (ปี 3 ภาค 1) ซึ่งเป็นพื้นฐานสำคัญ รวมถึงมีวิชาเลือกในกลุ่มวิชาเฉพาะด้าน เช่น 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 ที่จัดสอนในปีที่ 4 ภาคการศึกษาที่ 1 โดยมีลักษณะเป็นวิชาเลือกเฉพาะแขนง 3 หน่วยกิต ประเภทวิชาเลือก ซึ่งสอดคล้องกับเนื้อหาด้านฐานข้อมูลและวิศวกรรมข้อมูล.</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -3207,17 +3234,17 @@
       </c>
       <c r="M21" s="20" t="inlineStr">
         <is>
-          <t>ตอบ 'ได้' ถูก ชี้ 06026246/06026247 (หัวข้อพิเศษทางวิศวกรรมข้อมูล) และภาค 1 ตรงเฉลย แต่เรียกว่า 'วิชาบังคับ' (เป็นวิชาเลือก) และอ้างอาจารย์ที่เชี่ยวชาญฐานข้อมูลโดยไม่มีหลักฐานรองรับ ข้อนี้ผ่าน LLM ตอบเปลี่ยนทุกรอบ (รอบก่อนระบุภาค 2 และ 6 หน่วยกิตผิด)</t>
+          <t>ตอบ 'ได้' ถูก และชี้ 06026246/06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1-2 (3 หน่วยกิต วิชาเลือก) ซึ่งตรงกับเล่มหน้า 21 แต่ระบุว่าเปิดสอนปี 4 ภาค 1 ทั้งที่เล่มไม่ได้กำหนดภาคของวิชาเลือกนี้ (เฉลยในไฟล์ทดสอบเรียก 06026246 ว่าระบบฐานข้อมูลแบบกระจาย แต่ในเล่มวิชานั้นคือ 06026245) ข้อนี้ผ่าน LLM ตอบเปลี่ยนทุกรอบ</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>4.86s</t>
-        </is>
-      </c>
-      <c r="O21" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>5.40s</t>
+        </is>
+      </c>
+      <c r="O21" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3282,7 @@
       <c r="G22" s="16" t="inlineStr">
         <is>
           <t>ไม่ได้  
-วิชา 06026212 การสร้างคลังข้อมูล เป็นวิชาบังคับที่ต้องเรียนในปีที่ 3 ภาคการศึกษาที่ 1 และมีข้อกำหนดให้ต้องผ่านวิชา 06066300 แนวคิดระบบฐานข้อมูล ซึ่งเป็นวิชาบังคับในปีที่ 2 ภาคการศึกษาที่ 1 ก่อนจึงจะสามารถลงทะเบียนได้</t>
+วิชา 06026212 การสร้างคลังข้อมูล เป็นวิชาบังคับในปีที่ 3 ภาคการศึกษาที่ 1 และมีข้อกำหนดให้ต้องผ่านวิชา 06066300 แนวคิดระบบฐานข้อมูล ซึ่งเป็นวิชาบังคับในปีที่ 2 ภาคการศึกษาที่ 1 ก่อนจึงจะสามารถลงทะเบียนได้</t>
         </is>
       </c>
       <c r="H22" s="16" t="inlineStr">
@@ -3289,7 +3316,7 @@
       </c>
       <c r="N22" s="15" t="inlineStr">
         <is>
-          <t>3.05s</t>
+          <t>2.01s</t>
         </is>
       </c>
       <c r="O22" s="18" t="inlineStr">
@@ -3447,7 +3474,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.24s</t>
         </is>
       </c>
       <c r="O23" s="18" t="inlineStr">
@@ -3543,7 +3570,7 @@
       </c>
       <c r="N24" s="15" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="O24" s="18" t="inlineStr">
@@ -3585,9 +3612,9 @@
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>ใช่ ปีที่ 3 ต้องเลือกแขนง (หรือที่เรียกว่า กลุ่มวิชา) ซึ่งมี 3 แขนงให้เลือก ได้แก่:
+          <t>หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ได้ โดยมีแขนงให้เลือก 3 แขนง ดังนี้:
 - วิทยาการข้อมูล (Data Science)  
-- การวิเคราะห์เชิงสถิติ (Statistical Analysis)  
+- การวิเคราะห์เชิงสถิติ (Statistical Analytics)  
 - วิศวกรรมข้อมูล (Data Engineering)  
 [3][4][6]</t>
         </is>
@@ -3623,7 +3650,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>2.46s</t>
+          <t>2.53s</t>
         </is>
       </c>
       <c r="O25" s="18" t="inlineStr">
@@ -3709,7 +3736,7 @@
       </c>
       <c r="N26" s="15" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.28s</t>
         </is>
       </c>
       <c r="O26" s="18" t="inlineStr">
@@ -3751,9 +3778,9 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือกแขนงวิชาเดิม
-2. หลักสูตร IT 2565 ปรับลดหน่วยกิตรวมจาก 130 เหลือ 129 หน่วยกิต โดยลดหน่วยกิตในกลุ่มวิชาเฉพาะด้านจาก 94 เป็น 93 หน่วยกิต และลดหน่วยกิตกลุ่มวิชาบังคับเฉพาะแขนงจาก 30 เป็น 15 หน่วยกิต พร้อมเพิ่มกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศเป็น 9 หน่วยกิต (จากเดิม 6 หน่วยกิต) ซึ่งจัดเป็น 3 โมดูลอาชีพ ได้แก่ Full-Stack Web Developer, Network/System Engineer และ Game Developer
-3. อ้างข้อมูลจาก: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18, IT 2565 หน้า 6), โครงสร้างหลักสูตร (มคอ.2 IT 2565 หน้า 371, 374, 376, 378), คำอธิบายการปรับโครงสร้าง (มคอ.2 IT 2565 หน้า 370) — ประเภทวิชา: บังคับ/เลือก, ภาค/ปีที่เปิดสอน: ปีการศึกษา 2560 (IT 2560), 2565 (IT 2565)</t>
+          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูล แทนการเลือก "แขนงวิชา" 3 แขนง
+2. หลักสูตร IT 2565 ลดหน่วยกิตรวมจาก 130 เหลือ 129 หน่วยกิต โดยปรับโครงสร้างหมวดวิชาเฉพาะให้กลุ่มวิชาเฉพาะด้านเพิ่มจาก 46 เป็น 57 หน่วยกิต และกลุ่มวิชาบังคับเฉพาะแขนง/โมดูลลดจาก 30 เหลือ 15 หน่วยกิต พร้อมเพิ่มกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศเป็น 9 หน่วยกิต (จากเดิม 6 หน่วยกิต) ตามการจัดกลุ่มเป็น 3 โมดูลอาชีพ: M1 (Full-Stack Web Developer), M2 (Network/System Engineer), M3 (Game Developer)
+3. อ้างข้อมูลจาก: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18, IT 2565 หน้า 6); โครงสร้างหลักสูตร (มคอ.2 IT 2565 หน้า 371, 374, 376, 378); คำอธิบายการปรับโครงสร้าง (มคอ.2 IT 2565 หน้า 370)</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">
@@ -3782,12 +3809,12 @@
       </c>
       <c r="M27" s="20" t="inlineStr">
         <is>
-          <t>หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่ามี 3 แขนง) ตัวเลขย่อยรอบนี้ (เฉพาะด้าน 94→93, บังคับเฉพาะแขนง 30→15, เลือก IT 6→9) ตรงกับโครงสร้างในเล่ม ข้อนี้ผ่าน LLM ตัวเลขย่อยเปลี่ยนทุกรอบ (รอบก่อนมีประโยคที่ขัดกันเอง)</t>
+          <t>หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา) ตัวเลขย่อยรอบนี้ตรงกับโครงสร้างในเล่ม (กลุ่มเฉพาะด้าน 46→57, บังคับเฉพาะแขนง 30→15, เลือก IT 6→9) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่ามี 3 แขนง) ข้อนี้ผ่าน LLM ตัวเลขย่อยเปลี่ยนทุกรอบ</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>9.03s</t>
+          <t>7.52s</t>
         </is>
       </c>
       <c r="O27" s="15" t="inlineStr">
@@ -3869,7 +3896,7 @@
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.33s</t>
         </is>
       </c>
       <c r="O28" s="18" t="inlineStr">
@@ -3979,7 +4006,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="O29" s="18" t="inlineStr">
@@ -4051,7 +4078,7 @@
       <c r="M30" s="16" t="inlineStr"/>
       <c r="N30" s="15" t="inlineStr">
         <is>
-          <t>0.59s</t>
+          <t>0.63s</t>
         </is>
       </c>
       <c r="O30" s="18" t="inlineStr">
@@ -4128,7 +4155,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O31" s="18" t="inlineStr">
@@ -4170,10 +4197,11 @@
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
-          <t>วิชาที่เกี่ยวข้องกับ "แคลคูลัส 1 รหัส อะไร" — หลักสูตร DSBA
-■ DSBA 2565 — 1 วิชา รวม 3 หน่วยกิต
-  - 06026200 แคลคูลัส 1 (CALCULUS 1)
-      หน่วยกิต 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+          <t>วิชา 06026200 แคลคูลัส 1 (CALCULUS 1) — 3(3-0-6) หน่วยกิต · หลักสูตร DSBA 2565 (ปริญญาตรี)
+อยู่ในกลุ่มคณิตศาสตร์และสถิติ (ส่วนของกลุ่มวิชาแกน) (หน้า 17)
+เรียนตามแผนการศึกษา:
+  - ปีที่ 1 ภาคการศึกษาที่ 1 (ทั้งแผนปกติและแผนสหกิจ, หน้า 23, 30)
+วิชาบังคับก่อน: ไม่มี</t>
         </is>
       </c>
       <c r="H32" s="16" t="inlineStr">
@@ -4184,7 +4212,7 @@
       </c>
       <c r="I32" s="16" t="inlineStr">
         <is>
-          <t>Semantic topic search (bge-m3) → จัดรูปคำตอบเอง (อาจใช้ Typhoon คัดรหัสวิชา)</t>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J32" s="15" t="n">
@@ -4200,10 +4228,14 @@
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M32" s="16" t="inlineStr"/>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>ตอบจากตารางแผนและหัวข้อรายวิชา พร้อมกลุ่มวิชาและวิชาบังคับก่อน</t>
+        </is>
+      </c>
       <c r="N32" s="15" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="O32" s="18" t="inlineStr">
@@ -4295,7 +4327,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.40s</t>
         </is>
       </c>
       <c r="O33" s="18" t="inlineStr">
@@ -4387,7 +4419,7 @@
       </c>
       <c r="N34" s="15" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="O34" s="18" t="inlineStr">
@@ -4468,7 +4500,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.43s</t>
         </is>
       </c>
       <c r="O35" s="18" t="inlineStr">
@@ -4510,54 +4542,43 @@
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>วิชาที่เกี่ยวข้องกับ "Computer Programming" — หลักสูตร AIT
-■ AIT 2566 — 6 วิชา รวม 17 หน่วยกิต
-  - 06066303 การแก้ปัญหาและการโปรแกรมคอมพิวเตอร์ (PROBLEM SOLVING AND COMPUTER PROGRAMMING)
-      หน่วยกิต 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 1
-  - 06046403 การโปรแกรมคอมพิวเตอร์ (COMPUTER PROGRAMMING)
-      หน่วยกิต 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 2
-  - 06046409 คอมพิวเตอร์วิทัศน์เบื้องต้น (INTRODUCTION TO COMPUTER VISION)
-      หน่วยกิต 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
-  - 06046416 การเรียนรู้เชิงลึกสำหรับคอมพิวเตอร์วิทัศน์ (DEEP LEARNING FOR COMPUTER VISION)
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 90642111 สนุกกับการเขียนโค้ด
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 90642118 โปรแกรมคอมพิวเตอร์ประยุกต์ทางธุรกิจ
-      หน่วยกิต 2(1-2-3) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)</t>
+          <t>วิชา 06046403 การโปรแกรมคอมพิวเตอร์ (COMPUTER PROGRAMMING) — 3(2-2-5) หน่วยกิต · หลักสูตร AIT 2566 (ปริญญาตรี)
+ตามตารางรายวิชา: ปีที่ 1 ภาคการศึกษาที่ 2
+วิชาบังคับก่อน: ไม่มี</t>
         </is>
       </c>
       <c r="H36" s="16" t="inlineStr">
         <is>
           <t>AIT 2566 หน้า 23-24
-(หน้าที่ระบบคืนมา: AIT 2566 หน้า 20, 37, 38, 21)</t>
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 20, 23, 37, 289)</t>
         </is>
       </c>
       <c r="I36" s="16" t="inlineStr">
         <is>
-          <t>Semantic topic search (bge-m3) → จัดรูปคำตอบเอง (อาจใช้ Typhoon คัดรหัสวิชา)</t>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J36" s="15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K36" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L36" s="23" t="inlineStr">
-        <is>
-          <t>ถูกบางส่วน</t>
+      <c r="L36" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M36" s="16" t="inlineStr">
         <is>
-          <t>มีวิชาที่ถูกในรายการ แต่ปนวิชาอื่นอีก 5 วิชา (เช่น คอมพิวเตอร์วิทัศน์) ที่ไม่ได้ถาม ผู้อ่านต้องหาเอง</t>
+          <t>ตอบวิชาเดียวตรงคำถาม: 06046403 การโปรแกรมคอมพิวเตอร์ 3(2-2-5) ปี 1 ภาค 2 (ก่อนแก้ ปนวิชาอื่นอีก 5 วิชา)</t>
         </is>
       </c>
       <c r="N36" s="15" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.19s</t>
         </is>
       </c>
       <c r="O36" s="18" t="inlineStr">
@@ -4629,7 +4650,7 @@
       <c r="M37" s="20" t="inlineStr"/>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>0.85s</t>
+          <t>0.75s</t>
         </is>
       </c>
       <c r="O37" s="18" t="inlineStr">
@@ -4708,7 +4729,7 @@
       </c>
       <c r="N38" s="15" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.31s</t>
         </is>
       </c>
       <c r="O38" s="18" t="inlineStr">
@@ -4799,7 +4820,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>0.68s</t>
+          <t>0.90s</t>
         </is>
       </c>
       <c r="O39" s="18" t="inlineStr">
@@ -4912,7 +4933,7 @@
       </c>
       <c r="N40" s="15" t="inlineStr">
         <is>
-          <t>0.55s</t>
+          <t>0.52s</t>
         </is>
       </c>
       <c r="O40" s="18" t="inlineStr">
@@ -5005,7 +5026,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>0.72s</t>
+          <t>0.55s</t>
         </is>
       </c>
       <c r="O41" s="18" t="inlineStr">
@@ -5100,7 +5121,7 @@
       </c>
       <c r="N42" s="15" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="O42" s="18" t="inlineStr">
@@ -5195,7 +5216,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.11s</t>
         </is>
       </c>
       <c r="O43" s="18" t="inlineStr">
@@ -5272,7 +5293,7 @@
       <c r="M44" s="16" t="inlineStr"/>
       <c r="N44" s="15" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.24s</t>
         </is>
       </c>
       <c r="O44" s="18" t="inlineStr">
@@ -5345,7 +5366,7 @@
       <c r="M45" s="20" t="inlineStr"/>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="O45" s="18" t="inlineStr">
@@ -5422,7 +5443,7 @@
       </c>
       <c r="N46" s="15" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.29s</t>
         </is>
       </c>
       <c r="O46" s="18" t="inlineStr">
@@ -5501,7 +5522,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.21s</t>
         </is>
       </c>
       <c r="O47" s="18" t="inlineStr">
@@ -5576,7 +5597,7 @@
       <c r="M48" s="16" t="inlineStr"/>
       <c r="N48" s="15" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="O48" s="18" t="inlineStr">
@@ -5658,7 +5679,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="O49" s="18" t="inlineStr">
@@ -5747,7 +5768,7 @@
       </c>
       <c r="N50" s="15" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.20s</t>
         </is>
       </c>
       <c r="O50" s="18" t="inlineStr">
@@ -5832,7 +5853,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O51" s="18" t="inlineStr">
@@ -5909,7 +5930,7 @@
       </c>
       <c r="N52" s="15" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.13s</t>
         </is>
       </c>
       <c r="O52" s="18" t="inlineStr">
@@ -5951,78 +5972,65 @@
       </c>
       <c r="G53" s="20" t="inlineStr">
         <is>
-          <t>วิชาที่เกี่ยวข้องกับ "ถ้าเลือกแขนงวิศวกรรมข้อมูล ต้องเรียน เลือกกลุ่มไหน (เอกสารอาจใช้คำ: โมดูล / กลุ่ม / สาขา)" — หลักสูตร DSBA
-■ DSBA 2565 — 18 วิชา รวม 54 หน่วยกิต
-  - 06026206 การวิเคราะห์ข้อมูลและการโปรแกรม (DATA ANALYTICS AND PROGRAMMING)
-      หน่วยกิต 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 1
-  - 06026208 พื้นฐานวิทยาการข้อมูล (FUNDAMENTALS OF DATA SCIENCE)
-      หน่วยกิต 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
-  - 06026209 การแสดงข้อมูลด้วยแผนภาพ (DATA VISUALIZATION)
-      หน่วยกิต 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 2
-  - 06066301 โครงสร้างข้อมูลและอัลกอริทึม (DATA STRUCTURES AND ALGORITHMS)
-      หน่วยกิต 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 2
-  - 06026214 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 1 (PROJECT IN DATA SCIENCE AND BUSINESS ANALYTICS 1)
-      หน่วยกิต 3(0-9-0) | ปีที่ 3 ภาคการศึกษาที่ 2
-  - 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 (PROJECT IN DATA SCIENCE AND BUSINESS ANALYTICS 2)
-      หน่วยกิต 3(0-9-0) | ปีที่ 4 ภาคการศึกษาที่ 1
-  - 06026226 หัวข้อพิเศษทางวิทยาการข้อมูล 1 (SPECIAL TOPICS IN DATA SCIENCE 1)
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026227 หัวข้อพิเศษทางวิทยาการข้อมูล 2 (SPECIAL TOPICS IN DATA SCIENCE 2)
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026228 ปฏิบัติการพิเศษทางวิทยาการข้อมูล 1 (SPECIAL WORKSHOP IN DATA SCIENCE 1)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026229 ปฏิบัติการพิเศษทางวิทยาการข้อมูล 2 (SPECIAL WORKSHOP IN DATA SCIENCE 2)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026239 สถาปัตยกรรมข้อมูลแบบไปป์ไลน์ (DATA PIPELINE ARCHITECTURE)
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026244 การดูแลและบำรุงรักษาระบบฐานข้อมูล (DATABASE SYSTEM MAINTENANCE AND ADMINISTRATION)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 (SPECIAL TOPICS IN DATA ENGINEERING 1)
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 (SPECIAL TOPICS IN DATA ENGINEERING 2)
-      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026248 ปฏิบัติการพิเศษทางวิศวกรรมข้อมูล 1 (SPECIAL WORKSHOP IN DATA ENGINEERING 1)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026249 ปฏิบัติการพิเศษทางวิศวกรรมข้อมูล 2 (SPECIAL WORKSHOP IN DATA ENGINEERING 2)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026250 วิทยาการข้อมูลสำหรับธุรกิจ (DATA SCIENCE FOR BUSINESS)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
-  - 06026255 การได้มาและการจัดการข้อมูลทางด้านคลินิก (CLINICAL DATA ACQUISITION AND MANAGEMENT)
-      หน่วยกิต 3(2-2-5) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)</t>
+          <t>กลุ่มวิศวกรรมข้อมูล (ส่วนของกลุ่มวิชาชีพเฉพาะด้าน) — DSBA 2565 (ปริญญาตรี)
+  เรียนจากกลุ่มนี้ 12 หน่วยกิต · ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง · รายวิชาในเล่มหน้า 20
+  รายวิชาในกลุ่ม (11 วิชา):
+    - 06026239 สถาปัตยกรรมข้อมูลแบบไปป์ไลน์ (DATA PIPELINE ARCHITECTURE) — 3(3-0-6)
+    - 06026240 การพัฒนาระบบอัจฉริยะ (INTELLIGENT SYSTEM DEVELOPMENT) — 3(2-2-5)
+    - 06026241 การดำเนินงานการเรียนรู้ของเครื่อง (MACHINE LEARNING OPERATIONS) — 3(3-0-6)
+    - 06026242 โครงสร้างพื้นฐานด้านเทคโนโลยีกลุ่มเมฆ (CLOUD TECHNOLOGY INFRASTRUCTURE) — 3(3-0-6)
+    - 06026243 ระบบฐานข้อมูลขั้นสูง (ADVANCED DATABASE SYSTEMS) — 3 (3-0-6)
+    - 06026244 การดูแลและบำรุงรักษาระบบฐานข้อมูล (DATABASE SYSTEM MAINTENANCE AND ADMINISTRATION) — 3(2-2-5)
+    - 06026245 ระบบฐานข้อมูลแบบกระจาย (DISTRIBUTED DATABASE SYSTEMS) — 3 (3-0-6)
+    - 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 (SPECIAL TOPICS IN DATA ENGINEERING 1) — 3(3-0-6)
+    - 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 (SPECIAL TOPICS IN DATA ENGINEERING 2) — 3(3-0-6)
+    - 06026248 ปฏิบัติการพิเศษทางวิศวกรรมข้อมูล 1 (SPECIAL WORKSHOP IN DATA ENGINEERING 1) — 3(2-2-5)
+    - 06026249 ปฏิบัติการพิเศษทางวิศวกรรมข้อมูล 2 (SPECIAL WORKSHOP IN DATA ENGINEERING 2) — 3(2-2-5)
+  ลงในช่องวิชาเลือกตามแผน:
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1" (หน้า 27)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 2" (หน้า 27)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 3" (หน้า 28)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 4" (หน้า 28)
+    • แผนปกติ ปีที่ 4 ภาคการศึกษาที่ 1: "วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 1" (หน้า 29)
+    • แผนปกติ ปีที่ 4 ภาคการศึกษาที่ 1: "วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 2" (หน้า 29)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1" (หน้า 34)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 2" (หน้า 34)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 3" (หน้า 35)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 4" (หน้า 35)</t>
         </is>
       </c>
       <c r="H53" s="20" t="inlineStr">
         <is>
           <t>DSBA 2565 หน้า 27
-(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 355, 21, 354, 70)</t>
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 20, 27, 28, 29)</t>
         </is>
       </c>
       <c r="I53" s="20" t="inlineStr">
         <is>
-          <t>Semantic topic search (bge-m3) → จัดรูปคำตอบเอง (อาจใช้ Typhoon คัดรหัสวิชา)</t>
+          <t>Structured SQL (วิชาในแขนง/กลุ่มวิชาจากหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
       <c r="J53" s="19" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K53" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L53" s="25" t="inlineStr">
-        <is>
-          <t>ไม่ตรงเฉลย</t>
+      <c r="L53" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
         </is>
       </c>
       <c r="M53" s="20" t="inlineStr">
         <is>
-          <t>ตอบเป็นรายวิชา 18 วิชา 54 หน่วยกิตของทั้งหลักสูตร ไม่ได้ตอบว่ากลุ่มไหน ยังไม่ได้แก้ (ตาราง course ไม่มีข้อมูลว่าวิชาใดอยู่แขนงใด)</t>
+          <t>ตอบว่ากลุ่มวิศวกรรมข้อมูล (ส่วนของกลุ่มวิชาชีพเฉพาะด้าน) เลือกเรียนกลุ่มเดียว 12 หน่วยกิต พร้อมรายวิชา 11 วิชาและช่องวิชาเลือกที่ลงตามแผน (ก่อนแก้ ตอบรายวิชาทั้งหลักสูตร 18 วิชา)</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O53" s="18" t="inlineStr">
@@ -6114,7 +6122,7 @@
       <c r="M54" s="16" t="inlineStr"/>
       <c r="N54" s="15" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O54" s="18" t="inlineStr">
@@ -6211,7 +6219,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O55" s="18" t="inlineStr">
@@ -6294,7 +6302,7 @@
       <c r="M56" s="16" t="inlineStr"/>
       <c r="N56" s="15" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.16s</t>
         </is>
       </c>
       <c r="O56" s="18" t="inlineStr">
@@ -6380,7 +6388,7 @@
       <c r="M57" s="20" t="inlineStr"/>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.08s</t>
         </is>
       </c>
       <c r="O57" s="18" t="inlineStr">
@@ -6466,7 +6474,7 @@
       </c>
       <c r="N58" s="15" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.05s</t>
         </is>
       </c>
       <c r="O58" s="18" t="inlineStr">
@@ -6541,7 +6549,7 @@
       <c r="M59" s="20" t="inlineStr"/>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O59" s="18" t="inlineStr">
@@ -6616,7 +6624,7 @@
       <c r="M60" s="16" t="inlineStr"/>
       <c r="N60" s="15" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O60" s="18" t="inlineStr">
@@ -6694,7 +6702,7 @@
       <c r="M61" s="20" t="inlineStr"/>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O61" s="18" t="inlineStr">
@@ -6819,7 +6827,7 @@
       </c>
       <c r="N62" s="15" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.06s</t>
         </is>
       </c>
       <c r="O62" s="18" t="inlineStr">
@@ -6904,7 +6912,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.15s</t>
         </is>
       </c>
       <c r="O63" s="18" t="inlineStr">
@@ -6916,35 +6924,896 @@
     <row r="64" ht="80" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>fundamental web programming เรียนตอนไหน</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>06066302 การเขียนโปรแกรมเว็บพื้นฐาน ปีที่ 2 ภาคการศึกษาที่ 1 (ทั้งแผนปกติและแผนสหกิจ)</t>
+        </is>
+      </c>
+      <c r="G64" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06066302 การเขียนโปรแกรมเว็บพื้นฐาน (FUNDAMENTAL WEB PROGRAMMING) — 3(2-2-5) หน่วยกิต · หลักสูตร DSBA 2565 (ปริญญาตรี)
+อยู่ในกลุ่มพื้นฐานเทคโนโลยีสารสนเทศ (ส่วนของกลุ่มวิชาแกน) (หน้า 17)
+เรียนตามแผนการศึกษา:
+  - ปีที่ 2 ภาคการศึกษาที่ 1 (ทั้งแผนปกติและแผนสหกิจ, หน้า 25, 32)
+วิชาบังคับก่อน: ไม่มี</t>
+        </is>
+      </c>
+      <c r="H64" s="16" t="inlineStr">
+        <is>
+          <t>DSBA 2565 หน้า 25, 32
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 17, 25, 32, 18)</t>
+        </is>
+      </c>
+      <c r="I64" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J64" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M64" s="16" t="inlineStr">
+        <is>
+          <t>ก่อนแก้ ตอบไม่ได้ (ไม่มีประเภทคำถามค้นวิชาด้วยชื่อ)</t>
+        </is>
+      </c>
+      <c r="N64" s="15" t="inlineStr">
+        <is>
+          <t>0.06s</t>
+        </is>
+      </c>
+      <c r="O64" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="80" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D65" s="20" t="inlineStr">
+        <is>
+          <t>intelligent system development เรียนตอนไหน</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F65" s="20" t="inlineStr">
+        <is>
+          <t>06026240 วิชาเลือกในกลุ่มวิศวกรรมข้อมูล ไม่ผูกภาค ลงในช่องวิชาเลือกกลุ่มวิศวกรรมข้อมูลปี 3 (ภาค 1-2) หรือช่องวิชาเลือกปี 4 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G65" s="20" t="inlineStr">
+        <is>
+          <t>วิชา 06026240 การพัฒนาระบบอัจฉริยะ (INTELLIGENT SYSTEM DEVELOPMENT) — 3(2-2-5) หน่วยกิต · หลักสูตร DSBA 2565 (ปริญญาตรี)
+อยู่ในกลุ่มวิศวกรรมข้อมูล (ส่วนของกลุ่มวิชาชีพเฉพาะด้าน) — ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง (หน้า 20)
+ไม่ได้กำหนดปี/ภาคตายตัวในแผนการศึกษา (เป็นวิชาเลือกของกลุ่ม) ลงเรียนได้ในช่องวิชาเลือกตามแผน:
+  - แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1" (หน้า 27)
+  - แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 2" (หน้า 27)
+  - แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 3" (หน้า 28)
+  - แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 4" (หน้า 28)
+  - แผนปกติ ปีที่ 4 ภาคการศึกษาที่ 1: ช่อง "วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 1" (หน้า 29)
+  - แผนปกติ ปีที่ 4 ภาคการศึกษาที่ 1: ช่อง "วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 2" (หน้า 29)
+  - แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1" (หน้า 34)
+  - แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 2" (หน้า 34)
+  - แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 3" (หน้า 35)
+  - แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: ช่อง "วิชาเลือกกลุ่มวิศวกรรมข้อมูล 4" (หน้า 35)
+วิชาบังคับก่อน: ไม่มี</t>
+        </is>
+      </c>
+      <c r="H65" s="20" t="inlineStr">
+        <is>
+          <t>DSBA 2565 หน้า 20, 27-29
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 20, 27, 28, 29)</t>
+        </is>
+      </c>
+      <c r="I65" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J65" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M65" s="20" t="inlineStr">
+        <is>
+          <t>ก่อนแก้ ขึ้นแค่ชื่อหน่วยกิต ไม่มีข้อมูล ตอนนี้บอกกลุ่ม แขนง และช่องวิชาเลือกที่ลงได้</t>
+        </is>
+      </c>
+      <c r="N65" s="19" t="inlineStr">
+        <is>
+          <t>0.05s</t>
+        </is>
+      </c>
+      <c r="O65" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="80" customHeight="1">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>แขนงวิทยาการข้อมูลมีวิชาอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>14 วิชา 06026216-06026229 (ปัญญาประดิษฐ์ ... ปฏิบัติการพิเศษทางวิทยาการข้อมูล 2) เลือกเรียน 12 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>กลุ่มวิทยาการข้อมูล (ส่วนของกลุ่มวิชาชีพเฉพาะด้าน) — DSBA 2565 (ปริญญาตรี)
+  เรียนจากกลุ่มนี้ 12 หน่วยกิต · ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง · รายวิชาในเล่มหน้า 19
+  รายวิชาในกลุ่ม (14 วิชา):
+    - 06026216 ปัญญาประดิษฐ์ (ARTIFICIAL INTELLIGENCE) — 3(3-0-6)
+    - 06026217 การเรียนรู้ของเครื่อง (MACHINE LEARNING) — 3(3-0-6)
+    - 06026218 การเรียนรู้เชิงลึก (DEEP LEARNING) — 3(2-2-5)
+    - 06026219 การประมวลผลภาษาธรรมชาติ (NATURAL LANGUAGE PROCESSING) — 3(3-0-6)
+    - 06026220 การทำเหมืองข้อมูลกระบวนการ (PROCESS MINING) — 3(3-0-6)
+    - 06026221 การค้นคืนสารสนเทศ (INFORMATION RETRIEVAL) — 3(3-0-6)
+    - 06026222 คอมพิวเตอร์วิชัน (COMPUTER VISION) — 3(3-0-6)
+    - 06026223 การประมวลผลภาพ (IMAGE PROCESSING) — 3(3-0-6)
+    - 06026224 การแปลงข้อมูลและการรู้จำรูปภาพ (IMAGE TRANSFORMATION AND RECOGNITION) — 3(3-0-6)
+    - 06026225 การเรียนรู้เชิงลึกสำหรับการวิเคราะห์ภาพและวีดิโอทางการ แพทย์ (DEEP LEARNING IN MEDICAL IMAGE AND VIDEO ANALYSIS) — 3(2-2-5)
+    - 06026226 หัวข้อพิเศษทางวิทยาการข้อมูล 1 (SPECIAL TOPICS IN DATA SCIENCE 1) — 3(3-0-6)
+    - 06026227 หัวข้อพิเศษทางวิทยาการข้อมูล 2 (SPECIAL TOPICS IN DATA SCIENCE 2) — 3(3-0-6)
+    - 06026228 ปฏิบัติการพิเศษทางวิทยาการข้อมูล 1 (SPECIAL WORKSHOP IN DATA SCIENCE 1) — 3(2-2-5)
+    - 06026229 ปฏิบัติการพิเศษทางวิทยาการข้อมูล 2 (SPECIAL WORKSHOP IN DATA SCIENCE 2) — 3(2-2-5)
+  ลงในช่องวิชาเลือกตามแผน:
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิทยาการข้อมูล 1" (หน้า 27)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิทยาการข้อมูล 2" (หน้า 27)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิทยาการข้อมูล 3" (หน้า 28)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิทยาการข้อมูล 4" (หน้า 28)
+    • แผนปกติ ปีที่ 4 ภาคการศึกษาที่ 1: "วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 1" (หน้า 29)
+    • แผนปกติ ปีที่ 4 ภาคการศึกษาที่ 1: "วิชาเลือกในกลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 2" (หน้า 29)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิทยาการข้อมูล 1" (หน้า 34)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มวิทยาการข้อมูล 2" (หน้า 34)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิทยาการข้อมูล 3" (หน้า 35)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มวิทยาการข้อมูล 4" (หน้า 35)</t>
+        </is>
+      </c>
+      <c r="H66" s="16" t="inlineStr">
+        <is>
+          <t>DSBA 2565 หน้า 19-20
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 19, 27, 28, 29)</t>
+        </is>
+      </c>
+      <c r="I66" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (วิชาในแขนง/กลุ่มวิชาจากหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J66" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="K66" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M66" s="16" t="inlineStr">
+        <is>
+          <t>ก่อนแก้ ตอบรายวิชาทั้งหลักสูตรปนกัน</t>
+        </is>
+      </c>
+      <c r="N66" s="15" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O66" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="80" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B67" s="22" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C67" s="19" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D67" s="20" t="inlineStr">
+        <is>
+          <t>ปี 3 ถ้าเลือกแขนงการวิเคราะห์เชิงสถิติ ต้องเรียนวิชาอะไร</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F67" s="20" t="inlineStr">
+        <is>
+          <t>วิชาในกลุ่มการวิเคราะห์เชิงสถิติ (06026230-06026238) ลงในช่องวิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติปี 3 ภาค 1-2</t>
+        </is>
+      </c>
+      <c r="G67" s="20" t="inlineStr">
+        <is>
+          <t>กลุ่มการวิเคราะห์เชิงสถิติ (ส่วนของกลุ่มวิชาชีพเฉพาะด้าน) — DSBA 2565 (ปริญญาตรี)
+  เรียนจากกลุ่มนี้ 12 หน่วยกิต · ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง · รายวิชาในเล่มหน้า 20
+  รายวิชาในกลุ่ม (9 วิชา):
+    - 06026230 อนุกรมเวลาและการพยากรณ์ (TIME SERIES AND FORECASTING) — 3(3-0-6)
+    - 06026231 สถิติเชิงเบย์ (BAYESIAN STATISTICS) — 3(3-0-6)
+    - 06026232 กระบวนการสโตแคสติกเบื้องต้น (INTRODUCTION TO STOCHASTIC PROCESS) — 3(3-0-6)
+    - 06026233 การวิเคราห์ข้อมูลหลายตัวแปร (MULTIVARIATE DATA ANALYSIS) — 3(3-0-6)
+    - 06026234 การออกแบบการทดลอง (EXPERIMENTAL DESIGN) — 3(3-0-6)
+    - 06026235 หัวข้อพิเศษทางการวิเคราะห์เชิงสถิติ 1 (SPECIAL TOPICS IN STATISTICAL ANALYTICS 1) — 3(3-0-6)
+    - 06026236 หัวข้อพิเศษทางการวิเคราะห์เชิงสถิติ 2 (SPECIAL TOPICS IN STATISTICAL ANALYTICS 2) — 3(3-0-6)
+    - 06026237 ปฏิบัติการพิเศษทางการวิเคราะห์เชิงสถิติ 1 (SPECIAL WORKSHOP IN STATISTICAL ANALYTICS 1) — 3(2-2-5)
+    - 06026238 ปฏิบัติการพิเศษทางการวิเคราะห์เชิงสถิติ 2 (SPECIAL WORKSHOP IN STATISTICAL ANALYTICS 2) — 3(2-2-5)
+  ลงในช่องวิชาเลือกตามแผน:
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 1" (หน้า 27)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 2" (หน้า 27)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 3" (หน้า 28)
+    • แผนปกติ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 4" (หน้า 28)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 1" (หน้า 34)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 1: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 2" (หน้า 34)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 3" (หน้า 35)
+    • แผนสหกิจ ปีที่ 3 ภาคการศึกษาที่ 2: "วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 4" (หน้า 35)</t>
+        </is>
+      </c>
+      <c r="H67" s="20" t="inlineStr">
+        <is>
+          <t>DSBA 2565 หน้า 20, 27-28
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 20, 27, 28, 34)</t>
+        </is>
+      </c>
+      <c r="I67" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (วิชาในแขนง/กลุ่มวิชาจากหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J67" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K67" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M67" s="20" t="inlineStr"/>
+      <c r="N67" s="19" t="inlineStr">
+        <is>
+          <t>0.06s</t>
+        </is>
+      </c>
+      <c r="O67" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="80" customHeight="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="B68" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>โมดูลโครงสร้างพื้นฐานเทคโนโลยีสารสนเทศมีวิชาอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>06016419-06016423 (โครงสร้างพื้นฐานเครือข่ายการสื่อสาร, ระบบโครงสร้างพื้นฐานและการบริการ, ความมั่นคงปลอดภัยโครงสร้างพื้นฐาน, IoT, การออโตเมชั่น)</t>
+        </is>
+      </c>
+      <c r="G68" s="16" t="inlineStr">
+        <is>
+          <t>กลุ่มวิชาด้านโครงสร้างพื้นฐานเทคโนโลยีสารสนเทศ (ส่วนของกลุ่มวิชาบังคับเฉพาะสาขา) — IT 2565 (ปริญญาตรี)
+  ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง · รายวิชาในเล่มหน้า 25
+  รายวิชาในกลุ่ม (5 วิชา):
+    - 06016419 โครงสร้างพื้นฐานเครือข่ายการสื่อสาร (COMMUNICATION NETWORK INFRASTRUCTURE) — 3(2-2-5) | ปี 2 ภาค 2
+    - 06016420 ระบบโครงสร้างพื้นฐานและการบริการ — 3(2-2-5) | ปี 2 ภาค 2
+    - 06016421 ความมั่นคงปลอดภัยโครงสร้างพื้นฐานทางเทคโนโลยีสารสนเทศ (INFORMATION TECHNOLOGY INFRASTRUCTURE SECURITY) — 3(3-0-6) | ปี 3 ภาค 1
+    - 06016422 อินเทอร์เน็ตของสรรพสิ่ง (INTERNET OF THINGS) — 3(2-2-5) | ปี 3 ภาค 1
+    - 06016423 การออโตเมชั่นและโครงสร้างพื้นฐานที่สามารถโปรแกรมได้ (INFRASTRUCTURE PROGRAMMABILITY AND AUTOMATION) — 3(2-2-5) | ปี 3 ภาค 1</t>
+        </is>
+      </c>
+      <c r="H68" s="16" t="inlineStr">
+        <is>
+          <t>IT 2565 หน้า 25
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 25)</t>
+        </is>
+      </c>
+      <c r="I68" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (วิชาในแขนง/กลุ่มวิชาจากหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J68" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K68" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M68" s="16" t="inlineStr"/>
+      <c r="N68" s="15" t="inlineStr">
+        <is>
+          <t>0.16s</t>
+        </is>
+      </c>
+      <c r="O68" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="80" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C69" s="19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D69" s="20" t="inlineStr">
+        <is>
+          <t>อาจารย์ประจำหลักสูตรมีใครบ้าง</t>
+        </is>
+      </c>
+      <c r="E69" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F69" s="20" t="inlineStr">
+        <is>
+          <t>IT 2565 ปริญญาตรี 6 คน: รศ.ดร.โชติพัชร์ ภรณวลัย, รศ.ดร.ธีรพงศ์ ลีลานุภาพ, ผศ.ดร.สิริอร วิทยากร, ผศ.ดร.ธราวิเชษฐ์ ธิติจรูญโรจน์, ดร.สามารถ หมุดและ, ดร.สุพัณณดา โชติพันธ์</t>
+        </is>
+      </c>
+      <c r="G69" s="20" t="inlineStr">
+        <is>
+          <t>อาจารย์ประจำหลักสูตร IT 2565 (ปริญญาตรี) มี 6 คน (มคอ.2 หน้า 49–51):
+  1. รศ.ดร.โชติพัชร์ ภรณวลัย
+  2. รศ.ดร.ธีรพงศ์ ลีลานุภาพ
+  3. ผศ.ดร.สิริอร วิทยากร
+  4. ผศ.ดร.ธราวิเชษฐ์ ธิติจรูญโรจน์
+  5. ดร.สามารถ หมุดและ
+  6. ดร.สุพัณณดา โชติพันธ์
+ในเล่มยังมีรายชื่อ: อาจารย์ผู้รับผิดชอบหลักสูตร 6 คน · อาจารย์ผู้สอน 32 คน</t>
+        </is>
+      </c>
+      <c r="H69" s="20" t="inlineStr">
+        <is>
+          <t>IT 2565 หน้า 49-51
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 49, 50, 51)</t>
+        </is>
+      </c>
+      <c r="I69" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (ตาราง person) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J69" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="K69" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L69" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M69" s="20" t="inlineStr">
+        <is>
+          <t>ก่อนแก้ ตอบอาจารย์ของ ป.โท IT 2568 (ผิดหลักสูตร)</t>
+        </is>
+      </c>
+      <c r="N69" s="19" t="inlineStr">
+        <is>
+          <t>0.12s</t>
+        </is>
+      </c>
+      <c r="O69" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="80" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>อาจารย์ผู้สอนมีกี่คน</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
+        <is>
+          <t>33 คน (หัวข้อ 3.2.3 อาจารย์ผู้สอน)</t>
+        </is>
+      </c>
+      <c r="G70" s="16" t="inlineStr">
+        <is>
+          <t>อาจารย์ผู้สอน DSBA 2565 (ปริญญาตรี) มี 33 คน (มคอ.2 หน้า 44–61):
+  1. ศ.ดร.สุขสันต์ พาณิชพาพิบูล
+  2. รศ.ดร.นพพร โชติกกำธร
+  3. รศ.ดร.จันทร์บูรณ์ สถิตวิริยวงศ์
+  4. รศ.ดร.ศุภมิตร จิตตะยโศธร
+  5. รศ.ดร.วรพจน์ กรีสุระเดช
+  6. รศ.ดร.อาริต ธรรมโน
+  7. รศ.ดร.โชติพัชร์ ภรณวลัย
+  8. รศ.ดร.พรฤดี เนติโสภากุล
+  9. รศ.ดร.ปานวิทย์ ธุวะนุติ
+  10. รศ.ดร.ธีรพงศ์ ลีลานุภาพ
+  11. ผศ.ดร.บุญประเสริฐ สุรักษ์รัตนสกุล
+  12. ผศ.ดร.สมเกียรติ วังศิริพิทักษ์
+  13. ผศ.ดร.สุเมธ ประภาวัต
+  14. ผศ.ดร.ภัทรชัย ลลิตโรจน์วงศ์
+  15. ผศ.ดร.กันต์พงษ์ วรรัตน์ปัญญา
+  16. ผศ.ดร.มานพ พันธ์โคกกรวด
+  17. ผศ.ดร.สุภกิจ นุตยะสกุล
+  18. ผศ.ดร.บัณฑิต ฐานะโสภณ
+  19. ผศ.ดร.ลภัส ประดิษฐ์ทัศนีย์
+  20. ผศ.ดร.อนันตพัฒน์ อนันตชัย
+  21. ผศ.ดร.สิริอร วิทยากร
+  22. ผศ.ดร.ปรมาพร เรืองผกา
+  23. ผศ.ดร.ธราวิเชษฐ์ ฐิติจรูญโรจน์
+  24. ผศ.อัครินทร์ คุณกิตติ
+  25. ผศ.ศรีนวล นลินทิพยวงศ์
+  26. ดร.สุภวรรณ ทัศนประเสริฐ
+  27. ดร.พัฒนพงษ์ ฉันทมิตรโอภาส
+  28. ดร.สุพัณณดา โชติพันธ์
+  29. ดร.พรสุรีย์ แจ่มศรี
+  30. ดร.สามารถ หมุดและ
+  31. ดร.นนท์ คนึงสุขเกษม
+  32. ดร.ประพันธ์ ปวรางกูร
+  33. ดร.ศิรสิทธิ์ โล่ห์ชนะจิต
+ในเล่มยังมีรายชื่อ: อาจารย์ผู้รับผิดชอบหลักสูตร 5 คน · อาจารย์ประจำหลักสูตร 5 คน</t>
+        </is>
+      </c>
+      <c r="H70" s="16" t="inlineStr">
+        <is>
+          <t>DSBA 2565 หน้า 44-61
+(หน้าที่ระบบคืนมา: DSBA 2565 หน้า 44, 45, 46, 47)</t>
+        </is>
+      </c>
+      <c r="I70" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (ตาราง person) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J70" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="K70" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L70" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M70" s="16" t="inlineStr"/>
+      <c r="N70" s="15" t="inlineStr">
+        <is>
+          <t>0.05s</t>
+        </is>
+      </c>
+      <c r="O70" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="80" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>ระดับ 1: ง่าย (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C71" s="19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D71" s="20" t="inlineStr">
+        <is>
+          <t>วิชา server-side web development เรียนตอนไหน</t>
+        </is>
+      </c>
+      <c r="E71" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F71" s="20" t="inlineStr">
+        <is>
+          <t>06016418 ปีที่ 3 ภาคการศึกษาที่ 1 (อยู่ในโมดูลการพัฒนาซอฟต์แวร์และโมดูลสื่อประสม)</t>
+        </is>
+      </c>
+      <c r="G71" s="20" t="inlineStr">
+        <is>
+          <t>วิชา 06016418 การพัฒนาเว็บฝั่งเซิร์ฟเวอร์ (SERVER-SIDE WEB DEVELOPMENT) — 3(2-2-5) หน่วยกิต · หลักสูตร IT 2565 (ปริญญาตรี)
+อยู่ในกลุ่มวิชาด้านการพัฒนาซอฟต์แวร์ (ส่วนของกลุ่มวิชาบังคับเฉพาะสาขา) — ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง (หน้า 25)
+อยู่ในกลุ่มวิชาด้านสื่อประสมสำหรับการพัฒนาสื่อเชิงโต้ตอบ เว็บ และเกม (ส่วนของกลุ่มวิชาบังคับเฉพาะสาขา) — ต้องเลือกเรียนกลุ่มใดกลุ่มหนึ่ง (หน้า 25)
+เรียนตามแผนการศึกษา:
+  - ปีที่ 3 ภาคการศึกษาที่ 1 (ทั้งแผนปกติและแผนสหกิจ, หน้า 35, 42)
+วิชาบังคับก่อน: 06016408 การสร้างโปรแกรมเชิงวัตถุ</t>
+        </is>
+      </c>
+      <c r="H71" s="20" t="inlineStr">
+        <is>
+          <t>IT 2565 หน้า 25, 35
+(หน้าที่ระบบคืนมา: IT 2565 หน้า 25, 35, 42, 26)</t>
+        </is>
+      </c>
+      <c r="I71" s="20" t="inlineStr">
+        <is>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J71" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="K71" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M71" s="20" t="inlineStr"/>
+      <c r="N71" s="19" t="inlineStr">
+        <is>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="O71" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="80" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="B72" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>วิชา data structures and algorithms principles อยู่กลุ่มไหน เรียนปีไหน</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>06036120 กลุ่มเทคโนโลยีและวิธีการทางซอฟต์แวร์ ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="G72" s="16" t="inlineStr">
+        <is>
+          <t>วิชา 06036120 หลักการโครงสร้างข้อมูลและอัลกอริทึม (DATA STRUCTURES AND ALGORITHMS PRINCIPLES) — 3(3-0-6) หน่วยกิต · หลักสูตร BIT 2565 (ปริญญาตรี)
+อยู่ในกลุ่มเทคโนโลยีและวิธีการทางซอฟต์แวร์ (ส่วนของกลุ่มวิชาเฉพาะด้าน) (หน้า 23)
+เรียนตามแผนการศึกษา:
+  - ปีที่ 2 ภาคการศึกษาที่ 1 (ทั้งแผนปกติและแผนสหกิจ, หน้า 27, 32)
+วิชาบังคับก่อน: ไม่มี</t>
+        </is>
+      </c>
+      <c r="H72" s="16" t="inlineStr">
+        <is>
+          <t>BIT 2565
+(หน้าที่ระบบคืนมา: BIT 2565 หน้า 23, 27, 32, 75)</t>
+        </is>
+      </c>
+      <c r="I72" s="16" t="inlineStr">
+        <is>
+          <t>Structured SQL (ค้นวิชา: ตารางแผนและหัวข้อรายวิชาในเล่ม) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J72" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="K72" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" s="18" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M72" s="16" t="inlineStr"/>
+      <c r="N72" s="15" t="inlineStr">
+        <is>
+          <t>0.08s</t>
+        </is>
+      </c>
+      <c r="O72" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="80" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B73" s="21" t="inlineStr">
+        <is>
+          <t>ระดับ 2: ปานกลาง (ชุดจาก tester)</t>
+        </is>
+      </c>
+      <c r="C73" s="19" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D73" s="20" t="inlineStr">
+        <is>
+          <t>อาจารย์ศุภมิตร จิตตะยโศธร จบการศึกษาจากที่ไหน</t>
+        </is>
+      </c>
+      <c r="E73" s="20" t="inlineStr">
+        <is>
+          <t>ชุดเพิ่ม: ข้อเท็จจริง / prerequisite / วิชาที่ไม่มี / สรุปจากแผน (ตรวจเฉลยจากเล่ม)</t>
+        </is>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
+        <is>
+          <t>วศ.บ. วิศวกรรมคอมพิวเตอร์ สจล. 2523; Master of Engineering (Computer) AIT 2525; Ph.D. (Computer Science) The University of Queensland ออสเตรเลีย 2531 และต้องไม่แสดงเลขประจำตัวประชาชน 13 หลัก</t>
+        </is>
+      </c>
+      <c r="G73" s="20" t="inlineStr">
+        <is>
+          <t>ศ.ดร.ศุภมิตร จิตตะยโศธร สำเร็จการศึกษาระดับวศ.บ. (วิศวกรรมคอมพิวเตอร์) จากสถาบันเทคโนโลยีพระจอมเกล้าเจ้าคุณทหารลาดกระบัง ปี 2523 [1]</t>
+        </is>
+      </c>
+      <c r="H73" s="20" t="inlineStr">
+        <is>
+          <t>AIT 2566 หน้า 42
+(หน้าที่ระบบคืนมา: AIT 2566 หน้า 42, 75, 80, 79)</t>
+        </is>
+      </c>
+      <c r="I73" s="20" t="inlineStr">
+        <is>
+          <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
+        </is>
+      </c>
+      <c r="J73" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K73" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="23" t="inlineStr">
+        <is>
+          <t>ถูกบางส่วน</t>
+        </is>
+      </c>
+      <c r="M73" s="20" t="inlineStr">
+        <is>
+          <t>ตอบเฉพาะวุฒิปริญญาตรี (วศ.บ. สจล. 2523) ขาดปริญญาโท (AIT 2525) และปริญญาเอก (Queensland 2531) แต่ไม่มีเลขประจำตัวประชาชนหลุด</t>
+        </is>
+      </c>
+      <c r="N73" s="19" t="inlineStr">
+        <is>
+          <t>1.37s</t>
+        </is>
+      </c>
+      <c r="O73" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="80" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="B64" s="24" t="inlineStr">
+      <c r="B74" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตรของ DSBA ฉบับ 2560 กับฉบับ 2565 ต่างกันกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E64" s="16" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F64" s="16" t="inlineStr">
+      <c r="F74" s="16" t="inlineStr">
         <is>
           <t>2560 = 126 หน่วยกิต, 2565 = 132 หน่วยกิต ต่างกัน 6 หน่วยกิต (2565 มากกว่า)</t>
         </is>
       </c>
-      <c r="G64" s="16" t="inlineStr">
+      <c r="G74" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - DSBA 2560: 126 หน่วยกิต (มคอ.2 DSBA 2560 หน้า 17)
@@ -6952,78 +7821,78 @@
 สรุป: DSBA 2565 มากกว่า DSBA 2560 อยู่ 6 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H64" s="16" t="inlineStr">
+      <c r="H74" s="16" t="inlineStr">
         <is>
           <t>DSBA2560 หน้า 17; DSBA2565 หน้า 15
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 351, 349, 352; DSBA 2560 หน้า 17)</t>
         </is>
       </c>
-      <c r="I64" s="16" t="inlineStr">
+      <c r="I74" s="16" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J64" s="15" t="n">
+      <c r="J74" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K64" s="15" t="inlineStr">
+      <c r="K74" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L64" s="18" t="inlineStr">
+      <c r="L74" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M64" s="16" t="inlineStr">
+      <c r="M74" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N64" s="15" t="inlineStr">
-        <is>
-          <t>0.10s</t>
-        </is>
-      </c>
-      <c r="O64" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="80" customHeight="1">
-      <c r="A65" s="13" t="inlineStr">
+      <c r="N74" s="15" t="inlineStr">
+        <is>
+          <t>0.11s</t>
+        </is>
+      </c>
+      <c r="O74" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="80" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B65" s="24" t="inlineStr">
+      <c r="B75" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C65" s="19" t="inlineStr">
+      <c r="C75" s="19" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="D65" s="20" t="inlineStr">
+      <c r="D75" s="20" t="inlineStr">
         <is>
           <t>หลักสูตร BIT 2560 กับ BIT 2565 มีหน่วยกิตรวมตลอดหลักสูตรเท่ากันหรือไม่</t>
         </is>
       </c>
-      <c r="E65" s="20" t="inlineStr">
+      <c r="E75" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F65" s="20" t="inlineStr">
+      <c r="F75" s="20" t="inlineStr">
         <is>
           <t>เท่ากัน ทั้งสองฉบับ 126 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G65" s="20" t="inlineStr">
+      <c r="G75" s="20" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - BIT 2560: 126 หน่วยกิต (มคอ.2 BIT 2560 หน้า 17)
@@ -7031,78 +7900,78 @@
 สรุป: เท่ากัน (126 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H65" s="20" t="inlineStr">
+      <c r="H75" s="20" t="inlineStr">
         <is>
           <t>BIT2560 หน้า 17; BIT2565 หน้า 6
 (หน้าที่ระบบคืนมา: BIT 2565 หน้า 266, 264, 3, 265)</t>
         </is>
       </c>
-      <c r="I65" s="20" t="inlineStr">
+      <c r="I75" s="20" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J65" s="19" t="n">
+      <c r="J75" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="K65" s="15" t="inlineStr">
+      <c r="K75" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L65" s="18" t="inlineStr">
+      <c r="L75" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M65" s="20" t="inlineStr">
+      <c r="M75" s="20" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N65" s="19" t="inlineStr">
-        <is>
-          <t>0.08s</t>
-        </is>
-      </c>
-      <c r="O65" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="80" customHeight="1">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="N75" s="19" t="inlineStr">
+        <is>
+          <t>0.15s</t>
+        </is>
+      </c>
+      <c r="O75" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="80" customHeight="1">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>X3</t>
         </is>
       </c>
-      <c r="B66" s="24" t="inlineStr">
+      <c r="B76" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C66" s="15" t="inlineStr">
+      <c r="C76" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
+      <c r="D76" s="16" t="inlineStr">
         <is>
           <t>ระหว่างหลักสูตร DSBA 2565, AIT 2566 และ BIT 2565 หลักสูตรใดมีหน่วยกิตรวมมากที่สุด</t>
         </is>
       </c>
-      <c r="E66" s="16" t="inlineStr">
+      <c r="E76" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F66" s="16" t="inlineStr">
+      <c r="F76" s="16" t="inlineStr">
         <is>
           <t>DSBA 2565 มากที่สุด 132 หน่วยกิต (BIT 2565 = 126, AIT 2566 = 120)</t>
         </is>
       </c>
-      <c r="G66" s="16" t="inlineStr">
+      <c r="G76" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - DSBA 2565: 132 หน่วยกิต (มคอ.2 DSBA 2565 หน้า 2)
@@ -7111,78 +7980,78 @@
 สรุป: มากที่สุดคือ DSBA 2565 (132 หน่วยกิต) น้อยที่สุดคือ AIT 2566 (120 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H66" s="16" t="inlineStr">
+      <c r="H76" s="16" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 15; BIT2565 หน้า 6; AIT2566 หน้า 5
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 78; DSBA 2565 หน้า 352, 349; BIT 2565 หน้า 264)</t>
         </is>
       </c>
-      <c r="I66" s="16" t="inlineStr">
+      <c r="I76" s="16" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J66" s="15" t="n">
+      <c r="J76" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K66" s="15" t="inlineStr">
+      <c r="K76" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L66" s="18" t="inlineStr">
+      <c r="L76" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M66" s="16" t="inlineStr">
+      <c r="M76" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N66" s="15" t="inlineStr">
-        <is>
-          <t>0.22s</t>
-        </is>
-      </c>
-      <c r="O66" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="80" customHeight="1">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="N76" s="15" t="inlineStr">
+        <is>
+          <t>0.20s</t>
+        </is>
+      </c>
+      <c r="O76" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="80" customHeight="1">
+      <c r="A77" s="13" t="inlineStr">
         <is>
           <t>X4</t>
         </is>
       </c>
-      <c r="B67" s="24" t="inlineStr">
+      <c r="B77" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="C77" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D67" s="20" t="inlineStr">
+      <c r="D77" s="20" t="inlineStr">
         <is>
           <t>ในแผนสหกิจศึกษาของ DSBA 2565 ต้องลงทะเบียนวิชาสหกิจศึกษาในภาคไหน และกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E67" s="20" t="inlineStr">
+      <c r="E77" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F67" s="20" t="inlineStr">
+      <c r="F77" s="20" t="inlineStr">
         <is>
           <t>ปีที่ 4 ภาคการศึกษาที่ 2 จำนวน 6 หน่วยกิต (06026259 สหกิจศึกษา หรือ 06026260 สหกิจศึกษาต่างประเทศ)</t>
         </is>
       </c>
-      <c r="G67" s="20" t="inlineStr">
+      <c r="G77" s="20" t="inlineStr">
         <is>
           <t>รายวิชาที่มีเฉพาะในแผนที่เข้าโครงการสหกิจศึกษา (DSBA 2565 (ปริญญาตรี)):
 - 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0) | ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36)
@@ -7190,156 +8059,160 @@
 ภาคนั้นรวม 6 หน่วยกิตตามแผนในเล่ม (ในแผนปกติภาคเดียวกันรวม 9 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H67" s="20" t="inlineStr">
+      <c r="H77" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 36
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36)</t>
         </is>
       </c>
-      <c r="I67" s="20" t="inlineStr">
+      <c r="I77" s="20" t="inlineStr">
         <is>
           <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J67" s="19" t="n">
+      <c r="J77" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="K67" s="15" t="inlineStr">
+      <c r="K77" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L67" s="18" t="inlineStr">
+      <c r="L77" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M67" s="20" t="inlineStr">
+      <c r="M77" s="20" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ตอบจากตารางแผนสหกิจในเล่ม: สหกิจศึกษา 06026259/06026260 ปี 4 ภาค 2 6 หน่วยกิต (หน้า 36)</t>
         </is>
       </c>
-      <c r="N67" s="19" t="inlineStr">
-        <is>
-          <t>0.07s</t>
-        </is>
-      </c>
-      <c r="O67" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="80" customHeight="1">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="N77" s="19" t="inlineStr">
+        <is>
+          <t>0.05s</t>
+        </is>
+      </c>
+      <c r="O77" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="80" customHeight="1">
+      <c r="A78" s="13" t="inlineStr">
         <is>
           <t>X5</t>
         </is>
       </c>
-      <c r="B68" s="24" t="inlineStr">
+      <c r="B78" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C78" s="15" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>หลักสูตรปริญญาโท IT 2563 กับ 2568 แบ่งแผนการศึกษาต่างกันอย่างไร</t>
         </is>
       </c>
-      <c r="E68" s="16" t="inlineStr">
+      <c r="E78" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F68" s="16" t="inlineStr">
+      <c r="F78" s="16" t="inlineStr">
         <is>
           <t>2563: แผน ก (แบบ ก1, ก2) และแผน ข; 2568: แผน 1 แบบวิชาการ (แบบ 1.1, 1.2) และแผน 2 แบบวิชาชีพ; ทุกแผนเรียน 36 หน่วยกิตเท่ากัน</t>
         </is>
       </c>
-      <c r="G68" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2563 (IT 2563) มีแผนการศึกษาแบบ ก 1 และ ก 2 ซึ่งรับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ตั้งแต่ปีการศึกษา 2563 ถึง 2567 โดยมีนักศึกษาชั้นปีที่ 2 เริ่มเข้าศึกษาในปีการศึกษา 2564 เป็นต้นไป รวมนักศึกษาทั้งหมดในแต่ละปีไม่เกิน 10 คน และคาดว่าจะสำเร็จการศึกษา 5 คนต่อปีตั้งแต่ปีการศึกษา 2564 [3]
-ในขณะที่หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ ปีการศึกษา 2568 (IT 2568) มีแผนการศึกษา 3 แบบ ได้แก่ แผน 1 แบบวิชาการ แบบ 1.1 และ 1.2 รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ตั้งแต่ปีการศึกษา 2568 ถึง 2572 รวมนักศึกษาทั้งหมดในแต่ละปีไม่เกิน 6 คน และคาดว่าจะสำเร็จการศึกษา 3 คนต่อปีตั้งแต่ปีการศึกษา 2569 เป็นต้นไป พร้อมกันนี้ยังมีแผน 2 แบบวิชาชีพ รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ตั้งแต่ปีการศึกษา 2568 ถึง 2572 รวมนักศึกษาทั้งหมดในแต่ละปีไม่เกิน 60 คน และคาดว่าจะสำเร็จการศึกษา 30 คนต่อปีตั้งแต่ปีการศึกษา 2569 เป็นต้นไป [2]
-ดังนั้น ความแตกต่างคือ หลักสูตร 2563 มีเพียง 2 แผน (ก 1 และ ก 2) รับคนละ 5 คนต่อปี ขณะที่หลักสูตร 2568 มี 3 แผน แบ่งเป็นแผนวิชาการ (แบบ 1.1 และ 1.2) รับคนละ 3 คนต่อปี และแผนวิชาชีพรับ 30 คนต่อปี ทำให้จำนวนนักศึก</t>
-        </is>
-      </c>
-      <c r="H68" s="16" t="inlineStr">
+      <c r="G78" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ (IT) ปีการศึกษา 2563 และ 2568 มีการแบ่งแผนการศึกษาแตกต่างกันดังนี้:
+- **แผน ก แบบ ก 1 (ปี 2563)**: รับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ชั้นปีที่ 2 ปีละ 5 คน รวม 10 คนต่อปีการศึกษา คาดว่าสำเร็จการศึกษา 5 คนต่อปี [3]  
+- **แผน ก แบบ ก 2 (ปี 2563)**: รับนักศึกษาชั้นปีที่ 1 ปีละ 5 คน ชั้นปีที่ 2 ปีละ 5 คน รวม 10 คนต่อปีการศึกษา คาดว่าสำเร็จการศึกษา 5 คนต่อปี [3]  
+- **แผน 1 แบบวิชาการ แบบ 1.1 (ปี 2568)**: รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ชั้นปีที่ 2 ปีละ 3 คน รวม 6 คนต่อปีการศึกษา คาดว่าสำเร็จการศึกษา 3 คนต่อปี [2]  
+- **แผน 1 แบบวิชาการ แบบ 1.2 (ปี 2568)**: รับนักศึกษาชั้นปีที่ 1 ปีละ 3 คน ชั้นปีที่ 2 ปีละ 3 คน รวม 6 คนต่อปีการศึกษา คาดว่าสำเร็จการศึกษา 3 คนต่อปี [2]  
+- **แผน 2 แบบวิชาชีพ (ปี 2568)**: รับนักศึกษาชั้นปีที่ 1 ปีละ 30 คน ชั้นปีที่ 2 ปีละ 30 คน รวม 60 คนต่อปีการศึกษา คาดว่าสำเร็จการศึกษา 30 คนต่อปี [2]  
+สรุป: หลักสูตรปี 2568 มีแผนการศึกษาแยกเป็น 3 แบบ (แบบวิชาการ 1.1, 1.2 และแบบวิชาชีพ) โดยมีจำนวนรับนักศึกษาต่อปีมากกว่าปี 2563 และมีการแบ่งแผนชัดเจนตามประเภทการเรียนรู้ [2][3]</t>
+        </is>
+      </c>
+      <c r="H78" s="16" t="inlineStr">
         <is>
           <t>IT2563 หน้า 16; IT2568 หน้า 5
 (หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 153, 11; วท.ม. IT 2563 หน้า 15)</t>
         </is>
       </c>
-      <c r="I68" s="16" t="inlineStr">
+      <c r="I78" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J68" s="15" t="n">
+      <c r="J78" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="K68" s="15" t="inlineStr">
+      <c r="K78" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L68" s="23" t="inlineStr">
+      <c r="L78" s="23" t="inlineStr">
         <is>
           <t>ถูกบางส่วน</t>
         </is>
       </c>
-      <c r="M68" s="16" t="inlineStr">
+      <c r="M78" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] อธิบายแผนของ 2568 ถูก แต่ของ 2563 ขาดแผน ข และตอบจำนวนรับนักศึกษาแทนโครงสร้างแผน</t>
         </is>
       </c>
-      <c r="N68" s="15" t="inlineStr">
-        <is>
-          <t>12.81s</t>
-        </is>
-      </c>
-      <c r="O68" s="15" t="inlineStr">
+      <c r="N78" s="15" t="inlineStr">
+        <is>
+          <t>10.78s</t>
+        </is>
+      </c>
+      <c r="O78" s="15" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="80" customHeight="1">
-      <c r="A69" s="13" t="inlineStr">
+    <row r="79" ht="80" customHeight="1">
+      <c r="A79" s="13" t="inlineStr">
         <is>
           <t>X6</t>
         </is>
       </c>
-      <c r="B69" s="24" t="inlineStr">
+      <c r="B79" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C69" s="19" t="inlineStr">
+      <c r="C79" s="19" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D69" s="20" t="inlineStr">
+      <c r="D79" s="20" t="inlineStr">
         <is>
           <t>ถ้าจะเรียนวิชาพื้นฐานการเรียนรู้เชิงลึก (Fundamentals of Deep Learning) ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
         </is>
       </c>
-      <c r="E69" s="20" t="inlineStr">
+      <c r="E79" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F69" s="20" t="inlineStr">
+      <c r="F79" s="20" t="inlineStr">
         <is>
           <t>ต้องผ่านแคลคูลัส 2 (06046401) และพีชคณิตเชิงเส้น (06046402); แคลคูลัส 2 ต้องผ่านแคลคูลัส 1 (06046400) ก่อน; พีชคณิตเชิงเส้นและแคลคูลัส 1 ไม่มีวิชาบังคับก่อน</t>
         </is>
       </c>
-      <c r="G69" s="20" t="inlineStr">
+      <c r="G79" s="20" t="inlineStr">
         <is>
           <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   ต้องผ่านวิชาบังคับก่อน:
@@ -7348,158 +8221,155 @@
     • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
         </is>
       </c>
-      <c r="H69" s="20" t="inlineStr">
+      <c r="H79" s="20" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 287-288
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 37, 292, 19, 20)</t>
         </is>
       </c>
-      <c r="I69" s="20" t="inlineStr">
+      <c r="I79" s="20" t="inlineStr">
         <is>
           <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J69" s="19" t="n">
+      <c r="J79" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K69" s="15" t="inlineStr">
+      <c r="K79" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L69" s="18" t="inlineStr">
+      <c r="L79" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M69" s="20" t="inlineStr">
+      <c r="M79" s="20" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ไล่วิชาบังคับก่อน 2 ชั้นได้ครบ</t>
         </is>
       </c>
-      <c r="N69" s="19" t="inlineStr">
-        <is>
-          <t>0.90s</t>
-        </is>
-      </c>
-      <c r="O69" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="80" customHeight="1">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="N79" s="19" t="inlineStr">
+        <is>
+          <t>0.92s</t>
+        </is>
+      </c>
+      <c r="O79" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="80" customHeight="1">
+      <c r="A80" s="13" t="inlineStr">
         <is>
           <t>X7</t>
         </is>
       </c>
-      <c r="B70" s="24" t="inlineStr">
+      <c r="B80" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C70" s="15" t="inlineStr">
+      <c r="C80" s="15" t="inlineStr">
         <is>
           <t>AITBA</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>หลักสูตรปริญญาโท AITBA 2564 กับ 2569 หน่วยกิตที่เรียนตลอดหลักสูตรต่างกันไหม และชื่อแผนการศึกษาเปลี่ยนไปอย่างไร</t>
         </is>
       </c>
-      <c r="E70" s="16" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F70" s="16" t="inlineStr">
+      <c r="F80" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตไม่ต่าง ทุกแผน 36 หน่วยกิต; 2564 ใช้แผน ก (ก1, ก2) และแผน ข; 2569 ใช้แผนวิชาการ (แบบ 1.1, 1.2) และแผนวิชาชีพ</t>
         </is>
       </c>
-      <c r="G70" s="16" t="inlineStr">
-        <is>
-          <t>หลักสูตรปริญญาโท AITBA 2564 และ 2569 ไม่มีการเปลี่ยนแปลงจำนวนหน่วยกิตที่เรียนตลอดหลักสูตร เนื่องจากทั้งสองฉบับมีจำนวนหน่วยกิตรวมทั้งหมด 36 หน่วยกิต [6]  
-สำหรับชื่อแผนการศึกษา หลักสูตร AITBA 2569 มีการปรับปรุงชื่อแผนการศึกษาดังนี้:  
-- แผน ก แบบ ก1 เปลี่ยนเป็น แผน 1.1 (แบบวิชาการ) [3]  
-- แผน ก แบบ ก2 เปลี่ยนเป็น แผน 1.2 (แบบวิชาการ) [3]  
-- แผน ข เปลี่ยนเป็น แผน 2 (แบบวิชาชีพ) [3]</t>
-        </is>
-      </c>
-      <c r="H70" s="16" t="inlineStr">
+      <c r="G80" s="16" t="inlineStr">
+        <is>
+          <t>หลักสูตรปริญญาโท AITBA 2564 และ 2569 ไม่มีความแตกต่างด้านจำนวนหน่วยกิตที่เรียนตลอดหลักสูตร เนื่องจากทั้งสองฉบับกำหนดให้มีจำนวนหน่วยกิตรวมไม่น้อยกว่า 36 หน่วยกิต [6]  
+สำหรับชื่อแผนการศึกษา หลักสูตร AITBA 2569 ปรับปรุงชื่อแผนการศึกษาจากเดิม "แผน ก แบบ ก1", "แผน ก แบบ ก2", และ "แผน ข" เป็น "แผน 1.1", "แผน 1.2", และ "แผน 2" ตามลำดับ [3]</t>
+        </is>
+      </c>
+      <c r="H80" s="16" t="inlineStr">
         <is>
           <t>AITBA2564 หน้า 6; AITBA2569 หน้า 5
 (หน้าที่ระบบคืนมา: ปร.ด. AITBA 2569 หน้า 223, 99, 225, 167; วท.ม. AITBA 2564 หน้า 6, 3)</t>
         </is>
       </c>
-      <c r="I70" s="16" t="inlineStr">
+      <c r="I80" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J70" s="15" t="n">
+      <c r="J80" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="K70" s="15" t="inlineStr">
+      <c r="K80" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L70" s="18" t="inlineStr">
+      <c r="L80" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M70" s="16" t="inlineStr">
+      <c r="M80" s="16" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)]</t>
         </is>
       </c>
-      <c r="N70" s="15" t="inlineStr">
-        <is>
-          <t>4.96s</t>
-        </is>
-      </c>
-      <c r="O70" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="80" customHeight="1">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="N80" s="15" t="inlineStr">
+        <is>
+          <t>3.75s</t>
+        </is>
+      </c>
+      <c r="O80" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="80" customHeight="1">
+      <c r="A81" s="13" t="inlineStr">
         <is>
           <t>X8</t>
         </is>
       </c>
-      <c r="B71" s="24" t="inlineStr">
+      <c r="B81" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด X)</t>
         </is>
       </c>
-      <c r="C71" s="19" t="inlineStr">
+      <c r="C81" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D71" s="20" t="inlineStr">
+      <c r="D81" s="20" t="inlineStr">
         <is>
           <t>แผนปกติกับแผนสหกิจศึกษาของ DSBA 2565 มีหน่วยกิตรวมตลอดหลักสูตรต่างกันไหม</t>
         </is>
       </c>
-      <c r="E71" s="20" t="inlineStr">
+      <c r="E81" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F71" s="20" t="inlineStr">
+      <c r="F81" s="20" t="inlineStr">
         <is>
           <t>ไม่ต่าง ทั้งสองแผนรวม 132 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G71" s="20" t="inlineStr">
+      <c r="G81" s="20" t="inlineStr">
         <is>
           <t>เปรียบเทียบแผนการศึกษา DSBA 2565 (ปริญญาตรี): แผนปกติ (3.1.4.1) กับแผนที่เข้าโครงการสหกิจศึกษา (3.1.4.2)
 - ปีที่ 1 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
@@ -7538,78 +8408,78 @@
 ตามโครงสร้างหลักสูตร: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6)</t>
         </is>
       </c>
-      <c r="H71" s="20" t="inlineStr">
+      <c r="H81" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 15, 36
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29, 36)</t>
         </is>
       </c>
-      <c r="I71" s="20" t="inlineStr">
+      <c r="I81" s="20" t="inlineStr">
         <is>
           <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J71" s="19" t="n">
+      <c r="J81" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="K71" s="15" t="inlineStr">
+      <c r="K81" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L71" s="18" t="inlineStr">
+      <c r="L81" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M71" s="20" t="inlineStr">
+      <c r="M81" s="20" t="inlineStr">
         <is>
           <t>[ชุด X: ใช้ออกแบบการแก้รอบที่ 1 (ไม่ใช่ held-out)] ตอบเป็นตารางเทียบหน่วยกิตรายภาคของสองแผน รวมทั้งหลักสูตรเท่ากัน 132</t>
         </is>
       </c>
-      <c r="N71" s="19" t="inlineStr">
-        <is>
-          <t>0.21s</t>
-        </is>
-      </c>
-      <c r="O71" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="80" customHeight="1">
-      <c r="A72" s="13" t="inlineStr">
+      <c r="N81" s="19" t="inlineStr">
+        <is>
+          <t>0.27s</t>
+        </is>
+      </c>
+      <c r="O81" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="80" customHeight="1">
+      <c r="A82" s="13" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="B72" s="24" t="inlineStr">
+      <c r="B82" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C72" s="15" t="inlineStr">
+      <c r="C82" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D72" s="16" t="inlineStr">
+      <c r="D82" s="16" t="inlineStr">
         <is>
           <t>หลักสูตร AIT 2566 กับ IT 2565 ต้องเรียนหน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E72" s="16" t="inlineStr">
+      <c r="E82" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F72" s="16" t="inlineStr">
+      <c r="F82" s="16" t="inlineStr">
         <is>
           <t>AIT 2566 = 120, IT 2565 = 129 ต่างกัน 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G72" s="16" t="inlineStr">
+      <c r="G82" s="16" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - AIT 2566: 120 หน่วยกิต (มคอ.2 AIT 2566 หน้า 5)
@@ -7617,78 +8487,78 @@
 สรุป: IT 2565 มากกว่า AIT 2566 อยู่ 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H72" s="16" t="inlineStr">
+      <c r="H82" s="16" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 5; IT2565 หน้า 6/20
 (หน้าที่ระบบคืนมา: IT 2565 หน้า 369, 378, 371; AIT 2566 หน้า 78)</t>
         </is>
       </c>
-      <c r="I72" s="16" t="inlineStr">
+      <c r="I82" s="16" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J72" s="15" t="n">
+      <c r="J82" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K72" s="15" t="inlineStr">
+      <c r="K82" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L72" s="18" t="inlineStr">
+      <c r="L82" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M72" s="16" t="inlineStr">
+      <c r="M82" s="16" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N72" s="15" t="inlineStr">
-        <is>
-          <t>0.43s</t>
-        </is>
-      </c>
-      <c r="O72" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="80" customHeight="1">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="N82" s="15" t="inlineStr">
+        <is>
+          <t>0.48s</t>
+        </is>
+      </c>
+      <c r="O82" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="80" customHeight="1">
+      <c r="A83" s="13" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="B73" s="24" t="inlineStr">
+      <c r="B83" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C73" s="19" t="inlineStr">
+      <c r="C83" s="19" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="D73" s="20" t="inlineStr">
+      <c r="D83" s="20" t="inlineStr">
         <is>
           <t>BIT 2565 กับ DSBA 2560 หลักสูตรไหนต้องเรียนหน่วยกิตรวมมากกว่ากัน</t>
         </is>
       </c>
-      <c r="E73" s="20" t="inlineStr">
+      <c r="E83" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F73" s="20" t="inlineStr">
+      <c r="F83" s="20" t="inlineStr">
         <is>
           <t>เท่ากัน ทั้งคู่ 126 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G73" s="20" t="inlineStr">
+      <c r="G83" s="20" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
@@ -7696,156 +8566,156 @@
 สรุป: เท่ากัน (126 หน่วยกิต)</t>
         </is>
       </c>
-      <c r="H73" s="20" t="inlineStr">
+      <c r="H83" s="20" t="inlineStr">
         <is>
           <t>BIT2565 หน้า 6; DSBA2560 หน้า 17
 (หน้าที่ระบบคืนมา: BIT 2565 หน้า 266, 264, 267, 265)</t>
         </is>
       </c>
-      <c r="I73" s="20" t="inlineStr">
+      <c r="I83" s="20" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J73" s="19" t="n">
+      <c r="J83" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K73" s="15" t="inlineStr">
+      <c r="K83" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L73" s="18" t="inlineStr">
+      <c r="L83" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M73" s="20" t="inlineStr">
+      <c r="M83" s="20" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N73" s="19" t="inlineStr">
-        <is>
-          <t>0.17s</t>
-        </is>
-      </c>
-      <c r="O73" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="80" customHeight="1">
-      <c r="A74" s="13" t="inlineStr">
+      <c r="N83" s="19" t="inlineStr">
+        <is>
+          <t>0.23s</t>
+        </is>
+      </c>
+      <c r="O83" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="80" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="B74" s="24" t="inlineStr">
+      <c r="B84" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C74" s="15" t="inlineStr">
+      <c r="C84" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="D84" s="16" t="inlineStr">
         <is>
           <t>วิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ต้องผ่านวิชาอะไรมาก่อนบ้าง ไล่ย้อนทุกชั้น</t>
         </is>
       </c>
-      <c r="E74" s="16" t="inlineStr">
+      <c r="E84" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F74" s="16" t="inlineStr">
+      <c r="F84" s="16" t="inlineStr">
         <is>
           <t>ต้องผ่าน 06066001 ความน่าจะเป็นและสถิติ ซึ่งไม่มีวิชาบังคับก่อน (ชั้นเดียว)</t>
         </is>
       </c>
-      <c r="G74" s="16" t="inlineStr">
+      <c r="G84" s="16" t="inlineStr">
         <is>
           <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   ต้องผ่านวิชาบังคับก่อน:
     • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
         </is>
       </c>
-      <c r="H74" s="16" t="inlineStr">
+      <c r="H84" s="16" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 289, 291
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 37, 291, 19, 20)</t>
         </is>
       </c>
-      <c r="I74" s="16" t="inlineStr">
+      <c r="I84" s="16" t="inlineStr">
         <is>
           <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J74" s="15" t="n">
+      <c r="J84" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="K74" s="15" t="inlineStr">
+      <c r="K84" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L74" s="18" t="inlineStr">
+      <c r="L84" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M74" s="16" t="inlineStr">
+      <c r="M84" s="16" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N74" s="15" t="inlineStr">
-        <is>
-          <t>0.10s</t>
-        </is>
-      </c>
-      <c r="O74" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="80" customHeight="1">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="N84" s="15" t="inlineStr">
+        <is>
+          <t>0.18s</t>
+        </is>
+      </c>
+      <c r="O84" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="80" customHeight="1">
+      <c r="A85" s="13" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="B75" s="24" t="inlineStr">
+      <c r="B85" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C75" s="19" t="inlineStr">
+      <c r="C85" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D75" s="20" t="inlineStr">
+      <c r="D85" s="20" t="inlineStr">
         <is>
           <t>นักศึกษา DSBA 2565 ที่ไม่เข้าโครงการสหกิจศึกษา ต้องเรียนอะไรแทนสหกิจศึกษา กี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E75" s="20" t="inlineStr">
+      <c r="E85" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F75" s="20" t="inlineStr">
+      <c r="F85" s="20" t="inlineStr">
         <is>
           <t>กลุ่มวิชาการศึกษาทางเลือก (กลุ่มวิชาเลือก) 6 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G75" s="20" t="inlineStr">
+      <c r="G85" s="20" t="inlineStr">
         <is>
           <t>เปรียบเทียบแผนการศึกษา DSBA 2565 (ปริญญาตรี): แผนปกติ (3.1.4.1) กับแผนที่เข้าโครงการสหกิจศึกษา (3.1.4.2)
 - ปีที่ 1 ภาคการศึกษาที่ 1: แผนปกติ 18 หน่วยกิต · แผนสหกิจ 18 หน่วยกิต
@@ -7884,306 +8754,307 @@
 ตามโครงสร้างหลักสูตร: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน 6 · แผนสหกิจ: สหกิจศึกษา 6)</t>
         </is>
       </c>
-      <c r="H75" s="20" t="inlineStr">
+      <c r="H85" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 15, 21-22
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29, 36)</t>
         </is>
       </c>
-      <c r="I75" s="20" t="inlineStr">
+      <c r="I85" s="20" t="inlineStr">
         <is>
           <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J75" s="19" t="n">
+      <c r="J85" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="K75" s="15" t="inlineStr">
+      <c r="K85" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L75" s="18" t="inlineStr">
+      <c r="L85" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M75" s="20" t="inlineStr">
+      <c r="M85" s="20" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2] ตอบเป็นตารางเทียบสองแผนทั้งหมด ส่วนที่ถามอยู่ท้ายคำตอบ: กลุ่มวิชาการศึกษาทางเลือก 6 หน่วยกิต (แผนปกติ: กลุ่มวิชาเลือกหรือกลุ่มวิชาชีพเฉพาะด้าน)</t>
         </is>
       </c>
-      <c r="N75" s="19" t="inlineStr">
-        <is>
-          <t>0.06s</t>
-        </is>
-      </c>
-      <c r="O75" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="80" customHeight="1">
-      <c r="A76" s="13" t="inlineStr">
+      <c r="N85" s="19" t="inlineStr">
+        <is>
+          <t>0.08s</t>
+        </is>
+      </c>
+      <c r="O85" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="80" customHeight="1">
+      <c r="A86" s="13" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="B76" s="24" t="inlineStr">
+      <c r="B86" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C76" s="15" t="inlineStr">
+      <c r="C86" s="15" t="inlineStr">
         <is>
           <t>AITBA</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
+      <c r="D86" s="16" t="inlineStr">
         <is>
           <t>ปริญญาโท AITBA 2569 แผนวิชาชีพต้องเรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E76" s="16" t="inlineStr">
+      <c r="E86" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F76" s="16" t="inlineStr">
+      <c r="F86" s="16" t="inlineStr">
         <is>
           <t>36 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G76" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนไม่น้อยกว่า 36 หน่วยกิต [3]</t>
-        </is>
-      </c>
-      <c r="H76" s="16" t="inlineStr">
+      <c r="G86" s="16" t="inlineStr">
+        <is>
+          <t>ปริญญาโท AITBA 2569 แผนวิชาชีพ (แผน 2) ต้องเรียนรวมไม่น้อยกว่า 36 หน่วยกิต [3]</t>
+        </is>
+      </c>
+      <c r="H86" s="16" t="inlineStr">
         <is>
           <t>AITBA2569 หน้า 5
 (หน้าที่ระบบคืนมา: ปร.ด. AITBA 2569 หน้า 100, 5, 15, 228; วท.ม. AITBA 2569 หน้า 228, 21)</t>
         </is>
       </c>
-      <c r="I76" s="16" t="inlineStr">
+      <c r="I86" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J76" s="15" t="n">
+      <c r="J86" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="K76" s="15" t="inlineStr">
+      <c r="K86" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L76" s="18" t="inlineStr">
+      <c r="L86" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M76" s="16" t="inlineStr">
+      <c r="M86" s="16" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N76" s="15" t="inlineStr">
-        <is>
-          <t>1.16s</t>
-        </is>
-      </c>
-      <c r="O76" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="80" customHeight="1">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="N86" s="15" t="inlineStr">
+        <is>
+          <t>1.01s</t>
+        </is>
+      </c>
+      <c r="O86" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="80" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
-      <c r="B77" s="24" t="inlineStr">
+      <c r="B87" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Y)</t>
         </is>
       </c>
-      <c r="C77" s="19" t="inlineStr">
+      <c r="C87" s="19" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D77" s="20" t="inlineStr">
+      <c r="D87" s="20" t="inlineStr">
         <is>
           <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E77" s="20" t="inlineStr">
+      <c r="E87" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F77" s="20" t="inlineStr">
+      <c r="F87" s="20" t="inlineStr">
         <is>
           <t>36 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G77" s="20" t="inlineStr">
+      <c r="G87" s="20" t="inlineStr">
         <is>
           <t>ปริญญาโท IT 2568 แผนวิชาการแบบ 1.1 ต้องเรียนรวมทั้งหมด 36 หน่วยกิต [5]</t>
         </is>
       </c>
-      <c r="H77" s="20" t="inlineStr">
+      <c r="H87" s="20" t="inlineStr">
         <is>
           <t>IT2568 หน้า 5
 (หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 155, 25, 74, 18)</t>
         </is>
       </c>
-      <c r="I77" s="20" t="inlineStr">
+      <c r="I87" s="20" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J77" s="19" t="n">
+      <c r="J87" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="K77" s="15" t="inlineStr">
+      <c r="K87" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L77" s="18" t="inlineStr">
+      <c r="L87" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M77" s="20" t="inlineStr">
+      <c r="M87" s="20" t="inlineStr">
         <is>
           <t>[ชุด Y: เขียนก่อนแก้รอบที่ 1 (held-out ของรอบที่ 1) แล้วถูกใช้ดูต้นเหตุในรอบที่ 2]</t>
         </is>
       </c>
-      <c r="N77" s="19" t="inlineStr">
-        <is>
-          <t>1.11s</t>
-        </is>
-      </c>
-      <c r="O77" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="80" customHeight="1">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="N87" s="19" t="inlineStr">
+        <is>
+          <t>1.27s</t>
+        </is>
+      </c>
+      <c r="O87" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="80" customHeight="1">
+      <c r="A88" s="13" t="inlineStr">
         <is>
           <t>Z1</t>
         </is>
       </c>
-      <c r="B78" s="24" t="inlineStr">
+      <c r="B88" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C78" s="15" t="inlineStr">
+      <c r="C88" s="15" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D78" s="16" t="inlineStr">
+      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวมกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E78" s="16" t="inlineStr">
+      <c r="E88" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F78" s="16" t="inlineStr">
+      <c r="F88" s="16" t="inlineStr">
         <is>
           <t>75 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G78" s="16" t="inlineStr">
-        <is>
-          <t>ปริญญาเอก IT 2561 แบบ 1.2 (ผู้สำเร็จปริญญาตรี) ต้องเรียนหน่วยกิตรวม 75 หน่วยกิต [1]</t>
-        </is>
-      </c>
-      <c r="H78" s="16" t="inlineStr">
+      <c r="G88" s="16" t="inlineStr">
+        <is>
+          <t>75 หน่วยกิต  
+[1]</t>
+        </is>
+      </c>
+      <c r="H88" s="16" t="inlineStr">
         <is>
           <t>IT2561 หน้า 16
 (หน้าที่ระบบคืนมา: ปร.ด. IT 2561 หน้า 16, 38, 22, 131)</t>
         </is>
       </c>
-      <c r="I78" s="16" t="inlineStr">
+      <c r="I88" s="16" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J78" s="15" t="n">
+      <c r="J88" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="K78" s="15" t="inlineStr">
+      <c r="K88" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L78" s="18" t="inlineStr">
+      <c r="L88" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M78" s="16" t="inlineStr">
+      <c r="M88" s="16" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N78" s="15" t="inlineStr">
-        <is>
-          <t>1.27s</t>
-        </is>
-      </c>
-      <c r="O78" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="80" customHeight="1">
-      <c r="A79" s="13" t="inlineStr">
+      <c r="N88" s="15" t="inlineStr">
+        <is>
+          <t>0.45s</t>
+        </is>
+      </c>
+      <c r="O88" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="80" customHeight="1">
+      <c r="A89" s="13" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="B79" s="24" t="inlineStr">
+      <c r="B89" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C79" s="19" t="inlineStr">
+      <c r="C89" s="19" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D79" s="20" t="inlineStr">
+      <c r="D89" s="20" t="inlineStr">
         <is>
           <t>แผนสหกิจศึกษาของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E79" s="20" t="inlineStr">
+      <c r="E89" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F79" s="20" t="inlineStr">
+      <c r="F89" s="20" t="inlineStr">
         <is>
           <t>6 หน่วยกิต (สหกิจศึกษา 06026259 หรือ 06026260 ต่างประเทศ)</t>
         </is>
       </c>
-      <c r="G79" s="20" t="inlineStr">
+      <c r="G89" s="20" t="inlineStr">
         <is>
           <t>แผนที่เข้าโครงการสหกิจศึกษา — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 36):
   - 06026259 สหกิจศึกษาทางวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ — 6 (0-35-0)
@@ -8191,78 +9062,78 @@
   รวมภาคนี้ตามแผนในเล่ม: 6 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H79" s="20" t="inlineStr">
+      <c r="H89" s="20" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 36
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 36)</t>
         </is>
       </c>
-      <c r="I79" s="20" t="inlineStr">
+      <c r="I89" s="20" t="inlineStr">
         <is>
           <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J79" s="19" t="n">
+      <c r="J89" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="K79" s="15" t="inlineStr">
+      <c r="K89" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L79" s="18" t="inlineStr">
+      <c r="L89" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M79" s="20" t="inlineStr">
+      <c r="M89" s="20" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N79" s="19" t="inlineStr">
-        <is>
-          <t>0.17s</t>
-        </is>
-      </c>
-      <c r="O79" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="80" customHeight="1">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="N89" s="19" t="inlineStr">
+        <is>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="O89" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="80" customHeight="1">
+      <c r="A90" s="13" t="inlineStr">
         <is>
           <t>Z3</t>
         </is>
       </c>
-      <c r="B80" s="24" t="inlineStr">
+      <c r="B90" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C80" s="15" t="inlineStr">
+      <c r="C90" s="15" t="inlineStr">
         <is>
           <t>DSBA</t>
         </is>
       </c>
-      <c r="D80" s="16" t="inlineStr">
+      <c r="D90" s="16" t="inlineStr">
         <is>
           <t>แผนปกติของ DSBA 2565 ปีที่ 4 ภาคการศึกษาที่ 2 เรียนอะไร กี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E80" s="16" t="inlineStr">
+      <c r="E90" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F80" s="16" t="inlineStr">
+      <c r="F90" s="16" t="inlineStr">
         <is>
           <t>วิชาเลือกหมวดศึกษาทั่วไป 1 วิชา + วิชาเลือกเสรี 2 วิชา รวม 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G80" s="16" t="inlineStr">
+      <c r="G90" s="16" t="inlineStr">
         <is>
           <t>แผนปกติ (ไม่เข้าโครงการสหกิจศึกษา) — ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 29):
   - วิชาเลือกที่ต้องลงตามแผน: 3 ช่อง
@@ -8272,78 +9143,78 @@
   รวมภาคนี้ตามแผนในเล่ม: 9 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H80" s="16" t="inlineStr">
+      <c r="H90" s="16" t="inlineStr">
         <is>
           <t>DSBA2565 หน้า 29
 (หน้าที่ระบบคืนมา: DSBA 2565 หน้า 29)</t>
         </is>
       </c>
-      <c r="I80" s="16" t="inlineStr">
+      <c r="I90" s="16" t="inlineStr">
         <is>
           <t>Structured SQL (อ่านตารางแผนปกติ/แผนสหกิจจากเล่ม) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J80" s="15" t="n">
+      <c r="J90" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="K80" s="15" t="inlineStr">
+      <c r="K90" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L80" s="18" t="inlineStr">
+      <c r="L90" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M80" s="16" t="inlineStr">
+      <c r="M90" s="16" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)] ตอบ 3 ช่อง (วิชาเลือกศึกษาทั่วไป 1 + เลือกเสรี 2) รวม 9 หน่วยกิต ตรงเฉลย</t>
         </is>
       </c>
-      <c r="N80" s="15" t="inlineStr">
-        <is>
-          <t>0.13s</t>
-        </is>
-      </c>
-      <c r="O80" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="80" customHeight="1">
-      <c r="A81" s="13" t="inlineStr">
+      <c r="N90" s="15" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+      <c r="O90" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="80" customHeight="1">
+      <c r="A91" s="13" t="inlineStr">
         <is>
           <t>Z4</t>
         </is>
       </c>
-      <c r="B81" s="24" t="inlineStr">
+      <c r="B91" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C81" s="19" t="inlineStr">
+      <c r="C91" s="19" t="inlineStr">
         <is>
           <t>BIT</t>
         </is>
       </c>
-      <c r="D81" s="20" t="inlineStr">
+      <c r="D91" s="20" t="inlineStr">
         <is>
           <t>BIT 2565 กับ IT 2565 หน่วยกิตรวมต่างกันกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E81" s="20" t="inlineStr">
+      <c r="E91" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F81" s="20" t="inlineStr">
+      <c r="F91" s="20" t="inlineStr">
         <is>
           <t>BIT 2565 = 126, IT 2565 = 129 ต่างกัน 3 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G81" s="20" t="inlineStr">
+      <c r="G91" s="20" t="inlineStr">
         <is>
           <t>หน่วยกิตรวมตลอดหลักสูตร (จากหน้าโครงสร้างหลักสูตรในเล่ม):
 - BIT 2565: 126 หน่วยกิต (มคอ.2 BIT 2565 หน้า 6)
@@ -8351,201 +9222,201 @@
 สรุป: IT 2565 มากกว่า BIT 2565 อยู่ 3 หน่วยกิต</t>
         </is>
       </c>
-      <c r="H81" s="20" t="inlineStr">
+      <c r="H91" s="20" t="inlineStr">
         <is>
           <t>BIT2565 หน้า 6; IT2565 หน้า 6
 (หน้าที่ระบบคืนมา: BIT 2565 หน้า 264, 266, 7)</t>
         </is>
       </c>
-      <c r="I81" s="20" t="inlineStr">
+      <c r="I91" s="20" t="inlineStr">
         <is>
           <t>เทียบหน่วยกิตรวมจากตาราง rule (มี provenance) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J81" s="19" t="n">
+      <c r="J91" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K81" s="15" t="inlineStr">
+      <c r="K91" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L81" s="18" t="inlineStr">
+      <c r="L91" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M81" s="20" t="inlineStr">
+      <c r="M91" s="20" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N81" s="19" t="inlineStr">
-        <is>
-          <t>0.30s</t>
-        </is>
-      </c>
-      <c r="O81" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="80" customHeight="1">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="N91" s="19" t="inlineStr">
+        <is>
+          <t>0.19s</t>
+        </is>
+      </c>
+      <c r="O91" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="80" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
         <is>
           <t>Z5</t>
         </is>
       </c>
-      <c r="B82" s="24" t="inlineStr">
+      <c r="B92" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C82" s="15" t="inlineStr">
+      <c r="C92" s="15" t="inlineStr">
         <is>
           <t>AIT</t>
         </is>
       </c>
-      <c r="D82" s="16" t="inlineStr">
+      <c r="D92" s="16" t="inlineStr">
         <is>
           <t>วิชาพื้นฐานวิทยาการข้อมูลของ AIT ต้องผ่านวิชาอะไรมาก่อน</t>
         </is>
       </c>
-      <c r="E82" s="16" t="inlineStr">
+      <c r="E92" s="16" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F82" s="16" t="inlineStr">
+      <c r="F92" s="16" t="inlineStr">
         <is>
           <t>ไม่มีวิชาบังคับก่อน</t>
         </is>
       </c>
-      <c r="G82" s="16" t="inlineStr">
+      <c r="G92" s="16" t="inlineStr">
         <is>
           <t>วิชา 06046407 พื้นฐานวิทยาการข้อมูล (FUNDAMENTALS OF DATA SCIENCE) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
   ไม่มีวิชาบังคับก่อน (PREREQUISITE: None)</t>
         </is>
       </c>
-      <c r="H82" s="16" t="inlineStr">
+      <c r="H92" s="16" t="inlineStr">
         <is>
           <t>AIT2566 หน้า 292
 (หน้าที่ระบบคืนมา: AIT 2566 หน้า 20, 24, 38, 292)</t>
         </is>
       </c>
-      <c r="I82" s="16" t="inlineStr">
+      <c r="I92" s="16" t="inlineStr">
         <is>
           <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
         </is>
       </c>
-      <c r="J82" s="15" t="n">
+      <c r="J92" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K82" s="15" t="inlineStr">
+      <c r="K92" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L82" s="18" t="inlineStr">
+      <c r="L92" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M82" s="16" t="inlineStr">
+      <c r="M92" s="16" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N82" s="15" t="inlineStr">
-        <is>
-          <t>0.18s</t>
-        </is>
-      </c>
-      <c r="O82" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="80" customHeight="1">
-      <c r="A83" s="13" t="inlineStr">
+      <c r="N92" s="15" t="inlineStr">
+        <is>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="O92" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="80" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
         <is>
           <t>Z6</t>
         </is>
       </c>
-      <c r="B83" s="24" t="inlineStr">
+      <c r="B93" s="24" t="inlineStr">
         <is>
           <t>ระดับ 4: ท้าทายเพิ่มเติม (ชุด Z)</t>
         </is>
       </c>
-      <c r="C83" s="19" t="inlineStr">
+      <c r="C93" s="19" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D83" s="20" t="inlineStr">
+      <c r="D93" s="20" t="inlineStr">
         <is>
           <t>ปริญญาโท IT 2568 แผนวิชาชีพ ต้องเรียนกี่หน่วยกิต</t>
         </is>
       </c>
-      <c r="E83" s="20" t="inlineStr">
+      <c r="E93" s="20" t="inlineStr">
         <is>
           <t>Multi-hop / ข้ามเวอร์ชัน (เขียนเฉลยจากเล่มก่อนรัน)</t>
         </is>
       </c>
-      <c r="F83" s="20" t="inlineStr">
+      <c r="F93" s="20" t="inlineStr">
         <is>
           <t>36 หน่วยกิต</t>
         </is>
       </c>
-      <c r="G83" s="20" t="inlineStr">
-        <is>
-          <t>ปริญญาโท IT 2568 แผนวิชาชีพต้องเรียนรวมทั้งหมด 36 หน่วยกิต [2]</t>
-        </is>
-      </c>
-      <c r="H83" s="20" t="inlineStr">
+      <c r="G93" s="20" t="inlineStr">
+        <is>
+          <t>ปริญญาโท สาขาวิชาเทคโนโลยีสารสนเทศ หลักสูตรปี พ.ศ. 2568 แผนวิชาชีพ ต้องเรียนทั้งหมด 36 หน่วยกิต [2]</t>
+        </is>
+      </c>
+      <c r="H93" s="20" t="inlineStr">
         <is>
           <t>IT2568 หน้า 5
 (หน้าที่ระบบคืนมา: วท.ม. IT 2568 หน้า 25, 12, 156, 14)</t>
         </is>
       </c>
-      <c r="I83" s="20" t="inlineStr">
+      <c r="I93" s="20" t="inlineStr">
         <is>
           <t>Hybrid retrieval (FTS5+bge-m3) → Typhoon</t>
         </is>
       </c>
-      <c r="J83" s="19" t="n">
+      <c r="J93" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="K83" s="15" t="inlineStr">
+      <c r="K93" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L83" s="18" t="inlineStr">
+      <c r="L93" s="18" t="inlineStr">
         <is>
           <t>ถูกครบ</t>
         </is>
       </c>
-      <c r="M83" s="20" t="inlineStr">
+      <c r="M93" s="20" t="inlineStr">
         <is>
           <t>[ชุด Z: เขียนก่อนแก้รอบที่ 2 (held-out ของรอบที่ 2)]</t>
         </is>
       </c>
-      <c r="N83" s="19" t="inlineStr">
-        <is>
-          <t>1.17s</t>
-        </is>
-      </c>
-      <c r="O83" s="18" t="inlineStr">
+      <c r="N93" s="19" t="inlineStr">
+        <is>
+          <t>1.43s</t>
+        </is>
+      </c>
+      <c r="O93" s="18" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O83"/>
+  <autoFilter ref="A1:O93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8595,7 +9466,7 @@
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>1. ระดับ 4 ท้าทาย (Multi-hop &amp; Cross-version)</t>
         </is>
@@ -8612,12 +9483,12 @@
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>C1: หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา หน้า 18 / หน้า 6) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่ามี 3 แขนง) ตัวเลขย่อยรอบนี้ (เฉพาะด้าน 94→93, บังคับเฉพาะแขนง 30→15, เลือก IT 6→9) ตรงกับโครงสร้างในเล่ม ข้อนี้ผ่าน LLM ตัวเลขย่อยเปลี่ยนทุกรอบ (รอบก่อนมีประโยคที่ขัดกันเอง) · C2: พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง และระบุระดับที่ตรวจพบจากเนื้อหา (master ทั้งคู่) ตามที่ฐานข้อมูลเก็บ · C3: ตอบจากตารางแผนทั้งสองชุดในเล่ม (3.1.4.1 หน้า 23-29 และ 3.1.4.2 หน้า 30-36): ต่างกันที่ปี 4 ภาค 1 (ปกติ 9 / สหกิจ 12) และปี 4 ภาค 2 (ปกติ 9 / สหกิจศึกษา 06026259 6 หน่วยกิต) รวม 132 เท่ากัน ตรวจกับเล่มแล้ว หมายเหตุ: เฉลยในไฟล์ทดสอบเขียนว่าแผนปกติลงโครงงาน 2 ในปี 4 ภาค 2 และใช้รหัสสหกิจ 06026245 ซึ่งไม่ตรงเล่ม (โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน, รหัสสหกิจคือ 06026259/06026260)</t>
+          <t>C1: หน่วยกิตรวม 130 → 129 ถูก (ดึงจากตาราง rule ที่มีหน้าที่มา) ตัวเลขย่อยรอบนี้ตรงกับโครงสร้างในเล่ม (กลุ่มเฉพาะด้าน 46→57, บังคับเฉพาะแขนง 30→15, เลือก IT 6→9) แต่ส่วนแขนงวิชาบอกว่าเปลี่ยนเป็น 'โมดูลอาชีพ' แทนแขนง ซึ่งต่างจากเฉลย (เฉลยว่ามี 3 แขนง) ข้อนี้ผ่าน LLM ตัวเลขย่อยเปลี่ยนทุกรอบ · C2: พบว่าสองไฟล์เป็นไฟล์เดียวกันด้วย SHA-256/ขนาด/จำนวนหน้าถูกต้อง และระบุระดับที่ตรวจพบจากเนื้อหา (master ทั้งคู่) ตามที่ฐานข้อมูลเก็บ · C3: ตอบจากตารางแผนทั้งสองชุดในเล่ม (3.1.4.1 หน้า 23-29 และ 3.1.4.2 หน้า 30-36): ต่างกันที่ปี 4 ภาค 1 (ปกติ 9 / สหกิจ 12) และปี 4 ภาค 2 (ปกติ 9 / สหกิจศึกษา 06026259 6 หน่วยกิต) รวม 132 เท่ากัน ตรวจกับเล่มแล้ว หมายเหตุ: เฉลยในไฟล์ทดสอบเขียนว่าแผนปกติลงโครงงาน 2 ในปี 4 ภาค 2 และใช้รหัสสหกิจ 06026245 ซึ่งไม่ตรงเล่ม (โครงงาน 2 อยู่ปี 4 ภาค 1 ทั้งสองแผน, รหัสสหกิจคือ 06026259/06026260)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>2. ความเร็ว (Latency)</t>
         </is>
@@ -8629,7 +9500,7 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>ระดับยาก 7 ข้อ เฉลี่ย 1.60s ช้าสุด 4.86s · ทั้ง 28 ข้อ ต่ำกว่า 5s 27/28</t>
+          <t>ระดับยาก 7 ข้อ เฉลี่ย 1.54s ช้าสุด 5.40s · ทั้ง 28 ข้อ ต่ำกว่า 5s 26/28</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">

</xml_diff>